<commit_message>
Fix professional staffing detection in merit workbook
</commit_message>
<xml_diff>
--- a/downloads/Merit_2026_Employee_Bulk_Calculator_350_exact.xlsx
+++ b/downloads/Merit_2026_Employee_Bulk_Calculator_350_exact.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employee Merit 2026" sheetId="1" r:id="Rc6d0546b22104485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="R3d4bc1ee175c46f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employee Merit 2026" sheetId="1" r:id="R40ed1c6e69c442bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="R6a149820194e495c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -865,6 +865,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="21" max="21" width="0" hidden="0" customWidth="1"/>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="64" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
@@ -908,6 +909,9 @@
       <x:c r="Q1" s="3"/>
       <x:c r="R1" s="3"/>
       <x:c r="S1" s="3"/>
+      <x:c r="U1" t="str">
+        <x:v>Job Title Dropdown Source</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -931,6 +935,14 @@
       <x:c r="Q2" s="6"/>
       <x:c r="R2" s="6"/>
       <x:c r="S2" s="6"/>
+      <x:c r="U2" t="str">
+        <x:v>Accountant - II - Finance &amp; Legal (B Support / Professional) - P2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="U3" t="str">
+        <x:v>Accountant - III - Finance &amp; Legal (B Support / Professional) - P3</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -989,6 +1001,9 @@
       </x:c>
       <x:c r="S4" s="17" t="str">
         <x:v>Status</x:v>
+      </x:c>
+      <x:c r="U4" t="str">
+        <x:v>Administrative Assistant - II - Business Support (A) Admin/Finance/HR - B2</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
@@ -996,7 +1011,7 @@
       <x:c r="B5" s="30"/>
       <x:c r="C5" s="58"/>
       <x:c r="D5" s="49" t="str">
-        <x:f>IF($B5="","",IF(OR(RIGHT(TRIM($B5),2)="P1",RIGHT(TRIM($B5),2)="P2",RIGHT(TRIM($B5),2)="P3",RIGHT(TRIM($B5),2)="P4"),"PS","GS"))</x:f>
+        <x:f>IF($B5="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B5),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E5" s="61" t="str">
         <x:f>IF($D5="","",IF($D5="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1042,6 +1057,9 @@
       </x:c>
       <x:c r="S5" s="51" t="str">
         <x:f>IF(AND($A5="",$B5="",$C5=""),"",IF($A5="","Missing Assignment Number",IF($B5="","Select Job Title",IF($C5="","Enter Pay Rate",IF($F5="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U5" t="str">
+        <x:v>Administrative Assistant - III - Business Support (A) Admin/Finance/HR - B3</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
@@ -1049,7 +1067,7 @@
       <x:c r="B6" s="33"/>
       <x:c r="C6" s="59"/>
       <x:c r="D6" s="52" t="str">
-        <x:f>IF($B6="","",IF(OR(RIGHT(TRIM($B6),2)="P2",RIGHT(TRIM($B6),2)="P3",RIGHT(TRIM($B6),2)="P4",RIGHT(TRIM($B6),2)="P5"),"PS","GS"))</x:f>
+        <x:f>IF($B6="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B6),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E6" s="62" t="str">
         <x:f>IF($D6="","",IF($D6="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1095,6 +1113,9 @@
       </x:c>
       <x:c r="S6" s="54" t="str">
         <x:f>IF(AND($A6="",$B6="",$C6=""),"",IF($A6="","Missing Assignment Number",IF($B6="","Select Job Title",IF($C6="","Enter Pay Rate",IF($F6="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U6" t="str">
+        <x:v>Analytical Chemist - I - LAB (B Support / Research) - R1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
@@ -1102,7 +1123,7 @@
       <x:c r="B7" s="33"/>
       <x:c r="C7" s="59"/>
       <x:c r="D7" s="52" t="str">
-        <x:f>IF($B7="","",IF(OR(RIGHT(TRIM($B7),2)="P3",RIGHT(TRIM($B7),2)="P4",RIGHT(TRIM($B7),2)="P5",RIGHT(TRIM($B7),2)="P6"),"PS","GS"))</x:f>
+        <x:f>IF($B7="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B7),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E7" s="62" t="str">
         <x:f>IF($D7="","",IF($D7="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1148,6 +1169,9 @@
       </x:c>
       <x:c r="S7" s="54" t="str">
         <x:f>IF(AND($A7="",$B7="",$C7=""),"",IF($A7="","Missing Assignment Number",IF($B7="","Select Job Title",IF($C7="","Enter Pay Rate",IF($F7="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U7" t="str">
+        <x:v>Assembler - II - Production &amp; Operations Support (T): Industrial - O2 (Low)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
@@ -1155,7 +1179,7 @@
       <x:c r="B8" s="33"/>
       <x:c r="C8" s="59"/>
       <x:c r="D8" s="52" t="str">
-        <x:f>IF($B8="","",IF(OR(RIGHT(TRIM($B8),2)="P4",RIGHT(TRIM($B8),2)="P5",RIGHT(TRIM($B8),2)="P6",RIGHT(TRIM($B8),2)="P7"),"PS","GS"))</x:f>
+        <x:f>IF($B8="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B8),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E8" s="62" t="str">
         <x:f>IF($D8="","",IF($D8="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1201,6 +1225,9 @@
       </x:c>
       <x:c r="S8" s="54" t="str">
         <x:f>IF(AND($A8="",$B8="",$C8=""),"",IF($A8="","Missing Assignment Number",IF($B8="","Select Job Title",IF($C8="","Enter Pay Rate",IF($F8="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U8" t="str">
+        <x:v>Automation Engineer - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -1208,7 +1235,7 @@
       <x:c r="B9" s="33"/>
       <x:c r="C9" s="59"/>
       <x:c r="D9" s="52" t="str">
-        <x:f>IF($B9="","",IF(OR(RIGHT(TRIM($B9),2)="P5",RIGHT(TRIM($B9),2)="P6",RIGHT(TRIM($B9),2)="P7",RIGHT(TRIM($B9),2)="P8"),"PS","GS"))</x:f>
+        <x:f>IF($B9="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B9),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E9" s="62" t="str">
         <x:f>IF($D9="","",IF($D9="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1254,6 +1281,9 @@
       </x:c>
       <x:c r="S9" s="54" t="str">
         <x:f>IF(AND($A9="",$B9="",$C9=""),"",IF($A9="","Missing Assignment Number",IF($B9="","Select Job Title",IF($C9="","Enter Pay Rate",IF($F9="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U9" t="str">
+        <x:v>Biochemical Operator – ll - Production &amp; Operations Support (T): Industrial – O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
@@ -1261,7 +1291,7 @@
       <x:c r="B10" s="33"/>
       <x:c r="C10" s="59"/>
       <x:c r="D10" s="52" t="str">
-        <x:f>IF($B10="","",IF(OR(RIGHT(TRIM($B10),2)="P6",RIGHT(TRIM($B10),2)="P7",RIGHT(TRIM($B10),2)="P8",RIGHT(TRIM($B10),2)="P9"),"PS","GS"))</x:f>
+        <x:f>IF($B10="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B10),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E10" s="62" t="str">
         <x:f>IF($D10="","",IF($D10="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1307,6 +1337,9 @@
       </x:c>
       <x:c r="S10" s="54" t="str">
         <x:f>IF(AND($A10="",$B10="",$C10=""),"",IF($A10="","Missing Assignment Number",IF($B10="","Select Job Title",IF($C10="","Enter Pay Rate",IF($F10="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U10" t="str">
+        <x:v>Biochemist - I - LAB (B Support / Research) - R1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
@@ -1314,7 +1347,7 @@
       <x:c r="B11" s="33"/>
       <x:c r="C11" s="59"/>
       <x:c r="D11" s="52" t="str">
-        <x:f>IF($B11="","",IF(OR(RIGHT(TRIM($B11),2)="P7",RIGHT(TRIM($B11),2)="P8",RIGHT(TRIM($B11),2)="P9",RIGHT(TRIM($B11),2)="P10"),"PS","GS"))</x:f>
+        <x:f>IF($B11="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B11),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E11" s="62" t="str">
         <x:f>IF($D11="","",IF($D11="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1360,6 +1393,9 @@
       </x:c>
       <x:c r="S11" s="54" t="str">
         <x:f>IF(AND($A11="",$B11="",$C11=""),"",IF($A11="","Missing Assignment Number",IF($B11="","Select Job Title",IF($C11="","Enter Pay Rate",IF($F11="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U11" t="str">
+        <x:v>Biologist - I - LAB (B Support / Research) - R1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
@@ -1367,7 +1403,7 @@
       <x:c r="B12" s="33"/>
       <x:c r="C12" s="59"/>
       <x:c r="D12" s="52" t="str">
-        <x:f>IF($B12="","",IF(OR(RIGHT(TRIM($B12),2)="P8",RIGHT(TRIM($B12),2)="P9",RIGHT(TRIM($B12),2)="P10",RIGHT(TRIM($B12),2)="P11"),"PS","GS"))</x:f>
+        <x:f>IF($B12="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B12),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E12" s="62" t="str">
         <x:f>IF($D12="","",IF($D12="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1413,6 +1449,9 @@
       </x:c>
       <x:c r="S12" s="54" t="str">
         <x:f>IF(AND($A12="",$B12="",$C12=""),"",IF($A12="","Missing Assignment Number",IF($B12="","Select Job Title",IF($C12="","Enter Pay Rate",IF($F12="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U12" t="str">
+        <x:v>Business Analyst - II - Information Communications Technology (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
@@ -1420,7 +1459,7 @@
       <x:c r="B13" s="33"/>
       <x:c r="C13" s="59"/>
       <x:c r="D13" s="52" t="str">
-        <x:f>IF($B13="","",IF(OR(RIGHT(TRIM($B13),2)="P9",RIGHT(TRIM($B13),2)="P10",RIGHT(TRIM($B13),2)="P11",RIGHT(TRIM($B13),2)="P12"),"PS","GS"))</x:f>
+        <x:f>IF($B13="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B13),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E13" s="62" t="str">
         <x:f>IF($D13="","",IF($D13="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1466,6 +1505,9 @@
       </x:c>
       <x:c r="S13" s="54" t="str">
         <x:f>IF(AND($A13="",$B13="",$C13=""),"",IF($A13="","Missing Assignment Number",IF($B13="","Select Job Title",IF($C13="","Enter Pay Rate",IF($F13="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U13" t="str">
+        <x:v>Business Analyst - III - Information Communications Technology (B Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
@@ -1473,7 +1515,7 @@
       <x:c r="B14" s="33"/>
       <x:c r="C14" s="59"/>
       <x:c r="D14" s="52" t="str">
-        <x:f>IF($B14="","",IF(OR(RIGHT(TRIM($B14),2)="P10",RIGHT(TRIM($B14),2)="P11",RIGHT(TRIM($B14),2)="P12",RIGHT(TRIM($B14),2)="P13"),"PS","GS"))</x:f>
+        <x:f>IF($B14="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B14),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E14" s="62" t="str">
         <x:f>IF($D14="","",IF($D14="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1519,6 +1561,9 @@
       </x:c>
       <x:c r="S14" s="54" t="str">
         <x:f>IF(AND($A14="",$B14="",$C14=""),"",IF($A14="","Missing Assignment Number",IF($B14="","Select Job Title",IF($C14="","Enter Pay Rate",IF($F14="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U14" t="str">
+        <x:v>Business Analyst - IV - Information Communications Technology (B Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
@@ -1526,7 +1571,7 @@
       <x:c r="B15" s="33"/>
       <x:c r="C15" s="59"/>
       <x:c r="D15" s="52" t="str">
-        <x:f>IF($B15="","",IF(OR(RIGHT(TRIM($B15),2)="P11",RIGHT(TRIM($B15),2)="P12",RIGHT(TRIM($B15),2)="P13",RIGHT(TRIM($B15),2)="P14"),"PS","GS"))</x:f>
+        <x:f>IF($B15="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B15),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E15" s="62" t="str">
         <x:f>IF($D15="","",IF($D15="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1572,6 +1617,9 @@
       </x:c>
       <x:c r="S15" s="54" t="str">
         <x:f>IF(AND($A15="",$B15="",$C15=""),"",IF($A15="","Missing Assignment Number",IF($B15="","Select Job Title",IF($C15="","Enter Pay Rate",IF($F15="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U15" t="str">
+        <x:v>Business Consultant - IV - Information Communications Technology (B Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
@@ -1579,7 +1627,7 @@
       <x:c r="B16" s="33"/>
       <x:c r="C16" s="59"/>
       <x:c r="D16" s="52" t="str">
-        <x:f>IF($B16="","",IF(OR(RIGHT(TRIM($B16),2)="P12",RIGHT(TRIM($B16),2)="P13",RIGHT(TRIM($B16),2)="P14",RIGHT(TRIM($B16),2)="P15"),"PS","GS"))</x:f>
+        <x:f>IF($B16="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B16),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E16" s="62" t="str">
         <x:f>IF($D16="","",IF($D16="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1625,6 +1673,9 @@
       </x:c>
       <x:c r="S16" s="54" t="str">
         <x:f>IF(AND($A16="",$B16="",$C16=""),"",IF($A16="","Missing Assignment Number",IF($B16="","Select Job Title",IF($C16="","Enter Pay Rate",IF($F16="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U16" t="str">
+        <x:v>Chemical Engineer - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
@@ -1632,7 +1683,7 @@
       <x:c r="B17" s="33"/>
       <x:c r="C17" s="59"/>
       <x:c r="D17" s="52" t="str">
-        <x:f>IF($B17="","",IF(OR(RIGHT(TRIM($B17),2)="P13",RIGHT(TRIM($B17),2)="P14",RIGHT(TRIM($B17),2)="P15",RIGHT(TRIM($B17),2)="P16"),"PS","GS"))</x:f>
+        <x:f>IF($B17="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B17),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E17" s="62" t="str">
         <x:f>IF($D17="","",IF($D17="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1678,6 +1729,9 @@
       </x:c>
       <x:c r="S17" s="54" t="str">
         <x:f>IF(AND($A17="",$B17="",$C17=""),"",IF($A17="","Missing Assignment Number",IF($B17="","Select Job Title",IF($C17="","Enter Pay Rate",IF($F17="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U17" t="str">
+        <x:v>Civil Engineer - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
@@ -1685,7 +1739,7 @@
       <x:c r="B18" s="33"/>
       <x:c r="C18" s="59"/>
       <x:c r="D18" s="52" t="str">
-        <x:f>IF($B18="","",IF(OR(RIGHT(TRIM($B18),2)="P14",RIGHT(TRIM($B18),2)="P15",RIGHT(TRIM($B18),2)="P16",RIGHT(TRIM($B18),2)="P17"),"PS","GS"))</x:f>
+        <x:f>IF($B18="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B18),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E18" s="62" t="str">
         <x:f>IF($D18="","",IF($D18="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1731,6 +1785,9 @@
       </x:c>
       <x:c r="S18" s="54" t="str">
         <x:f>IF(AND($A18="",$B18="",$C18=""),"",IF($A18="","Missing Assignment Number",IF($B18="","Select Job Title",IF($C18="","Enter Pay Rate",IF($F18="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U18" t="str">
+        <x:v>Civil Engineer - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
@@ -1738,7 +1795,7 @@
       <x:c r="B19" s="33"/>
       <x:c r="C19" s="59"/>
       <x:c r="D19" s="52" t="str">
-        <x:f>IF($B19="","",IF(OR(RIGHT(TRIM($B19),2)="P15",RIGHT(TRIM($B19),2)="P16",RIGHT(TRIM($B19),2)="P17",RIGHT(TRIM($B19),2)="P18"),"PS","GS"))</x:f>
+        <x:f>IF($B19="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B19),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E19" s="62" t="str">
         <x:f>IF($D19="","",IF($D19="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1784,6 +1841,9 @@
       </x:c>
       <x:c r="S19" s="54" t="str">
         <x:f>IF(AND($A19="",$B19="",$C19=""),"",IF($A19="","Missing Assignment Number",IF($B19="","Select Job Title",IF($C19="","Enter Pay Rate",IF($F19="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U19" t="str">
+        <x:v>Compliance Specialist - I - Administrative (B Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
@@ -1791,7 +1851,7 @@
       <x:c r="B20" s="33"/>
       <x:c r="C20" s="59"/>
       <x:c r="D20" s="52" t="str">
-        <x:f>IF($B20="","",IF(OR(RIGHT(TRIM($B20),2)="P16",RIGHT(TRIM($B20),2)="P17",RIGHT(TRIM($B20),2)="P18",RIGHT(TRIM($B20),2)="P19"),"PS","GS"))</x:f>
+        <x:f>IF($B20="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B20),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E20" s="62" t="str">
         <x:f>IF($D20="","",IF($D20="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1837,6 +1897,9 @@
       </x:c>
       <x:c r="S20" s="54" t="str">
         <x:f>IF(AND($A20="",$B20="",$C20=""),"",IF($A20="","Missing Assignment Number",IF($B20="","Select Job Title",IF($C20="","Enter Pay Rate",IF($F20="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U20" t="str">
+        <x:v>Data Analyst - II - Information Communications Technology (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
@@ -1844,7 +1907,7 @@
       <x:c r="B21" s="33"/>
       <x:c r="C21" s="59"/>
       <x:c r="D21" s="52" t="str">
-        <x:f>IF($B21="","",IF(OR(RIGHT(TRIM($B21),2)="P17",RIGHT(TRIM($B21),2)="P18",RIGHT(TRIM($B21),2)="P19",RIGHT(TRIM($B21),2)="P20"),"PS","GS"))</x:f>
+        <x:f>IF($B21="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B21),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E21" s="62" t="str">
         <x:f>IF($D21="","",IF($D21="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1890,6 +1953,9 @@
       </x:c>
       <x:c r="S21" s="54" t="str">
         <x:f>IF(AND($A21="",$B21="",$C21=""),"",IF($A21="","Missing Assignment Number",IF($B21="","Select Job Title",IF($C21="","Enter Pay Rate",IF($F21="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U21" t="str">
+        <x:v>Data Entry Clerk - III - Business Support (A) Admin/Finance/HR - B3</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
@@ -1897,7 +1963,7 @@
       <x:c r="B22" s="33"/>
       <x:c r="C22" s="59"/>
       <x:c r="D22" s="52" t="str">
-        <x:f>IF($B22="","",IF(OR(RIGHT(TRIM($B22),2)="P18",RIGHT(TRIM($B22),2)="P19",RIGHT(TRIM($B22),2)="P20",RIGHT(TRIM($B22),2)="P21"),"PS","GS"))</x:f>
+        <x:f>IF($B22="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B22),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E22" s="62" t="str">
         <x:f>IF($D22="","",IF($D22="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1943,6 +2009,9 @@
       </x:c>
       <x:c r="S22" s="54" t="str">
         <x:f>IF(AND($A22="",$B22="",$C22=""),"",IF($A22="","Missing Assignment Number",IF($B22="","Select Job Title",IF($C22="","Enter Pay Rate",IF($F22="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U22" t="str">
+        <x:v>Documentation Specialist - I - Administrative (B Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
@@ -1950,7 +2019,7 @@
       <x:c r="B23" s="33"/>
       <x:c r="C23" s="59"/>
       <x:c r="D23" s="52" t="str">
-        <x:f>IF($B23="","",IF(OR(RIGHT(TRIM($B23),2)="P19",RIGHT(TRIM($B23),2)="P20",RIGHT(TRIM($B23),2)="P21",RIGHT(TRIM($B23),2)="P22"),"PS","GS"))</x:f>
+        <x:f>IF($B23="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B23),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E23" s="62" t="str">
         <x:f>IF($D23="","",IF($D23="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -1996,6 +2065,9 @@
       </x:c>
       <x:c r="S23" s="54" t="str">
         <x:f>IF(AND($A23="",$B23="",$C23=""),"",IF($A23="","Missing Assignment Number",IF($B23="","Select Job Title",IF($C23="","Enter Pay Rate",IF($F23="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U23" t="str">
+        <x:v>Documentation Specialist - III - Administrative (B Support / Professional) - B3</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
@@ -2003,7 +2075,7 @@
       <x:c r="B24" s="33"/>
       <x:c r="C24" s="59"/>
       <x:c r="D24" s="52" t="str">
-        <x:f>IF($B24="","",IF(OR(RIGHT(TRIM($B24),2)="P20",RIGHT(TRIM($B24),2)="P21",RIGHT(TRIM($B24),2)="P22",RIGHT(TRIM($B24),2)="P23"),"PS","GS"))</x:f>
+        <x:f>IF($B24="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B24),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E24" s="62" t="str">
         <x:f>IF($D24="","",IF($D24="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2049,6 +2121,9 @@
       </x:c>
       <x:c r="S24" s="54" t="str">
         <x:f>IF(AND($A24="",$B24="",$C24=""),"",IF($A24="","Missing Assignment Number",IF($B24="","Select Job Title",IF($C24="","Enter Pay Rate",IF($F24="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U24" t="str">
+        <x:v>Electrical Engineer - I - Engineering (P &amp; O Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
@@ -2056,7 +2131,7 @@
       <x:c r="B25" s="33"/>
       <x:c r="C25" s="59"/>
       <x:c r="D25" s="52" t="str">
-        <x:f>IF($B25="","",IF(OR(RIGHT(TRIM($B25),2)="P21",RIGHT(TRIM($B25),2)="P22",RIGHT(TRIM($B25),2)="P23",RIGHT(TRIM($B25),2)="P24"),"PS","GS"))</x:f>
+        <x:f>IF($B25="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B25),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E25" s="62" t="str">
         <x:f>IF($D25="","",IF($D25="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2102,6 +2177,9 @@
       </x:c>
       <x:c r="S25" s="54" t="str">
         <x:f>IF(AND($A25="",$B25="",$C25=""),"",IF($A25="","Missing Assignment Number",IF($B25="","Select Job Title",IF($C25="","Enter Pay Rate",IF($F25="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U25" t="str">
+        <x:v>Electrical Engineer - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
@@ -2109,7 +2187,7 @@
       <x:c r="B26" s="33"/>
       <x:c r="C26" s="59"/>
       <x:c r="D26" s="52" t="str">
-        <x:f>IF($B26="","",IF(OR(RIGHT(TRIM($B26),2)="P22",RIGHT(TRIM($B26),2)="P23",RIGHT(TRIM($B26),2)="P24",RIGHT(TRIM($B26),2)="P25"),"PS","GS"))</x:f>
+        <x:f>IF($B26="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B26),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E26" s="62" t="str">
         <x:f>IF($D26="","",IF($D26="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2155,6 +2233,9 @@
       </x:c>
       <x:c r="S26" s="54" t="str">
         <x:f>IF(AND($A26="",$B26="",$C26=""),"",IF($A26="","Missing Assignment Number",IF($B26="","Select Job Title",IF($C26="","Enter Pay Rate",IF($F26="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U26" t="str">
+        <x:v>Environmental Monitoring Specialist II - Environment Health &amp; Safety P&amp;O Support / Professional P2</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
@@ -2162,7 +2243,7 @@
       <x:c r="B27" s="33"/>
       <x:c r="C27" s="59"/>
       <x:c r="D27" s="52" t="str">
-        <x:f>IF($B27="","",IF(OR(RIGHT(TRIM($B27),2)="P23",RIGHT(TRIM($B27),2)="P24",RIGHT(TRIM($B27),2)="P25",RIGHT(TRIM($B27),2)="P26"),"PS","GS"))</x:f>
+        <x:f>IF($B27="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B27),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E27" s="62" t="str">
         <x:f>IF($D27="","",IF($D27="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2208,6 +2289,9 @@
       </x:c>
       <x:c r="S27" s="54" t="str">
         <x:f>IF(AND($A27="",$B27="",$C27=""),"",IF($A27="","Missing Assignment Number",IF($B27="","Select Job Title",IF($C27="","Enter Pay Rate",IF($F27="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U27" t="str">
+        <x:v>Executive Assistant - II - Business Support (A) Admin/Finance/HR - B2</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
@@ -2215,7 +2299,7 @@
       <x:c r="B28" s="33"/>
       <x:c r="C28" s="59"/>
       <x:c r="D28" s="52" t="str">
-        <x:f>IF($B28="","",IF(OR(RIGHT(TRIM($B28),2)="P24",RIGHT(TRIM($B28),2)="P25",RIGHT(TRIM($B28),2)="P26",RIGHT(TRIM($B28),2)="P27"),"PS","GS"))</x:f>
+        <x:f>IF($B28="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B28),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E28" s="62" t="str">
         <x:f>IF($D28="","",IF($D28="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2261,6 +2345,9 @@
       </x:c>
       <x:c r="S28" s="54" t="str">
         <x:f>IF(AND($A28="",$B28="",$C28=""),"",IF($A28="","Missing Assignment Number",IF($B28="","Select Job Title",IF($C28="","Enter Pay Rate",IF($F28="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U28" t="str">
+        <x:v>Health/Safety Specialist - II - Environment Health &amp; Safety (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
@@ -2268,7 +2355,7 @@
       <x:c r="B29" s="33"/>
       <x:c r="C29" s="59"/>
       <x:c r="D29" s="52" t="str">
-        <x:f>IF($B29="","",IF(OR(RIGHT(TRIM($B29),2)="P25",RIGHT(TRIM($B29),2)="P26",RIGHT(TRIM($B29),2)="P27",RIGHT(TRIM($B29),2)="P28"),"PS","GS"))</x:f>
+        <x:f>IF($B29="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B29),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E29" s="62" t="str">
         <x:f>IF($D29="","",IF($D29="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2314,6 +2401,9 @@
       </x:c>
       <x:c r="S29" s="54" t="str">
         <x:f>IF(AND($A29="",$B29="",$C29=""),"",IF($A29="","Missing Assignment Number",IF($B29="","Select Job Title",IF($C29="","Enter Pay Rate",IF($F29="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U29" t="str">
+        <x:v>Health/Safety Specialist - III - Environment Health &amp; Safety (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
@@ -2321,7 +2411,7 @@
       <x:c r="B30" s="33"/>
       <x:c r="C30" s="59"/>
       <x:c r="D30" s="52" t="str">
-        <x:f>IF($B30="","",IF(OR(RIGHT(TRIM($B30),2)="P26",RIGHT(TRIM($B30),2)="P27",RIGHT(TRIM($B30),2)="P28",RIGHT(TRIM($B30),2)="P29"),"PS","GS"))</x:f>
+        <x:f>IF($B30="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B30),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E30" s="62" t="str">
         <x:f>IF($D30="","",IF($D30="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2367,6 +2457,9 @@
       </x:c>
       <x:c r="S30" s="54" t="str">
         <x:f>IF(AND($A30="",$B30="",$C30=""),"",IF($A30="","Missing Assignment Number",IF($B30="","Select Job Title",IF($C30="","Enter Pay Rate",IF($F30="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U30" t="str">
+        <x:v>Health/Safety Specialist - IV - Environment Health &amp; Safety (P &amp; O Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
@@ -2374,7 +2467,7 @@
       <x:c r="B31" s="33"/>
       <x:c r="C31" s="59"/>
       <x:c r="D31" s="52" t="str">
-        <x:f>IF($B31="","",IF(OR(RIGHT(TRIM($B31),2)="P27",RIGHT(TRIM($B31),2)="P28",RIGHT(TRIM($B31),2)="P29",RIGHT(TRIM($B31),2)="P30"),"PS","GS"))</x:f>
+        <x:f>IF($B31="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B31),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E31" s="62" t="str">
         <x:f>IF($D31="","",IF($D31="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2420,6 +2513,9 @@
       </x:c>
       <x:c r="S31" s="54" t="str">
         <x:f>IF(AND($A31="",$B31="",$C31=""),"",IF($A31="","Missing Assignment Number",IF($B31="","Select Job Title",IF($C31="","Enter Pay Rate",IF($F31="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U31" t="str">
+        <x:v>HR Analyst - I - Human Resources (B Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
@@ -2427,7 +2523,7 @@
       <x:c r="B32" s="33"/>
       <x:c r="C32" s="59"/>
       <x:c r="D32" s="52" t="str">
-        <x:f>IF($B32="","",IF(OR(RIGHT(TRIM($B32),2)="P28",RIGHT(TRIM($B32),2)="P29",RIGHT(TRIM($B32),2)="P30",RIGHT(TRIM($B32),2)="P31"),"PS","GS"))</x:f>
+        <x:f>IF($B32="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B32),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E32" s="62" t="str">
         <x:f>IF($D32="","",IF($D32="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2473,6 +2569,9 @@
       </x:c>
       <x:c r="S32" s="54" t="str">
         <x:f>IF(AND($A32="",$B32="",$C32=""),"",IF($A32="","Missing Assignment Number",IF($B32="","Select Job Title",IF($C32="","Enter Pay Rate",IF($F32="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U32" t="str">
+        <x:v>HR Analyst - II - Human Resources (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
@@ -2480,7 +2579,7 @@
       <x:c r="B33" s="33"/>
       <x:c r="C33" s="59"/>
       <x:c r="D33" s="52" t="str">
-        <x:f>IF($B33="","",IF(OR(RIGHT(TRIM($B33),2)="P29",RIGHT(TRIM($B33),2)="P30",RIGHT(TRIM($B33),2)="P31",RIGHT(TRIM($B33),2)="P32"),"PS","GS"))</x:f>
+        <x:f>IF($B33="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B33),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E33" s="62" t="str">
         <x:f>IF($D33="","",IF($D33="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2526,6 +2625,9 @@
       </x:c>
       <x:c r="S33" s="54" t="str">
         <x:f>IF(AND($A33="",$B33="",$C33=""),"",IF($A33="","Missing Assignment Number",IF($B33="","Select Job Title",IF($C33="","Enter Pay Rate",IF($F33="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U33" t="str">
+        <x:v>Industrial Hygienist - I - Environment Health &amp; Safety P&amp;O Support / Professional - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
@@ -2533,7 +2635,7 @@
       <x:c r="B34" s="33"/>
       <x:c r="C34" s="59"/>
       <x:c r="D34" s="52" t="str">
-        <x:f>IF($B34="","",IF(OR(RIGHT(TRIM($B34),2)="P30",RIGHT(TRIM($B34),2)="P31",RIGHT(TRIM($B34),2)="P32",RIGHT(TRIM($B34),2)="P33"),"PS","GS"))</x:f>
+        <x:f>IF($B34="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B34),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E34" s="62" t="str">
         <x:f>IF($D34="","",IF($D34="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2579,6 +2681,9 @@
       </x:c>
       <x:c r="S34" s="54" t="str">
         <x:f>IF(AND($A34="",$B34="",$C34=""),"",IF($A34="","Missing Assignment Number",IF($B34="","Select Job Title",IF($C34="","Enter Pay Rate",IF($F34="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U34" t="str">
+        <x:v>Industrial Hygienist - II - Environment Health &amp; Safety P&amp;O Support / Professional - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="22" customHeight="1">
@@ -2586,7 +2691,7 @@
       <x:c r="B35" s="33"/>
       <x:c r="C35" s="59"/>
       <x:c r="D35" s="52" t="str">
-        <x:f>IF($B35="","",IF(OR(RIGHT(TRIM($B35),2)="P31",RIGHT(TRIM($B35),2)="P32",RIGHT(TRIM($B35),2)="P33",RIGHT(TRIM($B35),2)="P34"),"PS","GS"))</x:f>
+        <x:f>IF($B35="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B35),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E35" s="62" t="str">
         <x:f>IF($D35="","",IF($D35="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2632,6 +2737,9 @@
       </x:c>
       <x:c r="S35" s="54" t="str">
         <x:f>IF(AND($A35="",$B35="",$C35=""),"",IF($A35="","Missing Assignment Number",IF($B35="","Select Job Title",IF($C35="","Enter Pay Rate",IF($F35="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U35" t="str">
+        <x:v>Inspector Operator - III - Industrial (P &amp; O Support / Professional) - O3</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
@@ -2639,7 +2747,7 @@
       <x:c r="B36" s="33"/>
       <x:c r="C36" s="59"/>
       <x:c r="D36" s="52" t="str">
-        <x:f>IF($B36="","",IF(OR(RIGHT(TRIM($B36),2)="P32",RIGHT(TRIM($B36),2)="P33",RIGHT(TRIM($B36),2)="P34",RIGHT(TRIM($B36),2)="P35"),"PS","GS"))</x:f>
+        <x:f>IF($B36="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B36),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E36" s="62" t="str">
         <x:f>IF($D36="","",IF($D36="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2685,6 +2793,9 @@
       </x:c>
       <x:c r="S36" s="54" t="str">
         <x:f>IF(AND($A36="",$B36="",$C36=""),"",IF($A36="","Missing Assignment Number",IF($B36="","Select Job Title",IF($C36="","Enter Pay Rate",IF($F36="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U36" t="str">
+        <x:v>Lab Assistant - III - Business Support (T) Science/Medical/Clinical - B3</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
@@ -2692,7 +2803,7 @@
       <x:c r="B37" s="33"/>
       <x:c r="C37" s="59"/>
       <x:c r="D37" s="52" t="str">
-        <x:f>IF($B37="","",IF(OR(RIGHT(TRIM($B37),2)="P33",RIGHT(TRIM($B37),2)="P34",RIGHT(TRIM($B37),2)="P35",RIGHT(TRIM($B37),2)="P36"),"PS","GS"))</x:f>
+        <x:f>IF($B37="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B37),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E37" s="62" t="str">
         <x:f>IF($D37="","",IF($D37="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2738,6 +2849,9 @@
       </x:c>
       <x:c r="S37" s="54" t="str">
         <x:f>IF(AND($A37="",$B37="",$C37=""),"",IF($A37="","Missing Assignment Number",IF($B37="","Select Job Title",IF($C37="","Enter Pay Rate",IF($F37="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U37" t="str">
+        <x:v>Lab Technician - Animal - II - Production &amp; Operations Support (T) Science/Medical/Clinical - O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="22" customHeight="1">
@@ -2745,7 +2859,7 @@
       <x:c r="B38" s="33"/>
       <x:c r="C38" s="59"/>
       <x:c r="D38" s="52" t="str">
-        <x:f>IF($B38="","",IF(OR(RIGHT(TRIM($B38),2)="P34",RIGHT(TRIM($B38),2)="P35",RIGHT(TRIM($B38),2)="P36",RIGHT(TRIM($B38),2)="P37"),"PS","GS"))</x:f>
+        <x:f>IF($B38="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B38),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E38" s="62" t="str">
         <x:f>IF($D38="","",IF($D38="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2791,6 +2905,9 @@
       </x:c>
       <x:c r="S38" s="54" t="str">
         <x:f>IF(AND($A38="",$B38="",$C38=""),"",IF($A38="","Missing Assignment Number",IF($B38="","Select Job Title",IF($C38="","Enter Pay Rate",IF($F38="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U38" t="str">
+        <x:v>Lab Technician - II - Production &amp; Operations Support (T) Science/Medical/Clinical - O2 (High)</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
@@ -2798,7 +2915,7 @@
       <x:c r="B39" s="33"/>
       <x:c r="C39" s="59"/>
       <x:c r="D39" s="52" t="str">
-        <x:f>IF($B39="","",IF(OR(RIGHT(TRIM($B39),2)="P35",RIGHT(TRIM($B39),2)="P36",RIGHT(TRIM($B39),2)="P37",RIGHT(TRIM($B39),2)="P38"),"PS","GS"))</x:f>
+        <x:f>IF($B39="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B39),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E39" s="62" t="str">
         <x:f>IF($D39="","",IF($D39="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2844,6 +2961,9 @@
       </x:c>
       <x:c r="S39" s="54" t="str">
         <x:f>IF(AND($A39="",$B39="",$C39=""),"",IF($A39="","Missing Assignment Number",IF($B39="","Select Job Title",IF($C39="","Enter Pay Rate",IF($F39="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U39" t="str">
+        <x:v>Lab Technician - II - Production &amp; Operations Support (T) Science/Medical/Clinical - O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="22" customHeight="1">
@@ -2851,7 +2971,7 @@
       <x:c r="B40" s="33"/>
       <x:c r="C40" s="59"/>
       <x:c r="D40" s="52" t="str">
-        <x:f>IF($B40="","",IF(OR(RIGHT(TRIM($B40),2)="P36",RIGHT(TRIM($B40),2)="P37",RIGHT(TRIM($B40),2)="P38",RIGHT(TRIM($B40),2)="P39"),"PS","GS"))</x:f>
+        <x:f>IF($B40="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B40),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E40" s="62" t="str">
         <x:f>IF($D40="","",IF($D40="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2897,6 +3017,9 @@
       </x:c>
       <x:c r="S40" s="54" t="str">
         <x:f>IF(AND($A40="",$B40="",$C40=""),"",IF($A40="","Missing Assignment Number",IF($B40="","Select Job Title",IF($C40="","Enter Pay Rate",IF($F40="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U40" t="str">
+        <x:v>Lab Technician - III - Production &amp; Operations Support (T) Science/Medical/Clinical - O3</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
@@ -2904,7 +3027,7 @@
       <x:c r="B41" s="33"/>
       <x:c r="C41" s="59"/>
       <x:c r="D41" s="52" t="str">
-        <x:f>IF($B41="","",IF(OR(RIGHT(TRIM($B41),2)="P37",RIGHT(TRIM($B41),2)="P38",RIGHT(TRIM($B41),2)="P39",RIGHT(TRIM($B41),2)="P40"),"PS","GS"))</x:f>
+        <x:f>IF($B41="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B41),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E41" s="62" t="str">
         <x:f>IF($D41="","",IF($D41="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -2950,6 +3073,9 @@
       </x:c>
       <x:c r="S41" s="54" t="str">
         <x:f>IF(AND($A41="",$B41="",$C41=""),"",IF($A41="","Missing Assignment Number",IF($B41="","Select Job Title",IF($C41="","Enter Pay Rate",IF($F41="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U41" t="str">
+        <x:v>Maintenance Technician - II - Production &amp; Operations Support (T): Industrial - O2 (High)</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
@@ -2957,7 +3083,7 @@
       <x:c r="B42" s="33"/>
       <x:c r="C42" s="59"/>
       <x:c r="D42" s="52" t="str">
-        <x:f>IF($B42="","",IF(OR(RIGHT(TRIM($B42),2)="P38",RIGHT(TRIM($B42),2)="P39",RIGHT(TRIM($B42),2)="P40",RIGHT(TRIM($B42),2)="P41"),"PS","GS"))</x:f>
+        <x:f>IF($B42="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B42),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E42" s="62" t="str">
         <x:f>IF($D42="","",IF($D42="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3003,6 +3129,9 @@
       </x:c>
       <x:c r="S42" s="54" t="str">
         <x:f>IF(AND($A42="",$B42="",$C42=""),"",IF($A42="","Missing Assignment Number",IF($B42="","Select Job Title",IF($C42="","Enter Pay Rate",IF($F42="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U42" t="str">
+        <x:v>Maintenance Technician - II - Production &amp; Operations Support (T): Industrial O2 High – PS</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
@@ -3010,7 +3139,7 @@
       <x:c r="B43" s="33"/>
       <x:c r="C43" s="59"/>
       <x:c r="D43" s="52" t="str">
-        <x:f>IF($B43="","",IF(OR(RIGHT(TRIM($B43),2)="P39",RIGHT(TRIM($B43),2)="P40",RIGHT(TRIM($B43),2)="P41",RIGHT(TRIM($B43),2)="P42"),"PS","GS"))</x:f>
+        <x:f>IF($B43="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B43),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E43" s="62" t="str">
         <x:f>IF($D43="","",IF($D43="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3056,6 +3185,9 @@
       </x:c>
       <x:c r="S43" s="54" t="str">
         <x:f>IF(AND($A43="",$B43="",$C43=""),"",IF($A43="","Missing Assignment Number",IF($B43="","Select Job Title",IF($C43="","Enter Pay Rate",IF($F43="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U43" t="str">
+        <x:v>Maintenance Technician - II - Production &amp; Operations Support (T): Industrial O3 – PS</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
@@ -3063,7 +3195,7 @@
       <x:c r="B44" s="33"/>
       <x:c r="C44" s="59"/>
       <x:c r="D44" s="52" t="str">
-        <x:f>IF($B44="","",IF(OR(RIGHT(TRIM($B44),2)="P40",RIGHT(TRIM($B44),2)="P41",RIGHT(TRIM($B44),2)="P42",RIGHT(TRIM($B44),2)="P43"),"PS","GS"))</x:f>
+        <x:f>IF($B44="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B44),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E44" s="62" t="str">
         <x:f>IF($D44="","",IF($D44="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3109,6 +3241,9 @@
       </x:c>
       <x:c r="S44" s="54" t="str">
         <x:f>IF(AND($A44="",$B44="",$C44=""),"",IF($A44="","Missing Assignment Number",IF($B44="","Select Job Title",IF($C44="","Enter Pay Rate",IF($F44="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U44" t="str">
+        <x:v>Maintenance Technician - II - Production &amp; Operations Support (T): Industrial O4 – PS</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
@@ -3116,7 +3251,7 @@
       <x:c r="B45" s="33"/>
       <x:c r="C45" s="59"/>
       <x:c r="D45" s="52" t="str">
-        <x:f>IF($B45="","",IF(OR(RIGHT(TRIM($B45),2)="P41",RIGHT(TRIM($B45),2)="P42",RIGHT(TRIM($B45),2)="P43",RIGHT(TRIM($B45),2)="P44"),"PS","GS"))</x:f>
+        <x:f>IF($B45="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B45),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E45" s="62" t="str">
         <x:f>IF($D45="","",IF($D45="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3162,6 +3297,9 @@
       </x:c>
       <x:c r="S45" s="54" t="str">
         <x:f>IF(AND($A45="",$B45="",$C45=""),"",IF($A45="","Missing Assignment Number",IF($B45="","Select Job Title",IF($C45="","Enter Pay Rate",IF($F45="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U45" t="str">
+        <x:v>Maintenance Technician - IV - Production &amp; Operations Support (T): Industrial - O4</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="22" customHeight="1">
@@ -3169,7 +3307,7 @@
       <x:c r="B46" s="33"/>
       <x:c r="C46" s="59"/>
       <x:c r="D46" s="52" t="str">
-        <x:f>IF($B46="","",IF(OR(RIGHT(TRIM($B46),2)="P42",RIGHT(TRIM($B46),2)="P43",RIGHT(TRIM($B46),2)="P44",RIGHT(TRIM($B46),2)="P45"),"PS","GS"))</x:f>
+        <x:f>IF($B46="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B46),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E46" s="62" t="str">
         <x:f>IF($D46="","",IF($D46="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3215,6 +3353,9 @@
       </x:c>
       <x:c r="S46" s="54" t="str">
         <x:f>IF(AND($A46="",$B46="",$C46=""),"",IF($A46="","Missing Assignment Number",IF($B46="","Select Job Title",IF($C46="","Enter Pay Rate",IF($F46="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U46" t="str">
+        <x:v>Marketing Research Specialist - II - Creative (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="22" customHeight="1">
@@ -3222,7 +3363,7 @@
       <x:c r="B47" s="33"/>
       <x:c r="C47" s="59"/>
       <x:c r="D47" s="52" t="str">
-        <x:f>IF($B47="","",IF(OR(RIGHT(TRIM($B47),2)="P43",RIGHT(TRIM($B47),2)="P44",RIGHT(TRIM($B47),2)="P45",RIGHT(TRIM($B47),2)="P46"),"PS","GS"))</x:f>
+        <x:f>IF($B47="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B47),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E47" s="62" t="str">
         <x:f>IF($D47="","",IF($D47="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3268,6 +3409,9 @@
       </x:c>
       <x:c r="S47" s="54" t="str">
         <x:f>IF(AND($A47="",$B47="",$C47=""),"",IF($A47="","Missing Assignment Number",IF($B47="","Select Job Title",IF($C47="","Enter Pay Rate",IF($F47="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U47" t="str">
+        <x:v>Mechanical Engineer - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="22" customHeight="1">
@@ -3275,7 +3419,7 @@
       <x:c r="B48" s="33"/>
       <x:c r="C48" s="59"/>
       <x:c r="D48" s="52" t="str">
-        <x:f>IF($B48="","",IF(OR(RIGHT(TRIM($B48),2)="P44",RIGHT(TRIM($B48),2)="P45",RIGHT(TRIM($B48),2)="P46",RIGHT(TRIM($B48),2)="P47"),"PS","GS"))</x:f>
+        <x:f>IF($B48="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B48),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E48" s="62" t="str">
         <x:f>IF($D48="","",IF($D48="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3321,6 +3465,9 @@
       </x:c>
       <x:c r="S48" s="54" t="str">
         <x:f>IF(AND($A48="",$B48="",$C48=""),"",IF($A48="","Missing Assignment Number",IF($B48="","Select Job Title",IF($C48="","Enter Pay Rate",IF($F48="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U48" t="str">
+        <x:v>Mechanical Engineer - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="22" customHeight="1">
@@ -3328,7 +3475,7 @@
       <x:c r="B49" s="33"/>
       <x:c r="C49" s="59"/>
       <x:c r="D49" s="52" t="str">
-        <x:f>IF($B49="","",IF(OR(RIGHT(TRIM($B49),2)="P45",RIGHT(TRIM($B49),2)="P46",RIGHT(TRIM($B49),2)="P47",RIGHT(TRIM($B49),2)="P48"),"PS","GS"))</x:f>
+        <x:f>IF($B49="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B49),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E49" s="62" t="str">
         <x:f>IF($D49="","",IF($D49="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3374,6 +3521,9 @@
       </x:c>
       <x:c r="S49" s="54" t="str">
         <x:f>IF(AND($A49="",$B49="",$C49=""),"",IF($A49="","Missing Assignment Number",IF($B49="","Select Job Title",IF($C49="","Enter Pay Rate",IF($F49="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U49" t="str">
+        <x:v>Operations Manager - I - Industrial (P &amp; O Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="22" customHeight="1">
@@ -3381,7 +3531,7 @@
       <x:c r="B50" s="33"/>
       <x:c r="C50" s="59"/>
       <x:c r="D50" s="52" t="str">
-        <x:f>IF($B50="","",IF(OR(RIGHT(TRIM($B50),2)="P46",RIGHT(TRIM($B50),2)="P47",RIGHT(TRIM($B50),2)="P48",RIGHT(TRIM($B50),2)="P49"),"PS","GS"))</x:f>
+        <x:f>IF($B50="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B50),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E50" s="62" t="str">
         <x:f>IF($D50="","",IF($D50="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3427,6 +3577,9 @@
       </x:c>
       <x:c r="S50" s="54" t="str">
         <x:f>IF(AND($A50="",$B50="",$C50=""),"",IF($A50="","Missing Assignment Number",IF($B50="","Select Job Title",IF($C50="","Enter Pay Rate",IF($F50="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U50" t="str">
+        <x:v>Operations Manager - II - Industrial (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
@@ -3434,7 +3587,7 @@
       <x:c r="B51" s="33"/>
       <x:c r="C51" s="59"/>
       <x:c r="D51" s="52" t="str">
-        <x:f>IF($B51="","",IF(OR(RIGHT(TRIM($B51),2)="P47",RIGHT(TRIM($B51),2)="P48",RIGHT(TRIM($B51),2)="P49",RIGHT(TRIM($B51),2)="P50"),"PS","GS"))</x:f>
+        <x:f>IF($B51="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B51),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E51" s="62" t="str">
         <x:f>IF($D51="","",IF($D51="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3480,6 +3633,9 @@
       </x:c>
       <x:c r="S51" s="54" t="str">
         <x:f>IF(AND($A51="",$B51="",$C51=""),"",IF($A51="","Missing Assignment Number",IF($B51="","Select Job Title",IF($C51="","Enter Pay Rate",IF($F51="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U51" t="str">
+        <x:v>Operations Manager - IV - Industrial (P &amp; O Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
@@ -3487,7 +3643,7 @@
       <x:c r="B52" s="33"/>
       <x:c r="C52" s="59"/>
       <x:c r="D52" s="52" t="str">
-        <x:f>IF($B52="","",IF(OR(RIGHT(TRIM($B52),2)="P48",RIGHT(TRIM($B52),2)="P49",RIGHT(TRIM($B52),2)="P50",RIGHT(TRIM($B52),2)="P51"),"PS","GS"))</x:f>
+        <x:f>IF($B52="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B52),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E52" s="62" t="str">
         <x:f>IF($D52="","",IF($D52="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3533,6 +3689,9 @@
       </x:c>
       <x:c r="S52" s="54" t="str">
         <x:f>IF(AND($A52="",$B52="",$C52=""),"",IF($A52="","Missing Assignment Number",IF($B52="","Select Job Title",IF($C52="","Enter Pay Rate",IF($F52="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U52" t="str">
+        <x:v>Packaging Engineer - II - Industrial (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
@@ -3540,7 +3699,7 @@
       <x:c r="B53" s="33"/>
       <x:c r="C53" s="59"/>
       <x:c r="D53" s="52" t="str">
-        <x:f>IF($B53="","",IF(OR(RIGHT(TRIM($B53),2)="P49",RIGHT(TRIM($B53),2)="P50",RIGHT(TRIM($B53),2)="P51",RIGHT(TRIM($B53),2)="P52"),"PS","GS"))</x:f>
+        <x:f>IF($B53="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B53),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E53" s="62" t="str">
         <x:f>IF($D53="","",IF($D53="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3586,6 +3745,9 @@
       </x:c>
       <x:c r="S53" s="54" t="str">
         <x:f>IF(AND($A53="",$B53="",$C53=""),"",IF($A53="","Missing Assignment Number",IF($B53="","Select Job Title",IF($C53="","Enter Pay Rate",IF($F53="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U53" t="str">
+        <x:v>Packaging Operator - I - Production &amp; Operations Support (T): Industrial - O1</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="22" customHeight="1">
@@ -3593,7 +3755,7 @@
       <x:c r="B54" s="33"/>
       <x:c r="C54" s="59"/>
       <x:c r="D54" s="52" t="str">
-        <x:f>IF($B54="","",IF(OR(RIGHT(TRIM($B54),2)="P50",RIGHT(TRIM($B54),2)="P51",RIGHT(TRIM($B54),2)="P52",RIGHT(TRIM($B54),2)="P53"),"PS","GS"))</x:f>
+        <x:f>IF($B54="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B54),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E54" s="62" t="str">
         <x:f>IF($D54="","",IF($D54="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3639,6 +3801,9 @@
       </x:c>
       <x:c r="S54" s="54" t="str">
         <x:f>IF(AND($A54="",$B54="",$C54=""),"",IF($A54="","Missing Assignment Number",IF($B54="","Select Job Title",IF($C54="","Enter Pay Rate",IF($F54="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U54" t="str">
+        <x:v>Packaging Operator - II - Production &amp; Operations Support (T): Industrial - O2 (Low)</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="22" customHeight="1">
@@ -3646,7 +3811,7 @@
       <x:c r="B55" s="33"/>
       <x:c r="C55" s="59"/>
       <x:c r="D55" s="52" t="str">
-        <x:f>IF($B55="","",IF(OR(RIGHT(TRIM($B55),2)="P51",RIGHT(TRIM($B55),2)="P52",RIGHT(TRIM($B55),2)="P53",RIGHT(TRIM($B55),2)="P54"),"PS","GS"))</x:f>
+        <x:f>IF($B55="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B55),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E55" s="62" t="str">
         <x:f>IF($D55="","",IF($D55="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3692,6 +3857,9 @@
       </x:c>
       <x:c r="S55" s="54" t="str">
         <x:f>IF(AND($A55="",$B55="",$C55=""),"",IF($A55="","Missing Assignment Number",IF($B55="","Select Job Title",IF($C55="","Enter Pay Rate",IF($F55="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U55" t="str">
+        <x:v>Packaging Operator - II - Production &amp; Operations Support (T): Industrial - O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="22" customHeight="1">
@@ -3699,7 +3867,7 @@
       <x:c r="B56" s="33"/>
       <x:c r="C56" s="59"/>
       <x:c r="D56" s="52" t="str">
-        <x:f>IF($B56="","",IF(OR(RIGHT(TRIM($B56),2)="P52",RIGHT(TRIM($B56),2)="P53",RIGHT(TRIM($B56),2)="P54",RIGHT(TRIM($B56),2)="P55"),"PS","GS"))</x:f>
+        <x:f>IF($B56="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B56),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E56" s="62" t="str">
         <x:f>IF($D56="","",IF($D56="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3745,6 +3913,9 @@
       </x:c>
       <x:c r="S56" s="54" t="str">
         <x:f>IF(AND($A56="",$B56="",$C56=""),"",IF($A56="","Missing Assignment Number",IF($B56="","Select Job Title",IF($C56="","Enter Pay Rate",IF($F56="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U56" t="str">
+        <x:v>Packaging Operator - III - Production &amp; Operations Support (T): Industrial - O3</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="22" customHeight="1">
@@ -3752,7 +3923,7 @@
       <x:c r="B57" s="33"/>
       <x:c r="C57" s="59"/>
       <x:c r="D57" s="52" t="str">
-        <x:f>IF($B57="","",IF(OR(RIGHT(TRIM($B57),2)="P53",RIGHT(TRIM($B57),2)="P54",RIGHT(TRIM($B57),2)="P55",RIGHT(TRIM($B57),2)="P56"),"PS","GS"))</x:f>
+        <x:f>IF($B57="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B57),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E57" s="62" t="str">
         <x:f>IF($D57="","",IF($D57="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3798,6 +3969,9 @@
       </x:c>
       <x:c r="S57" s="54" t="str">
         <x:f>IF(AND($A57="",$B57="",$C57=""),"",IF($A57="","Missing Assignment Number",IF($B57="","Select Job Title",IF($C57="","Enter Pay Rate",IF($F57="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U57" t="str">
+        <x:v>Pharmaceutical Specialist - I - Engineering (P &amp; O Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="22" customHeight="1">
@@ -3805,7 +3979,7 @@
       <x:c r="B58" s="33"/>
       <x:c r="C58" s="59"/>
       <x:c r="D58" s="52" t="str">
-        <x:f>IF($B58="","",IF(OR(RIGHT(TRIM($B58),2)="P54",RIGHT(TRIM($B58),2)="P55",RIGHT(TRIM($B58),2)="P56",RIGHT(TRIM($B58),2)="P57"),"PS","GS"))</x:f>
+        <x:f>IF($B58="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B58),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E58" s="62" t="str">
         <x:f>IF($D58="","",IF($D58="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3851,6 +4025,9 @@
       </x:c>
       <x:c r="S58" s="54" t="str">
         <x:f>IF(AND($A58="",$B58="",$C58=""),"",IF($A58="","Missing Assignment Number",IF($B58="","Select Job Title",IF($C58="","Enter Pay Rate",IF($F58="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U58" t="str">
+        <x:v>Pharmaceutical Specialist - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="22" customHeight="1">
@@ -3858,7 +4035,7 @@
       <x:c r="B59" s="33"/>
       <x:c r="C59" s="59"/>
       <x:c r="D59" s="52" t="str">
-        <x:f>IF($B59="","",IF(OR(RIGHT(TRIM($B59),2)="P55",RIGHT(TRIM($B59),2)="P56",RIGHT(TRIM($B59),2)="P57",RIGHT(TRIM($B59),2)="P58"),"PS","GS"))</x:f>
+        <x:f>IF($B59="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B59),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E59" s="62" t="str">
         <x:f>IF($D59="","",IF($D59="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3904,6 +4081,9 @@
       </x:c>
       <x:c r="S59" s="54" t="str">
         <x:f>IF(AND($A59="",$B59="",$C59=""),"",IF($A59="","Missing Assignment Number",IF($B59="","Select Job Title",IF($C59="","Enter Pay Rate",IF($F59="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U59" t="str">
+        <x:v>Process Engineer - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="22" customHeight="1">
@@ -3911,7 +4091,7 @@
       <x:c r="B60" s="33"/>
       <x:c r="C60" s="59"/>
       <x:c r="D60" s="52" t="str">
-        <x:f>IF($B60="","",IF(OR(RIGHT(TRIM($B60),2)="P56",RIGHT(TRIM($B60),2)="P57",RIGHT(TRIM($B60),2)="P58",RIGHT(TRIM($B60),2)="P59"),"PS","GS"))</x:f>
+        <x:f>IF($B60="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B60),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E60" s="62" t="str">
         <x:f>IF($D60="","",IF($D60="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -3957,6 +4137,9 @@
       </x:c>
       <x:c r="S60" s="54" t="str">
         <x:f>IF(AND($A60="",$B60="",$C60=""),"",IF($A60="","Missing Assignment Number",IF($B60="","Select Job Title",IF($C60="","Enter Pay Rate",IF($F60="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U60" t="str">
+        <x:v>Process Engineer - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="22" customHeight="1">
@@ -3964,7 +4147,7 @@
       <x:c r="B61" s="33"/>
       <x:c r="C61" s="59"/>
       <x:c r="D61" s="52" t="str">
-        <x:f>IF($B61="","",IF(OR(RIGHT(TRIM($B61),2)="P57",RIGHT(TRIM($B61),2)="P58",RIGHT(TRIM($B61),2)="P59",RIGHT(TRIM($B61),2)="P60"),"PS","GS"))</x:f>
+        <x:f>IF($B61="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B61),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E61" s="62" t="str">
         <x:f>IF($D61="","",IF($D61="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4010,6 +4193,9 @@
       </x:c>
       <x:c r="S61" s="54" t="str">
         <x:f>IF(AND($A61="",$B61="",$C61=""),"",IF($A61="","Missing Assignment Number",IF($B61="","Select Job Title",IF($C61="","Enter Pay Rate",IF($F61="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U61" t="str">
+        <x:v>Process Engineer - IV - Engineering (P &amp; O Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="22" customHeight="1">
@@ -4017,7 +4203,7 @@
       <x:c r="B62" s="33"/>
       <x:c r="C62" s="59"/>
       <x:c r="D62" s="52" t="str">
-        <x:f>IF($B62="","",IF(OR(RIGHT(TRIM($B62),2)="P58",RIGHT(TRIM($B62),2)="P59",RIGHT(TRIM($B62),2)="P60",RIGHT(TRIM($B62),2)="P61"),"PS","GS"))</x:f>
+        <x:f>IF($B62="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B62),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E62" s="62" t="str">
         <x:f>IF($D62="","",IF($D62="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4063,6 +4249,9 @@
       </x:c>
       <x:c r="S62" s="54" t="str">
         <x:f>IF(AND($A62="",$B62="",$C62=""),"",IF($A62="","Missing Assignment Number",IF($B62="","Select Job Title",IF($C62="","Enter Pay Rate",IF($F62="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U62" t="str">
+        <x:v>Procurement Specialist - III - Administrative (B Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="22" customHeight="1">
@@ -4070,7 +4259,7 @@
       <x:c r="B63" s="33"/>
       <x:c r="C63" s="59"/>
       <x:c r="D63" s="52" t="str">
-        <x:f>IF($B63="","",IF(OR(RIGHT(TRIM($B63),2)="P59",RIGHT(TRIM($B63),2)="P60",RIGHT(TRIM($B63),2)="P61",RIGHT(TRIM($B63),2)="P62"),"PS","GS"))</x:f>
+        <x:f>IF($B63="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B63),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E63" s="62" t="str">
         <x:f>IF($D63="","",IF($D63="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4116,6 +4305,9 @@
       </x:c>
       <x:c r="S63" s="54" t="str">
         <x:f>IF(AND($A63="",$B63="",$C63=""),"",IF($A63="","Missing Assignment Number",IF($B63="","Select Job Title",IF($C63="","Enter Pay Rate",IF($F63="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U63" t="str">
+        <x:v>Production Operator - II - Production &amp; Operations Support (T): Industrial - O2 (High)</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="22" customHeight="1">
@@ -4123,7 +4315,7 @@
       <x:c r="B64" s="33"/>
       <x:c r="C64" s="59"/>
       <x:c r="D64" s="52" t="str">
-        <x:f>IF($B64="","",IF(OR(RIGHT(TRIM($B64),2)="P60",RIGHT(TRIM($B64),2)="P61",RIGHT(TRIM($B64),2)="P62",RIGHT(TRIM($B64),2)="P63"),"PS","GS"))</x:f>
+        <x:f>IF($B64="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B64),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E64" s="62" t="str">
         <x:f>IF($D64="","",IF($D64="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4169,6 +4361,9 @@
       </x:c>
       <x:c r="S64" s="54" t="str">
         <x:f>IF(AND($A64="",$B64="",$C64=""),"",IF($A64="","Missing Assignment Number",IF($B64="","Select Job Title",IF($C64="","Enter Pay Rate",IF($F64="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U64" t="str">
+        <x:v>Production Operator - II - Production &amp; Operations Support (T): Industrial - O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="22" customHeight="1">
@@ -4176,7 +4371,7 @@
       <x:c r="B65" s="33"/>
       <x:c r="C65" s="59"/>
       <x:c r="D65" s="52" t="str">
-        <x:f>IF($B65="","",IF(OR(RIGHT(TRIM($B65),2)="P61",RIGHT(TRIM($B65),2)="P62",RIGHT(TRIM($B65),2)="P63",RIGHT(TRIM($B65),2)="P64"),"PS","GS"))</x:f>
+        <x:f>IF($B65="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B65),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E65" s="62" t="str">
         <x:f>IF($D65="","",IF($D65="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4222,6 +4417,9 @@
       </x:c>
       <x:c r="S65" s="54" t="str">
         <x:f>IF(AND($A65="",$B65="",$C65=""),"",IF($A65="","Missing Assignment Number",IF($B65="","Select Job Title",IF($C65="","Enter Pay Rate",IF($F65="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U65" t="str">
+        <x:v>Production Tech - II - Production &amp; Operations Support (T): Industrial - O2 (High)</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="22" customHeight="1">
@@ -4229,7 +4427,7 @@
       <x:c r="B66" s="33"/>
       <x:c r="C66" s="59"/>
       <x:c r="D66" s="52" t="str">
-        <x:f>IF($B66="","",IF(OR(RIGHT(TRIM($B66),2)="P62",RIGHT(TRIM($B66),2)="P63",RIGHT(TRIM($B66),2)="P64",RIGHT(TRIM($B66),2)="P65"),"PS","GS"))</x:f>
+        <x:f>IF($B66="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B66),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E66" s="62" t="str">
         <x:f>IF($D66="","",IF($D66="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4275,6 +4473,9 @@
       </x:c>
       <x:c r="S66" s="54" t="str">
         <x:f>IF(AND($A66="",$B66="",$C66=""),"",IF($A66="","Missing Assignment Number",IF($B66="","Select Job Title",IF($C66="","Enter Pay Rate",IF($F66="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U66" t="str">
+        <x:v>Production Tech - II - Production &amp; Operations Support (T): Industrial - O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="22" customHeight="1">
@@ -4282,7 +4483,7 @@
       <x:c r="B67" s="33"/>
       <x:c r="C67" s="59"/>
       <x:c r="D67" s="52" t="str">
-        <x:f>IF($B67="","",IF(OR(RIGHT(TRIM($B67),2)="P63",RIGHT(TRIM($B67),2)="P64",RIGHT(TRIM($B67),2)="P65",RIGHT(TRIM($B67),2)="P66"),"PS","GS"))</x:f>
+        <x:f>IF($B67="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B67),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E67" s="62" t="str">
         <x:f>IF($D67="","",IF($D67="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4328,6 +4529,9 @@
       </x:c>
       <x:c r="S67" s="54" t="str">
         <x:f>IF(AND($A67="",$B67="",$C67=""),"",IF($A67="","Missing Assignment Number",IF($B67="","Select Job Title",IF($C67="","Enter Pay Rate",IF($F67="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U67" t="str">
+        <x:v>Project Coordinator - I - Administrative (B Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="22" customHeight="1">
@@ -4335,7 +4539,7 @@
       <x:c r="B68" s="33"/>
       <x:c r="C68" s="59"/>
       <x:c r="D68" s="52" t="str">
-        <x:f>IF($B68="","",IF(OR(RIGHT(TRIM($B68),2)="P64",RIGHT(TRIM($B68),2)="P65",RIGHT(TRIM($B68),2)="P66",RIGHT(TRIM($B68),2)="P67"),"PS","GS"))</x:f>
+        <x:f>IF($B68="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B68),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E68" s="62" t="str">
         <x:f>IF($D68="","",IF($D68="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4381,6 +4585,9 @@
       </x:c>
       <x:c r="S68" s="54" t="str">
         <x:f>IF(AND($A68="",$B68="",$C68=""),"",IF($A68="","Missing Assignment Number",IF($B68="","Select Job Title",IF($C68="","Enter Pay Rate",IF($F68="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U68" t="str">
+        <x:v>Project Coordinator - II - Administrative (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="22" customHeight="1">
@@ -4388,7 +4595,7 @@
       <x:c r="B69" s="33"/>
       <x:c r="C69" s="59"/>
       <x:c r="D69" s="52" t="str">
-        <x:f>IF($B69="","",IF(OR(RIGHT(TRIM($B69),2)="P65",RIGHT(TRIM($B69),2)="P66",RIGHT(TRIM($B69),2)="P67",RIGHT(TRIM($B69),2)="P68"),"PS","GS"))</x:f>
+        <x:f>IF($B69="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B69),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E69" s="62" t="str">
         <x:f>IF($D69="","",IF($D69="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4434,6 +4641,9 @@
       </x:c>
       <x:c r="S69" s="54" t="str">
         <x:f>IF(AND($A69="",$B69="",$C69=""),"",IF($A69="","Missing Assignment Number",IF($B69="","Select Job Title",IF($C69="","Enter Pay Rate",IF($F69="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U69" t="str">
+        <x:v>Project Manager - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="22" customHeight="1">
@@ -4441,7 +4651,7 @@
       <x:c r="B70" s="33"/>
       <x:c r="C70" s="59"/>
       <x:c r="D70" s="52" t="str">
-        <x:f>IF($B70="","",IF(OR(RIGHT(TRIM($B70),2)="P66",RIGHT(TRIM($B70),2)="P67",RIGHT(TRIM($B70),2)="P68",RIGHT(TRIM($B70),2)="P69"),"PS","GS"))</x:f>
+        <x:f>IF($B70="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B70),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E70" s="62" t="str">
         <x:f>IF($D70="","",IF($D70="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4487,6 +4697,9 @@
       </x:c>
       <x:c r="S70" s="54" t="str">
         <x:f>IF(AND($A70="",$B70="",$C70=""),"",IF($A70="","Missing Assignment Number",IF($B70="","Select Job Title",IF($C70="","Enter Pay Rate",IF($F70="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U70" t="str">
+        <x:v>Project Manager - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="22" customHeight="1">
@@ -4494,7 +4707,7 @@
       <x:c r="B71" s="33"/>
       <x:c r="C71" s="59"/>
       <x:c r="D71" s="52" t="str">
-        <x:f>IF($B71="","",IF(OR(RIGHT(TRIM($B71),2)="P67",RIGHT(TRIM($B71),2)="P68",RIGHT(TRIM($B71),2)="P69",RIGHT(TRIM($B71),2)="P70"),"PS","GS"))</x:f>
+        <x:f>IF($B71="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B71),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E71" s="62" t="str">
         <x:f>IF($D71="","",IF($D71="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4540,6 +4753,9 @@
       </x:c>
       <x:c r="S71" s="54" t="str">
         <x:f>IF(AND($A71="",$B71="",$C71=""),"",IF($A71="","Missing Assignment Number",IF($B71="","Select Job Title",IF($C71="","Enter Pay Rate",IF($F71="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U71" t="str">
+        <x:v>Project Manager - IT - II - Information Communications Technology (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="22" customHeight="1">
@@ -4547,7 +4763,7 @@
       <x:c r="B72" s="33"/>
       <x:c r="C72" s="59"/>
       <x:c r="D72" s="52" t="str">
-        <x:f>IF($B72="","",IF(OR(RIGHT(TRIM($B72),2)="P68",RIGHT(TRIM($B72),2)="P69",RIGHT(TRIM($B72),2)="P70",RIGHT(TRIM($B72),2)="P71"),"PS","GS"))</x:f>
+        <x:f>IF($B72="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B72),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E72" s="62" t="str">
         <x:f>IF($D72="","",IF($D72="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4593,6 +4809,9 @@
       </x:c>
       <x:c r="S72" s="54" t="str">
         <x:f>IF(AND($A72="",$B72="",$C72=""),"",IF($A72="","Missing Assignment Number",IF($B72="","Select Job Title",IF($C72="","Enter Pay Rate",IF($F72="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U72" t="str">
+        <x:v>Project Manager - IT - III - Information Communications Technology (B Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="22" customHeight="1">
@@ -4600,7 +4819,7 @@
       <x:c r="B73" s="33"/>
       <x:c r="C73" s="59"/>
       <x:c r="D73" s="52" t="str">
-        <x:f>IF($B73="","",IF(OR(RIGHT(TRIM($B73),2)="P69",RIGHT(TRIM($B73),2)="P70",RIGHT(TRIM($B73),2)="P71",RIGHT(TRIM($B73),2)="P72"),"PS","GS"))</x:f>
+        <x:f>IF($B73="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B73),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E73" s="62" t="str">
         <x:f>IF($D73="","",IF($D73="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4646,6 +4865,9 @@
       </x:c>
       <x:c r="S73" s="54" t="str">
         <x:f>IF(AND($A73="",$B73="",$C73=""),"",IF($A73="","Missing Assignment Number",IF($B73="","Select Job Title",IF($C73="","Enter Pay Rate",IF($F73="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U73" t="str">
+        <x:v>Project Manager - IT - IV - Information Communications Technology (B Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="22" customHeight="1">
@@ -4653,7 +4875,7 @@
       <x:c r="B74" s="33"/>
       <x:c r="C74" s="59"/>
       <x:c r="D74" s="52" t="str">
-        <x:f>IF($B74="","",IF(OR(RIGHT(TRIM($B74),2)="P70",RIGHT(TRIM($B74),2)="P71",RIGHT(TRIM($B74),2)="P72",RIGHT(TRIM($B74),2)="P73"),"PS","GS"))</x:f>
+        <x:f>IF($B74="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B74),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E74" s="62" t="str">
         <x:f>IF($D74="","",IF($D74="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4699,6 +4921,9 @@
       </x:c>
       <x:c r="S74" s="54" t="str">
         <x:f>IF(AND($A74="",$B74="",$C74=""),"",IF($A74="","Missing Assignment Number",IF($B74="","Select Job Title",IF($C74="","Enter Pay Rate",IF($F74="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U74" t="str">
+        <x:v>Project Manager - IV - Engineering (P &amp; O Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="22" customHeight="1">
@@ -4706,7 +4931,7 @@
       <x:c r="B75" s="33"/>
       <x:c r="C75" s="59"/>
       <x:c r="D75" s="52" t="str">
-        <x:f>IF($B75="","",IF(OR(RIGHT(TRIM($B75),2)="P71",RIGHT(TRIM($B75),2)="P72",RIGHT(TRIM($B75),2)="P73",RIGHT(TRIM($B75),2)="P74"),"PS","GS"))</x:f>
+        <x:f>IF($B75="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B75),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E75" s="62" t="str">
         <x:f>IF($D75="","",IF($D75="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4752,6 +4977,9 @@
       </x:c>
       <x:c r="S75" s="54" t="str">
         <x:f>IF(AND($A75="",$B75="",$C75=""),"",IF($A75="","Missing Assignment Number",IF($B75="","Select Job Title",IF($C75="","Enter Pay Rate",IF($F75="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U75" t="str">
+        <x:v>Project Manager - Non IT - II - Administrative (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="22" customHeight="1">
@@ -4759,7 +4987,7 @@
       <x:c r="B76" s="33"/>
       <x:c r="C76" s="59"/>
       <x:c r="D76" s="52" t="str">
-        <x:f>IF($B76="","",IF(OR(RIGHT(TRIM($B76),2)="P72",RIGHT(TRIM($B76),2)="P73",RIGHT(TRIM($B76),2)="P74",RIGHT(TRIM($B76),2)="P75"),"PS","GS"))</x:f>
+        <x:f>IF($B76="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B76),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E76" s="62" t="str">
         <x:f>IF($D76="","",IF($D76="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4805,6 +5033,9 @@
       </x:c>
       <x:c r="S76" s="54" t="str">
         <x:f>IF(AND($A76="",$B76="",$C76=""),"",IF($A76="","Missing Assignment Number",IF($B76="","Select Job Title",IF($C76="","Enter Pay Rate",IF($F76="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U76" t="str">
+        <x:v>Project Manager - Non IT - III - Administrative (B Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="22" customHeight="1">
@@ -4812,7 +5043,7 @@
       <x:c r="B77" s="33"/>
       <x:c r="C77" s="59"/>
       <x:c r="D77" s="52" t="str">
-        <x:f>IF($B77="","",IF(OR(RIGHT(TRIM($B77),2)="P73",RIGHT(TRIM($B77),2)="P74",RIGHT(TRIM($B77),2)="P75",RIGHT(TRIM($B77),2)="P76"),"PS","GS"))</x:f>
+        <x:f>IF($B77="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B77),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E77" s="62" t="str">
         <x:f>IF($D77="","",IF($D77="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4858,6 +5089,9 @@
       </x:c>
       <x:c r="S77" s="54" t="str">
         <x:f>IF(AND($A77="",$B77="",$C77=""),"",IF($A77="","Missing Assignment Number",IF($B77="","Select Job Title",IF($C77="","Enter Pay Rate",IF($F77="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U77" t="str">
+        <x:v>Project Manager - Non IT - IV - Administrative (B Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="22" customHeight="1">
@@ -4865,7 +5099,7 @@
       <x:c r="B78" s="33"/>
       <x:c r="C78" s="59"/>
       <x:c r="D78" s="52" t="str">
-        <x:f>IF($B78="","",IF(OR(RIGHT(TRIM($B78),2)="P74",RIGHT(TRIM($B78),2)="P75",RIGHT(TRIM($B78),2)="P76",RIGHT(TRIM($B78),2)="P77"),"PS","GS"))</x:f>
+        <x:f>IF($B78="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B78),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E78" s="62" t="str">
         <x:f>IF($D78="","",IF($D78="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4911,6 +5145,9 @@
       </x:c>
       <x:c r="S78" s="54" t="str">
         <x:f>IF(AND($A78="",$B78="",$C78=""),"",IF($A78="","Missing Assignment Number",IF($B78="","Select Job Title",IF($C78="","Enter Pay Rate",IF($F78="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U78" t="str">
+        <x:v>Qualified Person - III - Administrative (B Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="22" customHeight="1">
@@ -4918,7 +5155,7 @@
       <x:c r="B79" s="33"/>
       <x:c r="C79" s="59"/>
       <x:c r="D79" s="52" t="str">
-        <x:f>IF($B79="","",IF(OR(RIGHT(TRIM($B79),2)="P75",RIGHT(TRIM($B79),2)="P76",RIGHT(TRIM($B79),2)="P77",RIGHT(TRIM($B79),2)="P78"),"PS","GS"))</x:f>
+        <x:f>IF($B79="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B79),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E79" s="62" t="str">
         <x:f>IF($D79="","",IF($D79="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -4964,6 +5201,9 @@
       </x:c>
       <x:c r="S79" s="54" t="str">
         <x:f>IF(AND($A79="",$B79="",$C79=""),"",IF($A79="","Missing Assignment Number",IF($B79="","Select Job Title",IF($C79="","Enter Pay Rate",IF($F79="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U79" t="str">
+        <x:v>Quality Assurance - Packaging - I - Industrial (P &amp; O Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="22" customHeight="1">
@@ -4971,7 +5211,7 @@
       <x:c r="B80" s="33"/>
       <x:c r="C80" s="59"/>
       <x:c r="D80" s="52" t="str">
-        <x:f>IF($B80="","",IF(OR(RIGHT(TRIM($B80),2)="P76",RIGHT(TRIM($B80),2)="P77",RIGHT(TRIM($B80),2)="P78",RIGHT(TRIM($B80),2)="P79"),"PS","GS"))</x:f>
+        <x:f>IF($B80="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B80),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E80" s="62" t="str">
         <x:f>IF($D80="","",IF($D80="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5017,6 +5257,9 @@
       </x:c>
       <x:c r="S80" s="54" t="str">
         <x:f>IF(AND($A80="",$B80="",$C80=""),"",IF($A80="","Missing Assignment Number",IF($B80="","Select Job Title",IF($C80="","Enter Pay Rate",IF($F80="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U80" t="str">
+        <x:v>Quality Assurance - Packaging - II - Industrial (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="22" customHeight="1">
@@ -5024,7 +5267,7 @@
       <x:c r="B81" s="33"/>
       <x:c r="C81" s="59"/>
       <x:c r="D81" s="52" t="str">
-        <x:f>IF($B81="","",IF(OR(RIGHT(TRIM($B81),2)="P77",RIGHT(TRIM($B81),2)="P78",RIGHT(TRIM($B81),2)="P79",RIGHT(TRIM($B81),2)="P80"),"PS","GS"))</x:f>
+        <x:f>IF($B81="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B81),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E81" s="62" t="str">
         <x:f>IF($D81="","",IF($D81="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5070,6 +5313,9 @@
       </x:c>
       <x:c r="S81" s="54" t="str">
         <x:f>IF(AND($A81="",$B81="",$C81=""),"",IF($A81="","Missing Assignment Number",IF($B81="","Select Job Title",IF($C81="","Enter Pay Rate",IF($F81="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U81" t="str">
+        <x:v>Quality Assurance - Packaging - IV - Industrial (P &amp; O Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="22" customHeight="1">
@@ -5077,7 +5323,7 @@
       <x:c r="B82" s="33"/>
       <x:c r="C82" s="59"/>
       <x:c r="D82" s="52" t="str">
-        <x:f>IF($B82="","",IF(OR(RIGHT(TRIM($B82),2)="P78",RIGHT(TRIM($B82),2)="P79",RIGHT(TRIM($B82),2)="P80",RIGHT(TRIM($B82),2)="P81"),"PS","GS"))</x:f>
+        <x:f>IF($B82="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B82),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E82" s="62" t="str">
         <x:f>IF($D82="","",IF($D82="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5123,6 +5369,9 @@
       </x:c>
       <x:c r="S82" s="54" t="str">
         <x:f>IF(AND($A82="",$B82="",$C82=""),"",IF($A82="","Missing Assignment Number",IF($B82="","Select Job Title",IF($C82="","Enter Pay Rate",IF($F82="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U82" t="str">
+        <x:v>Quality Auditor - I - Administrative (B Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="22" customHeight="1">
@@ -5130,7 +5379,7 @@
       <x:c r="B83" s="33"/>
       <x:c r="C83" s="59"/>
       <x:c r="D83" s="52" t="str">
-        <x:f>IF($B83="","",IF(OR(RIGHT(TRIM($B83),2)="P79",RIGHT(TRIM($B83),2)="P80",RIGHT(TRIM($B83),2)="P81",RIGHT(TRIM($B83),2)="P82"),"PS","GS"))</x:f>
+        <x:f>IF($B83="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B83),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E83" s="62" t="str">
         <x:f>IF($D83="","",IF($D83="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5176,6 +5425,9 @@
       </x:c>
       <x:c r="S83" s="54" t="str">
         <x:f>IF(AND($A83="",$B83="",$C83=""),"",IF($A83="","Missing Assignment Number",IF($B83="","Select Job Title",IF($C83="","Enter Pay Rate",IF($F83="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U83" t="str">
+        <x:v>Quality Auditor - II - Administrative (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="22" customHeight="1">
@@ -5183,7 +5435,7 @@
       <x:c r="B84" s="33"/>
       <x:c r="C84" s="59"/>
       <x:c r="D84" s="52" t="str">
-        <x:f>IF($B84="","",IF(OR(RIGHT(TRIM($B84),2)="P80",RIGHT(TRIM($B84),2)="P81",RIGHT(TRIM($B84),2)="P82",RIGHT(TRIM($B84),2)="P83"),"PS","GS"))</x:f>
+        <x:f>IF($B84="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B84),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E84" s="62" t="str">
         <x:f>IF($D84="","",IF($D84="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5229,6 +5481,9 @@
       </x:c>
       <x:c r="S84" s="54" t="str">
         <x:f>IF(AND($A84="",$B84="",$C84=""),"",IF($A84="","Missing Assignment Number",IF($B84="","Select Job Title",IF($C84="","Enter Pay Rate",IF($F84="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U84" t="str">
+        <x:v>Quality Auditor - III - Administrative (B Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="22" customHeight="1">
@@ -5236,7 +5491,7 @@
       <x:c r="B85" s="33"/>
       <x:c r="C85" s="59"/>
       <x:c r="D85" s="52" t="str">
-        <x:f>IF($B85="","",IF(OR(RIGHT(TRIM($B85),2)="P81",RIGHT(TRIM($B85),2)="P82",RIGHT(TRIM($B85),2)="P83",RIGHT(TRIM($B85),2)="P84"),"PS","GS"))</x:f>
+        <x:f>IF($B85="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B85),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E85" s="62" t="str">
         <x:f>IF($D85="","",IF($D85="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5282,6 +5537,9 @@
       </x:c>
       <x:c r="S85" s="54" t="str">
         <x:f>IF(AND($A85="",$B85="",$C85=""),"",IF($A85="","Missing Assignment Number",IF($B85="","Select Job Title",IF($C85="","Enter Pay Rate",IF($F85="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U85" t="str">
+        <x:v>Quality Control Specialist - II - LAB (O Support / Research) - O2 (High)</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="22" customHeight="1">
@@ -5289,7 +5547,7 @@
       <x:c r="B86" s="33"/>
       <x:c r="C86" s="59"/>
       <x:c r="D86" s="52" t="str">
-        <x:f>IF($B86="","",IF(OR(RIGHT(TRIM($B86),2)="P82",RIGHT(TRIM($B86),2)="P83",RIGHT(TRIM($B86),2)="P84",RIGHT(TRIM($B86),2)="P85"),"PS","GS"))</x:f>
+        <x:f>IF($B86="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B86),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E86" s="62" t="str">
         <x:f>IF($D86="","",IF($D86="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5335,6 +5593,9 @@
       </x:c>
       <x:c r="S86" s="54" t="str">
         <x:f>IF(AND($A86="",$B86="",$C86=""),"",IF($A86="","Missing Assignment Number",IF($B86="","Select Job Title",IF($C86="","Enter Pay Rate",IF($F86="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U86" t="str">
+        <x:v>Quality Control Specialist - II - LAB (O Support / Research) - O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="22" customHeight="1">
@@ -5342,7 +5603,7 @@
       <x:c r="B87" s="33"/>
       <x:c r="C87" s="59"/>
       <x:c r="D87" s="52" t="str">
-        <x:f>IF($B87="","",IF(OR(RIGHT(TRIM($B87),2)="P83",RIGHT(TRIM($B87),2)="P84",RIGHT(TRIM($B87),2)="P85",RIGHT(TRIM($B87),2)="P86"),"PS","GS"))</x:f>
+        <x:f>IF($B87="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B87),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E87" s="62" t="str">
         <x:f>IF($D87="","",IF($D87="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5388,6 +5649,9 @@
       </x:c>
       <x:c r="S87" s="54" t="str">
         <x:f>IF(AND($A87="",$B87="",$C87=""),"",IF($A87="","Missing Assignment Number",IF($B87="","Select Job Title",IF($C87="","Enter Pay Rate",IF($F87="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U87" t="str">
+        <x:v>Quality Control Specialist - III - LAB (O Support / Research) - O3</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="22" customHeight="1">
@@ -5395,7 +5659,7 @@
       <x:c r="B88" s="33"/>
       <x:c r="C88" s="59"/>
       <x:c r="D88" s="52" t="str">
-        <x:f>IF($B88="","",IF(OR(RIGHT(TRIM($B88),2)="P84",RIGHT(TRIM($B88),2)="P85",RIGHT(TRIM($B88),2)="P86",RIGHT(TRIM($B88),2)="P87"),"PS","GS"))</x:f>
+        <x:f>IF($B88="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B88),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E88" s="62" t="str">
         <x:f>IF($D88="","",IF($D88="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5441,6 +5705,9 @@
       </x:c>
       <x:c r="S88" s="54" t="str">
         <x:f>IF(AND($A88="",$B88="",$C88=""),"",IF($A88="","Missing Assignment Number",IF($B88="","Select Job Title",IF($C88="","Enter Pay Rate",IF($F88="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U88" t="str">
+        <x:v>Quality Engineer - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="22" customHeight="1">
@@ -5448,7 +5715,7 @@
       <x:c r="B89" s="33"/>
       <x:c r="C89" s="59"/>
       <x:c r="D89" s="52" t="str">
-        <x:f>IF($B89="","",IF(OR(RIGHT(TRIM($B89),2)="P85",RIGHT(TRIM($B89),2)="P86",RIGHT(TRIM($B89),2)="P87",RIGHT(TRIM($B89),2)="P88"),"PS","GS"))</x:f>
+        <x:f>IF($B89="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B89),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E89" s="62" t="str">
         <x:f>IF($D89="","",IF($D89="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5494,6 +5761,9 @@
       </x:c>
       <x:c r="S89" s="54" t="str">
         <x:f>IF(AND($A89="",$B89="",$C89=""),"",IF($A89="","Missing Assignment Number",IF($B89="","Select Job Title",IF($C89="","Enter Pay Rate",IF($F89="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U89" t="str">
+        <x:v>Regulatory Affairs Specialist - II - Environment Health &amp; Safety (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="22" customHeight="1">
@@ -5501,7 +5771,7 @@
       <x:c r="B90" s="33"/>
       <x:c r="C90" s="59"/>
       <x:c r="D90" s="52" t="str">
-        <x:f>IF($B90="","",IF(OR(RIGHT(TRIM($B90),2)="P86",RIGHT(TRIM($B90),2)="P87",RIGHT(TRIM($B90),2)="P88",RIGHT(TRIM($B90),2)="P89"),"PS","GS"))</x:f>
+        <x:f>IF($B90="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B90),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E90" s="62" t="str">
         <x:f>IF($D90="","",IF($D90="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5547,6 +5817,9 @@
       </x:c>
       <x:c r="S90" s="54" t="str">
         <x:f>IF(AND($A90="",$B90="",$C90=""),"",IF($A90="","Missing Assignment Number",IF($B90="","Select Job Title",IF($C90="","Enter Pay Rate",IF($F90="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U90" t="str">
+        <x:v>Regulatory Affairs Specialist III - Environment Health &amp; Safety (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="22" customHeight="1">
@@ -5554,7 +5827,7 @@
       <x:c r="B91" s="33"/>
       <x:c r="C91" s="59"/>
       <x:c r="D91" s="52" t="str">
-        <x:f>IF($B91="","",IF(OR(RIGHT(TRIM($B91),2)="P87",RIGHT(TRIM($B91),2)="P88",RIGHT(TRIM($B91),2)="P89",RIGHT(TRIM($B91),2)="P90"),"PS","GS"))</x:f>
+        <x:f>IF($B91="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B91),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E91" s="62" t="str">
         <x:f>IF($D91="","",IF($D91="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5600,6 +5873,9 @@
       </x:c>
       <x:c r="S91" s="54" t="str">
         <x:f>IF(AND($A91="",$B91="",$C91=""),"",IF($A91="","Missing Assignment Number",IF($B91="","Select Job Title",IF($C91="","Enter Pay Rate",IF($F91="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U91" t="str">
+        <x:v>Reliability Engineer - I - Engineering (P &amp; O Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="22" customHeight="1">
@@ -5607,7 +5883,7 @@
       <x:c r="B92" s="33"/>
       <x:c r="C92" s="59"/>
       <x:c r="D92" s="52" t="str">
-        <x:f>IF($B92="","",IF(OR(RIGHT(TRIM($B92),2)="P88",RIGHT(TRIM($B92),2)="P89",RIGHT(TRIM($B92),2)="P90",RIGHT(TRIM($B92),2)="P91"),"PS","GS"))</x:f>
+        <x:f>IF($B92="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B92),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E92" s="62" t="str">
         <x:f>IF($D92="","",IF($D92="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5653,6 +5929,9 @@
       </x:c>
       <x:c r="S92" s="54" t="str">
         <x:f>IF(AND($A92="",$B92="",$C92=""),"",IF($A92="","Missing Assignment Number",IF($B92="","Select Job Title",IF($C92="","Enter Pay Rate",IF($F92="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U92" t="str">
+        <x:v>Reliability Engineer - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="22" customHeight="1">
@@ -5660,7 +5939,7 @@
       <x:c r="B93" s="33"/>
       <x:c r="C93" s="59"/>
       <x:c r="D93" s="52" t="str">
-        <x:f>IF($B93="","",IF(OR(RIGHT(TRIM($B93),2)="P89",RIGHT(TRIM($B93),2)="P90",RIGHT(TRIM($B93),2)="P91",RIGHT(TRIM($B93),2)="P92"),"PS","GS"))</x:f>
+        <x:f>IF($B93="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B93),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E93" s="62" t="str">
         <x:f>IF($D93="","",IF($D93="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5706,6 +5985,9 @@
       </x:c>
       <x:c r="S93" s="54" t="str">
         <x:f>IF(AND($A93="",$B93="",$C93=""),"",IF($A93="","Missing Assignment Number",IF($B93="","Select Job Title",IF($C93="","Enter Pay Rate",IF($F93="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U93" t="str">
+        <x:v>Reliability Engineer - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="22" customHeight="1">
@@ -5713,7 +5995,7 @@
       <x:c r="B94" s="33"/>
       <x:c r="C94" s="59"/>
       <x:c r="D94" s="52" t="str">
-        <x:f>IF($B94="","",IF(OR(RIGHT(TRIM($B94),2)="P90",RIGHT(TRIM($B94),2)="P91",RIGHT(TRIM($B94),2)="P92",RIGHT(TRIM($B94),2)="P93"),"PS","GS"))</x:f>
+        <x:f>IF($B94="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B94),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E94" s="62" t="str">
         <x:f>IF($D94="","",IF($D94="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5759,6 +6041,9 @@
       </x:c>
       <x:c r="S94" s="54" t="str">
         <x:f>IF(AND($A94="",$B94="",$C94=""),"",IF($A94="","Missing Assignment Number",IF($B94="","Select Job Title",IF($C94="","Enter Pay Rate",IF($F94="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U94" t="str">
+        <x:v>Reliability Engineer - IV - Engineering (P &amp; O Support / Professional) - O4</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="22" customHeight="1">
@@ -5766,7 +6051,7 @@
       <x:c r="B95" s="33"/>
       <x:c r="C95" s="59"/>
       <x:c r="D95" s="52" t="str">
-        <x:f>IF($B95="","",IF(OR(RIGHT(TRIM($B95),2)="P91",RIGHT(TRIM($B95),2)="P92",RIGHT(TRIM($B95),2)="P93",RIGHT(TRIM($B95),2)="P94"),"PS","GS"))</x:f>
+        <x:f>IF($B95="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B95),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E95" s="62" t="str">
         <x:f>IF($D95="","",IF($D95="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5812,6 +6097,9 @@
       </x:c>
       <x:c r="S95" s="54" t="str">
         <x:f>IF(AND($A95="",$B95="",$C95=""),"",IF($A95="","Missing Assignment Number",IF($B95="","Select Job Title",IF($C95="","Enter Pay Rate",IF($F95="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U95" t="str">
+        <x:v>Sales Assistant - I - Administrative (B Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="22" customHeight="1">
@@ -5819,7 +6107,7 @@
       <x:c r="B96" s="33"/>
       <x:c r="C96" s="59"/>
       <x:c r="D96" s="52" t="str">
-        <x:f>IF($B96="","",IF(OR(RIGHT(TRIM($B96),2)="P92",RIGHT(TRIM($B96),2)="P93",RIGHT(TRIM($B96),2)="P94",RIGHT(TRIM($B96),2)="P95"),"PS","GS"))</x:f>
+        <x:f>IF($B96="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B96),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E96" s="62" t="str">
         <x:f>IF($D96="","",IF($D96="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5865,6 +6153,9 @@
       </x:c>
       <x:c r="S96" s="54" t="str">
         <x:f>IF(AND($A96="",$B96="",$C96=""),"",IF($A96="","Missing Assignment Number",IF($B96="","Select Job Title",IF($C96="","Enter Pay Rate",IF($F96="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U96" t="str">
+        <x:v>Scientific Technical Specialist - I - Engineering (P &amp; O Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="22" customHeight="1">
@@ -5872,7 +6163,7 @@
       <x:c r="B97" s="33"/>
       <x:c r="C97" s="59"/>
       <x:c r="D97" s="52" t="str">
-        <x:f>IF($B97="","",IF(OR(RIGHT(TRIM($B97),2)="P93",RIGHT(TRIM($B97),2)="P94",RIGHT(TRIM($B97),2)="P95",RIGHT(TRIM($B97),2)="P96"),"PS","GS"))</x:f>
+        <x:f>IF($B97="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B97),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E97" s="62" t="str">
         <x:f>IF($D97="","",IF($D97="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5918,6 +6209,9 @@
       </x:c>
       <x:c r="S97" s="54" t="str">
         <x:f>IF(AND($A97="",$B97="",$C97=""),"",IF($A97="","Missing Assignment Number",IF($B97="","Select Job Title",IF($C97="","Enter Pay Rate",IF($F97="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U97" t="str">
+        <x:v>Scientific Technical Specialist - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="22" customHeight="1">
@@ -5925,7 +6219,7 @@
       <x:c r="B98" s="33"/>
       <x:c r="C98" s="59"/>
       <x:c r="D98" s="52" t="str">
-        <x:f>IF($B98="","",IF(OR(RIGHT(TRIM($B98),2)="P94",RIGHT(TRIM($B98),2)="P95",RIGHT(TRIM($B98),2)="P96",RIGHT(TRIM($B98),2)="P97"),"PS","GS"))</x:f>
+        <x:f>IF($B98="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B98),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E98" s="62" t="str">
         <x:f>IF($D98="","",IF($D98="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -5971,6 +6265,9 @@
       </x:c>
       <x:c r="S98" s="54" t="str">
         <x:f>IF(AND($A98="",$B98="",$C98=""),"",IF($A98="","Missing Assignment Number",IF($B98="","Select Job Title",IF($C98="","Enter Pay Rate",IF($F98="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U98" t="str">
+        <x:v>Scientific Technical Specialist - III - Engineering (P &amp; O Support / Professional) - O3</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="22" customHeight="1">
@@ -5978,7 +6275,7 @@
       <x:c r="B99" s="33"/>
       <x:c r="C99" s="59"/>
       <x:c r="D99" s="52" t="str">
-        <x:f>IF($B99="","",IF(OR(RIGHT(TRIM($B99),2)="P95",RIGHT(TRIM($B99),2)="P96",RIGHT(TRIM($B99),2)="P97",RIGHT(TRIM($B99),2)="P98"),"PS","GS"))</x:f>
+        <x:f>IF($B99="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B99),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E99" s="62" t="str">
         <x:f>IF($D99="","",IF($D99="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6024,6 +6321,9 @@
       </x:c>
       <x:c r="S99" s="54" t="str">
         <x:f>IF(AND($A99="",$B99="",$C99=""),"",IF($A99="","Missing Assignment Number",IF($B99="","Select Job Title",IF($C99="","Enter Pay Rate",IF($F99="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U99" t="str">
+        <x:v>Scientist - I - Science (P &amp; O / Research) - R1</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="22" customHeight="1">
@@ -6031,7 +6331,7 @@
       <x:c r="B100" s="33"/>
       <x:c r="C100" s="59"/>
       <x:c r="D100" s="52" t="str">
-        <x:f>IF($B100="","",IF(OR(RIGHT(TRIM($B100),2)="P96",RIGHT(TRIM($B100),2)="P97",RIGHT(TRIM($B100),2)="P98",RIGHT(TRIM($B100),2)="P99"),"PS","GS"))</x:f>
+        <x:f>IF($B100="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B100),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E100" s="62" t="str">
         <x:f>IF($D100="","",IF($D100="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6077,6 +6377,9 @@
       </x:c>
       <x:c r="S100" s="54" t="str">
         <x:f>IF(AND($A100="",$B100="",$C100=""),"",IF($A100="","Missing Assignment Number",IF($B100="","Select Job Title",IF($C100="","Enter Pay Rate",IF($F100="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U100" t="str">
+        <x:v>Scientist - I - Science (P &amp; O / Research) - R1 - GS</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="22" customHeight="1">
@@ -6084,7 +6387,7 @@
       <x:c r="B101" s="33"/>
       <x:c r="C101" s="59"/>
       <x:c r="D101" s="52" t="str">
-        <x:f>IF($B101="","",IF(OR(RIGHT(TRIM($B101),2)="P97",RIGHT(TRIM($B101),2)="P98",RIGHT(TRIM($B101),2)="P99",RIGHT(TRIM($B101),2)="P100"),"PS","GS"))</x:f>
+        <x:f>IF($B101="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B101),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E101" s="62" t="str">
         <x:f>IF($D101="","",IF($D101="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6130,6 +6433,9 @@
       </x:c>
       <x:c r="S101" s="54" t="str">
         <x:f>IF(AND($A101="",$B101="",$C101=""),"",IF($A101="","Missing Assignment Number",IF($B101="","Select Job Title",IF($C101="","Enter Pay Rate",IF($F101="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U101" t="str">
+        <x:v>Scientist - II - Science (P &amp; O / Research) - R2</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="22" customHeight="1">
@@ -6137,7 +6443,7 @@
       <x:c r="B102" s="33"/>
       <x:c r="C102" s="59"/>
       <x:c r="D102" s="52" t="str">
-        <x:f>IF($B102="","",IF(OR(RIGHT(TRIM($B102),2)="P98",RIGHT(TRIM($B102),2)="P99",RIGHT(TRIM($B102),2)="P100",RIGHT(TRIM($B102),2)="P101"),"PS","GS"))</x:f>
+        <x:f>IF($B102="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B102),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E102" s="62" t="str">
         <x:f>IF($D102="","",IF($D102="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6183,6 +6489,9 @@
       </x:c>
       <x:c r="S102" s="54" t="str">
         <x:f>IF(AND($A102="",$B102="",$C102=""),"",IF($A102="","Missing Assignment Number",IF($B102="","Select Job Title",IF($C102="","Enter Pay Rate",IF($F102="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U102" t="str">
+        <x:v>Scientist - III - Science (P &amp; O / Research) - R3</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="22" customHeight="1">
@@ -6190,7 +6499,7 @@
       <x:c r="B103" s="33"/>
       <x:c r="C103" s="59"/>
       <x:c r="D103" s="52" t="str">
-        <x:f>IF($B103="","",IF(OR(RIGHT(TRIM($B103),2)="P99",RIGHT(TRIM($B103),2)="P100",RIGHT(TRIM($B103),2)="P101",RIGHT(TRIM($B103),2)="P102"),"PS","GS"))</x:f>
+        <x:f>IF($B103="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B103),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E103" s="62" t="str">
         <x:f>IF($D103="","",IF($D103="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6236,6 +6545,9 @@
       </x:c>
       <x:c r="S103" s="54" t="str">
         <x:f>IF(AND($A103="",$B103="",$C103=""),"",IF($A103="","Missing Assignment Number",IF($B103="","Select Job Title",IF($C103="","Enter Pay Rate",IF($F103="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U103" t="str">
+        <x:v>Shipping/Receiving Clerk - II - Production &amp; Operations Support (T): Industrial - O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="22" customHeight="1">
@@ -6243,7 +6555,7 @@
       <x:c r="B104" s="33"/>
       <x:c r="C104" s="59"/>
       <x:c r="D104" s="52" t="str">
-        <x:f>IF($B104="","",IF(OR(RIGHT(TRIM($B104),2)="P100",RIGHT(TRIM($B104),2)="P101",RIGHT(TRIM($B104),2)="P102",RIGHT(TRIM($B104),2)="P103"),"PS","GS"))</x:f>
+        <x:f>IF($B104="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B104),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E104" s="62" t="str">
         <x:f>IF($D104="","",IF($D104="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6289,6 +6601,9 @@
       </x:c>
       <x:c r="S104" s="54" t="str">
         <x:f>IF(AND($A104="",$B104="",$C104=""),"",IF($A104="","Missing Assignment Number",IF($B104="","Select Job Title",IF($C104="","Enter Pay Rate",IF($F104="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U104" t="str">
+        <x:v>Supply Chain Specialist - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="22" customHeight="1">
@@ -6296,7 +6611,7 @@
       <x:c r="B105" s="33"/>
       <x:c r="C105" s="59"/>
       <x:c r="D105" s="52" t="str">
-        <x:f>IF($B105="","",IF(OR(RIGHT(TRIM($B105),2)="P101",RIGHT(TRIM($B105),2)="P102",RIGHT(TRIM($B105),2)="P103",RIGHT(TRIM($B105),2)="P104"),"PS","GS"))</x:f>
+        <x:f>IF($B105="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B105),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E105" s="62" t="str">
         <x:f>IF($D105="","",IF($D105="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6342,6 +6657,9 @@
       </x:c>
       <x:c r="S105" s="54" t="str">
         <x:f>IF(AND($A105="",$B105="",$C105=""),"",IF($A105="","Missing Assignment Number",IF($B105="","Select Job Title",IF($C105="","Enter Pay Rate",IF($F105="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U105" t="str">
+        <x:v>Supply Chain Specialist - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="22" customHeight="1">
@@ -6349,7 +6667,7 @@
       <x:c r="B106" s="33"/>
       <x:c r="C106" s="59"/>
       <x:c r="D106" s="52" t="str">
-        <x:f>IF($B106="","",IF(OR(RIGHT(TRIM($B106),2)="P102",RIGHT(TRIM($B106),2)="P103",RIGHT(TRIM($B106),2)="P104",RIGHT(TRIM($B106),2)="P105"),"PS","GS"))</x:f>
+        <x:f>IF($B106="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B106),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E106" s="62" t="str">
         <x:f>IF($D106="","",IF($D106="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6395,6 +6713,9 @@
       </x:c>
       <x:c r="S106" s="54" t="str">
         <x:f>IF(AND($A106="",$B106="",$C106=""),"",IF($A106="","Missing Assignment Number",IF($B106="","Select Job Title",IF($C106="","Enter Pay Rate",IF($F106="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U106" t="str">
+        <x:v>Supply Chain Specialist - IV - Engineering (P &amp; O Support / Professional) - P4</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="22" customHeight="1">
@@ -6402,7 +6723,7 @@
       <x:c r="B107" s="33"/>
       <x:c r="C107" s="59"/>
       <x:c r="D107" s="52" t="str">
-        <x:f>IF($B107="","",IF(OR(RIGHT(TRIM($B107),2)="P103",RIGHT(TRIM($B107),2)="P104",RIGHT(TRIM($B107),2)="P105",RIGHT(TRIM($B107),2)="P106"),"PS","GS"))</x:f>
+        <x:f>IF($B107="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B107),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E107" s="62" t="str">
         <x:f>IF($D107="","",IF($D107="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6448,6 +6769,9 @@
       </x:c>
       <x:c r="S107" s="54" t="str">
         <x:f>IF(AND($A107="",$B107="",$C107=""),"",IF($A107="","Missing Assignment Number",IF($B107="","Select Job Title",IF($C107="","Enter Pay Rate",IF($F107="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U107" t="str">
+        <x:v>Technical Support Analyst - I - Information Communications Tech (B Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="22" customHeight="1">
@@ -6455,7 +6779,7 @@
       <x:c r="B108" s="33"/>
       <x:c r="C108" s="59"/>
       <x:c r="D108" s="52" t="str">
-        <x:f>IF($B108="","",IF(OR(RIGHT(TRIM($B108),2)="P104",RIGHT(TRIM($B108),2)="P105",RIGHT(TRIM($B108),2)="P106",RIGHT(TRIM($B108),2)="P107"),"PS","GS"))</x:f>
+        <x:f>IF($B108="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B108),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E108" s="62" t="str">
         <x:f>IF($D108="","",IF($D108="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6501,6 +6825,9 @@
       </x:c>
       <x:c r="S108" s="54" t="str">
         <x:f>IF(AND($A108="",$B108="",$C108=""),"",IF($A108="","Missing Assignment Number",IF($B108="","Select Job Title",IF($C108="","Enter Pay Rate",IF($F108="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U108" t="str">
+        <x:v>Technical Support Analyst - II - Information Communications Tech (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="22" customHeight="1">
@@ -6508,7 +6835,7 @@
       <x:c r="B109" s="33"/>
       <x:c r="C109" s="59"/>
       <x:c r="D109" s="52" t="str">
-        <x:f>IF($B109="","",IF(OR(RIGHT(TRIM($B109),2)="P105",RIGHT(TRIM($B109),2)="P106",RIGHT(TRIM($B109),2)="P107",RIGHT(TRIM($B109),2)="P108"),"PS","GS"))</x:f>
+        <x:f>IF($B109="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B109),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E109" s="62" t="str">
         <x:f>IF($D109="","",IF($D109="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6554,6 +6881,9 @@
       </x:c>
       <x:c r="S109" s="54" t="str">
         <x:f>IF(AND($A109="",$B109="",$C109=""),"",IF($A109="","Missing Assignment Number",IF($B109="","Select Job Title",IF($C109="","Enter Pay Rate",IF($F109="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U109" t="str">
+        <x:v>Technical Writer - II - Information Communications Technology (B Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="22" customHeight="1">
@@ -6561,7 +6891,7 @@
       <x:c r="B110" s="33"/>
       <x:c r="C110" s="59"/>
       <x:c r="D110" s="52" t="str">
-        <x:f>IF($B110="","",IF(OR(RIGHT(TRIM($B110),2)="P106",RIGHT(TRIM($B110),2)="P107",RIGHT(TRIM($B110),2)="P108",RIGHT(TRIM($B110),2)="P109"),"PS","GS"))</x:f>
+        <x:f>IF($B110="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B110),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E110" s="62" t="str">
         <x:f>IF($D110="","",IF($D110="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6607,6 +6937,9 @@
       </x:c>
       <x:c r="S110" s="54" t="str">
         <x:f>IF(AND($A110="",$B110="",$C110=""),"",IF($A110="","Missing Assignment Number",IF($B110="","Select Job Title",IF($C110="","Enter Pay Rate",IF($F110="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U110" t="str">
+        <x:v>Validation Engineer - I - Engineering (P &amp; O Support / Professional) - P1</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="22" customHeight="1">
@@ -6614,7 +6947,7 @@
       <x:c r="B111" s="33"/>
       <x:c r="C111" s="59"/>
       <x:c r="D111" s="52" t="str">
-        <x:f>IF($B111="","",IF(OR(RIGHT(TRIM($B111),2)="P107",RIGHT(TRIM($B111),2)="P108",RIGHT(TRIM($B111),2)="P109",RIGHT(TRIM($B111),2)="P110"),"PS","GS"))</x:f>
+        <x:f>IF($B111="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B111),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E111" s="62" t="str">
         <x:f>IF($D111="","",IF($D111="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6660,6 +6993,9 @@
       </x:c>
       <x:c r="S111" s="54" t="str">
         <x:f>IF(AND($A111="",$B111="",$C111=""),"",IF($A111="","Missing Assignment Number",IF($B111="","Select Job Title",IF($C111="","Enter Pay Rate",IF($F111="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U111" t="str">
+        <x:v>Validation Engineer - II - Engineering (P &amp; O Support / Professional) - P2</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="22" customHeight="1">
@@ -6667,7 +7003,7 @@
       <x:c r="B112" s="33"/>
       <x:c r="C112" s="59"/>
       <x:c r="D112" s="52" t="str">
-        <x:f>IF($B112="","",IF(OR(RIGHT(TRIM($B112),2)="P108",RIGHT(TRIM($B112),2)="P109",RIGHT(TRIM($B112),2)="P110",RIGHT(TRIM($B112),2)="P111"),"PS","GS"))</x:f>
+        <x:f>IF($B112="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B112),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E112" s="62" t="str">
         <x:f>IF($D112="","",IF($D112="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6713,6 +7049,9 @@
       </x:c>
       <x:c r="S112" s="54" t="str">
         <x:f>IF(AND($A112="",$B112="",$C112=""),"",IF($A112="","Missing Assignment Number",IF($B112="","Select Job Title",IF($C112="","Enter Pay Rate",IF($F112="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U112" t="str">
+        <x:v>Validation Engineer - III - Engineering (P &amp; O Support / Professional) - P3</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="22" customHeight="1">
@@ -6720,7 +7059,7 @@
       <x:c r="B113" s="33"/>
       <x:c r="C113" s="59"/>
       <x:c r="D113" s="52" t="str">
-        <x:f>IF($B113="","",IF(OR(RIGHT(TRIM($B113),2)="P109",RIGHT(TRIM($B113),2)="P110",RIGHT(TRIM($B113),2)="P111",RIGHT(TRIM($B113),2)="P112"),"PS","GS"))</x:f>
+        <x:f>IF($B113="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B113),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E113" s="62" t="str">
         <x:f>IF($D113="","",IF($D113="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6766,6 +7105,9 @@
       </x:c>
       <x:c r="S113" s="54" t="str">
         <x:f>IF(AND($A113="",$B113="",$C113=""),"",IF($A113="","Missing Assignment Number",IF($B113="","Select Job Title",IF($C113="","Enter Pay Rate",IF($F113="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U113" t="str">
+        <x:v>Warehouse Clerk - II - Production &amp; Operations Support (T): Industrial - O2 (Mid)</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="22" customHeight="1">
@@ -6773,7 +7115,7 @@
       <x:c r="B114" s="33"/>
       <x:c r="C114" s="59"/>
       <x:c r="D114" s="52" t="str">
-        <x:f>IF($B114="","",IF(OR(RIGHT(TRIM($B114),2)="P110",RIGHT(TRIM($B114),2)="P111",RIGHT(TRIM($B114),2)="P112",RIGHT(TRIM($B114),2)="P113"),"PS","GS"))</x:f>
+        <x:f>IF($B114="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B114),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E114" s="62" t="str">
         <x:f>IF($D114="","",IF($D114="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6826,7 +7168,7 @@
       <x:c r="B115" s="33"/>
       <x:c r="C115" s="59"/>
       <x:c r="D115" s="52" t="str">
-        <x:f>IF($B115="","",IF(OR(RIGHT(TRIM($B115),2)="P111",RIGHT(TRIM($B115),2)="P112",RIGHT(TRIM($B115),2)="P113",RIGHT(TRIM($B115),2)="P114"),"PS","GS"))</x:f>
+        <x:f>IF($B115="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B115),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E115" s="62" t="str">
         <x:f>IF($D115="","",IF($D115="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6879,7 +7221,7 @@
       <x:c r="B116" s="33"/>
       <x:c r="C116" s="59"/>
       <x:c r="D116" s="52" t="str">
-        <x:f>IF($B116="","",IF(OR(RIGHT(TRIM($B116),2)="P112",RIGHT(TRIM($B116),2)="P113",RIGHT(TRIM($B116),2)="P114",RIGHT(TRIM($B116),2)="P115"),"PS","GS"))</x:f>
+        <x:f>IF($B116="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B116),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E116" s="62" t="str">
         <x:f>IF($D116="","",IF($D116="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6932,7 +7274,7 @@
       <x:c r="B117" s="33"/>
       <x:c r="C117" s="59"/>
       <x:c r="D117" s="52" t="str">
-        <x:f>IF($B117="","",IF(OR(RIGHT(TRIM($B117),2)="P113",RIGHT(TRIM($B117),2)="P114",RIGHT(TRIM($B117),2)="P115",RIGHT(TRIM($B117),2)="P116"),"PS","GS"))</x:f>
+        <x:f>IF($B117="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B117),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E117" s="62" t="str">
         <x:f>IF($D117="","",IF($D117="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -6985,7 +7327,7 @@
       <x:c r="B118" s="33"/>
       <x:c r="C118" s="59"/>
       <x:c r="D118" s="52" t="str">
-        <x:f>IF($B118="","",IF(OR(RIGHT(TRIM($B118),2)="P114",RIGHT(TRIM($B118),2)="P115",RIGHT(TRIM($B118),2)="P116",RIGHT(TRIM($B118),2)="P117"),"PS","GS"))</x:f>
+        <x:f>IF($B118="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B118),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E118" s="62" t="str">
         <x:f>IF($D118="","",IF($D118="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7038,7 +7380,7 @@
       <x:c r="B119" s="33"/>
       <x:c r="C119" s="59"/>
       <x:c r="D119" s="52" t="str">
-        <x:f>IF($B119="","",IF(OR(RIGHT(TRIM($B119),2)="P115",RIGHT(TRIM($B119),2)="P116",RIGHT(TRIM($B119),2)="P117",RIGHT(TRIM($B119),2)="P118"),"PS","GS"))</x:f>
+        <x:f>IF($B119="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B119),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E119" s="62" t="str">
         <x:f>IF($D119="","",IF($D119="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7091,7 +7433,7 @@
       <x:c r="B120" s="33"/>
       <x:c r="C120" s="59"/>
       <x:c r="D120" s="52" t="str">
-        <x:f>IF($B120="","",IF(OR(RIGHT(TRIM($B120),2)="P116",RIGHT(TRIM($B120),2)="P117",RIGHT(TRIM($B120),2)="P118",RIGHT(TRIM($B120),2)="P119"),"PS","GS"))</x:f>
+        <x:f>IF($B120="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B120),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E120" s="62" t="str">
         <x:f>IF($D120="","",IF($D120="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7144,7 +7486,7 @@
       <x:c r="B121" s="33"/>
       <x:c r="C121" s="59"/>
       <x:c r="D121" s="52" t="str">
-        <x:f>IF($B121="","",IF(OR(RIGHT(TRIM($B121),2)="P117",RIGHT(TRIM($B121),2)="P118",RIGHT(TRIM($B121),2)="P119",RIGHT(TRIM($B121),2)="P120"),"PS","GS"))</x:f>
+        <x:f>IF($B121="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B121),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E121" s="62" t="str">
         <x:f>IF($D121="","",IF($D121="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7197,7 +7539,7 @@
       <x:c r="B122" s="33"/>
       <x:c r="C122" s="59"/>
       <x:c r="D122" s="52" t="str">
-        <x:f>IF($B122="","",IF(OR(RIGHT(TRIM($B122),2)="P118",RIGHT(TRIM($B122),2)="P119",RIGHT(TRIM($B122),2)="P120",RIGHT(TRIM($B122),2)="P121"),"PS","GS"))</x:f>
+        <x:f>IF($B122="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B122),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E122" s="62" t="str">
         <x:f>IF($D122="","",IF($D122="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7250,7 +7592,7 @@
       <x:c r="B123" s="33"/>
       <x:c r="C123" s="59"/>
       <x:c r="D123" s="52" t="str">
-        <x:f>IF($B123="","",IF(OR(RIGHT(TRIM($B123),2)="P119",RIGHT(TRIM($B123),2)="P120",RIGHT(TRIM($B123),2)="P121",RIGHT(TRIM($B123),2)="P122"),"PS","GS"))</x:f>
+        <x:f>IF($B123="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B123),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E123" s="62" t="str">
         <x:f>IF($D123="","",IF($D123="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7303,7 +7645,7 @@
       <x:c r="B124" s="33"/>
       <x:c r="C124" s="59"/>
       <x:c r="D124" s="52" t="str">
-        <x:f>IF($B124="","",IF(OR(RIGHT(TRIM($B124),2)="P120",RIGHT(TRIM($B124),2)="P121",RIGHT(TRIM($B124),2)="P122",RIGHT(TRIM($B124),2)="P123"),"PS","GS"))</x:f>
+        <x:f>IF($B124="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B124),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E124" s="62" t="str">
         <x:f>IF($D124="","",IF($D124="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7356,7 +7698,7 @@
       <x:c r="B125" s="33"/>
       <x:c r="C125" s="59"/>
       <x:c r="D125" s="52" t="str">
-        <x:f>IF($B125="","",IF(OR(RIGHT(TRIM($B125),2)="P121",RIGHT(TRIM($B125),2)="P122",RIGHT(TRIM($B125),2)="P123",RIGHT(TRIM($B125),2)="P124"),"PS","GS"))</x:f>
+        <x:f>IF($B125="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B125),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E125" s="62" t="str">
         <x:f>IF($D125="","",IF($D125="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7409,7 +7751,7 @@
       <x:c r="B126" s="33"/>
       <x:c r="C126" s="59"/>
       <x:c r="D126" s="52" t="str">
-        <x:f>IF($B126="","",IF(OR(RIGHT(TRIM($B126),2)="P122",RIGHT(TRIM($B126),2)="P123",RIGHT(TRIM($B126),2)="P124",RIGHT(TRIM($B126),2)="P125"),"PS","GS"))</x:f>
+        <x:f>IF($B126="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B126),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E126" s="62" t="str">
         <x:f>IF($D126="","",IF($D126="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7462,7 +7804,7 @@
       <x:c r="B127" s="33"/>
       <x:c r="C127" s="59"/>
       <x:c r="D127" s="52" t="str">
-        <x:f>IF($B127="","",IF(OR(RIGHT(TRIM($B127),2)="P123",RIGHT(TRIM($B127),2)="P124",RIGHT(TRIM($B127),2)="P125",RIGHT(TRIM($B127),2)="P126"),"PS","GS"))</x:f>
+        <x:f>IF($B127="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B127),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E127" s="62" t="str">
         <x:f>IF($D127="","",IF($D127="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7515,7 +7857,7 @@
       <x:c r="B128" s="33"/>
       <x:c r="C128" s="59"/>
       <x:c r="D128" s="52" t="str">
-        <x:f>IF($B128="","",IF(OR(RIGHT(TRIM($B128),2)="P124",RIGHT(TRIM($B128),2)="P125",RIGHT(TRIM($B128),2)="P126",RIGHT(TRIM($B128),2)="P127"),"PS","GS"))</x:f>
+        <x:f>IF($B128="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B128),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E128" s="62" t="str">
         <x:f>IF($D128="","",IF($D128="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7568,7 +7910,7 @@
       <x:c r="B129" s="33"/>
       <x:c r="C129" s="59"/>
       <x:c r="D129" s="52" t="str">
-        <x:f>IF($B129="","",IF(OR(RIGHT(TRIM($B129),2)="P125",RIGHT(TRIM($B129),2)="P126",RIGHT(TRIM($B129),2)="P127",RIGHT(TRIM($B129),2)="P128"),"PS","GS"))</x:f>
+        <x:f>IF($B129="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B129),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E129" s="62" t="str">
         <x:f>IF($D129="","",IF($D129="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7621,7 +7963,7 @@
       <x:c r="B130" s="33"/>
       <x:c r="C130" s="59"/>
       <x:c r="D130" s="52" t="str">
-        <x:f>IF($B130="","",IF(OR(RIGHT(TRIM($B130),2)="P126",RIGHT(TRIM($B130),2)="P127",RIGHT(TRIM($B130),2)="P128",RIGHT(TRIM($B130),2)="P129"),"PS","GS"))</x:f>
+        <x:f>IF($B130="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B130),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E130" s="62" t="str">
         <x:f>IF($D130="","",IF($D130="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7674,7 +8016,7 @@
       <x:c r="B131" s="33"/>
       <x:c r="C131" s="59"/>
       <x:c r="D131" s="52" t="str">
-        <x:f>IF($B131="","",IF(OR(RIGHT(TRIM($B131),2)="P127",RIGHT(TRIM($B131),2)="P128",RIGHT(TRIM($B131),2)="P129",RIGHT(TRIM($B131),2)="P130"),"PS","GS"))</x:f>
+        <x:f>IF($B131="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B131),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E131" s="62" t="str">
         <x:f>IF($D131="","",IF($D131="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7727,7 +8069,7 @@
       <x:c r="B132" s="33"/>
       <x:c r="C132" s="59"/>
       <x:c r="D132" s="52" t="str">
-        <x:f>IF($B132="","",IF(OR(RIGHT(TRIM($B132),2)="P128",RIGHT(TRIM($B132),2)="P129",RIGHT(TRIM($B132),2)="P130",RIGHT(TRIM($B132),2)="P131"),"PS","GS"))</x:f>
+        <x:f>IF($B132="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B132),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E132" s="62" t="str">
         <x:f>IF($D132="","",IF($D132="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7780,7 +8122,7 @@
       <x:c r="B133" s="33"/>
       <x:c r="C133" s="59"/>
       <x:c r="D133" s="52" t="str">
-        <x:f>IF($B133="","",IF(OR(RIGHT(TRIM($B133),2)="P129",RIGHT(TRIM($B133),2)="P130",RIGHT(TRIM($B133),2)="P131",RIGHT(TRIM($B133),2)="P132"),"PS","GS"))</x:f>
+        <x:f>IF($B133="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B133),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E133" s="62" t="str">
         <x:f>IF($D133="","",IF($D133="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7833,7 +8175,7 @@
       <x:c r="B134" s="33"/>
       <x:c r="C134" s="59"/>
       <x:c r="D134" s="52" t="str">
-        <x:f>IF($B134="","",IF(OR(RIGHT(TRIM($B134),2)="P130",RIGHT(TRIM($B134),2)="P131",RIGHT(TRIM($B134),2)="P132",RIGHT(TRIM($B134),2)="P133"),"PS","GS"))</x:f>
+        <x:f>IF($B134="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B134),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E134" s="62" t="str">
         <x:f>IF($D134="","",IF($D134="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7886,7 +8228,7 @@
       <x:c r="B135" s="33"/>
       <x:c r="C135" s="59"/>
       <x:c r="D135" s="52" t="str">
-        <x:f>IF($B135="","",IF(OR(RIGHT(TRIM($B135),2)="P131",RIGHT(TRIM($B135),2)="P132",RIGHT(TRIM($B135),2)="P133",RIGHT(TRIM($B135),2)="P134"),"PS","GS"))</x:f>
+        <x:f>IF($B135="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B135),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E135" s="62" t="str">
         <x:f>IF($D135="","",IF($D135="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7939,7 +8281,7 @@
       <x:c r="B136" s="33"/>
       <x:c r="C136" s="59"/>
       <x:c r="D136" s="52" t="str">
-        <x:f>IF($B136="","",IF(OR(RIGHT(TRIM($B136),2)="P132",RIGHT(TRIM($B136),2)="P133",RIGHT(TRIM($B136),2)="P134",RIGHT(TRIM($B136),2)="P135"),"PS","GS"))</x:f>
+        <x:f>IF($B136="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B136),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E136" s="62" t="str">
         <x:f>IF($D136="","",IF($D136="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -7992,7 +8334,7 @@
       <x:c r="B137" s="33"/>
       <x:c r="C137" s="59"/>
       <x:c r="D137" s="52" t="str">
-        <x:f>IF($B137="","",IF(OR(RIGHT(TRIM($B137),2)="P133",RIGHT(TRIM($B137),2)="P134",RIGHT(TRIM($B137),2)="P135",RIGHT(TRIM($B137),2)="P136"),"PS","GS"))</x:f>
+        <x:f>IF($B137="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B137),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E137" s="62" t="str">
         <x:f>IF($D137="","",IF($D137="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8045,7 +8387,7 @@
       <x:c r="B138" s="33"/>
       <x:c r="C138" s="59"/>
       <x:c r="D138" s="52" t="str">
-        <x:f>IF($B138="","",IF(OR(RIGHT(TRIM($B138),2)="P134",RIGHT(TRIM($B138),2)="P135",RIGHT(TRIM($B138),2)="P136",RIGHT(TRIM($B138),2)="P137"),"PS","GS"))</x:f>
+        <x:f>IF($B138="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B138),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E138" s="62" t="str">
         <x:f>IF($D138="","",IF($D138="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8098,7 +8440,7 @@
       <x:c r="B139" s="33"/>
       <x:c r="C139" s="59"/>
       <x:c r="D139" s="52" t="str">
-        <x:f>IF($B139="","",IF(OR(RIGHT(TRIM($B139),2)="P135",RIGHT(TRIM($B139),2)="P136",RIGHT(TRIM($B139),2)="P137",RIGHT(TRIM($B139),2)="P138"),"PS","GS"))</x:f>
+        <x:f>IF($B139="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B139),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E139" s="62" t="str">
         <x:f>IF($D139="","",IF($D139="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8151,7 +8493,7 @@
       <x:c r="B140" s="33"/>
       <x:c r="C140" s="59"/>
       <x:c r="D140" s="52" t="str">
-        <x:f>IF($B140="","",IF(OR(RIGHT(TRIM($B140),2)="P136",RIGHT(TRIM($B140),2)="P137",RIGHT(TRIM($B140),2)="P138",RIGHT(TRIM($B140),2)="P139"),"PS","GS"))</x:f>
+        <x:f>IF($B140="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B140),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E140" s="62" t="str">
         <x:f>IF($D140="","",IF($D140="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8204,7 +8546,7 @@
       <x:c r="B141" s="33"/>
       <x:c r="C141" s="59"/>
       <x:c r="D141" s="52" t="str">
-        <x:f>IF($B141="","",IF(OR(RIGHT(TRIM($B141),2)="P137",RIGHT(TRIM($B141),2)="P138",RIGHT(TRIM($B141),2)="P139",RIGHT(TRIM($B141),2)="P140"),"PS","GS"))</x:f>
+        <x:f>IF($B141="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B141),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E141" s="62" t="str">
         <x:f>IF($D141="","",IF($D141="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8257,7 +8599,7 @@
       <x:c r="B142" s="33"/>
       <x:c r="C142" s="59"/>
       <x:c r="D142" s="52" t="str">
-        <x:f>IF($B142="","",IF(OR(RIGHT(TRIM($B142),2)="P138",RIGHT(TRIM($B142),2)="P139",RIGHT(TRIM($B142),2)="P140",RIGHT(TRIM($B142),2)="P141"),"PS","GS"))</x:f>
+        <x:f>IF($B142="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B142),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E142" s="62" t="str">
         <x:f>IF($D142="","",IF($D142="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8310,7 +8652,7 @@
       <x:c r="B143" s="33"/>
       <x:c r="C143" s="59"/>
       <x:c r="D143" s="52" t="str">
-        <x:f>IF($B143="","",IF(OR(RIGHT(TRIM($B143),2)="P139",RIGHT(TRIM($B143),2)="P140",RIGHT(TRIM($B143),2)="P141",RIGHT(TRIM($B143),2)="P142"),"PS","GS"))</x:f>
+        <x:f>IF($B143="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B143),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E143" s="62" t="str">
         <x:f>IF($D143="","",IF($D143="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8363,7 +8705,7 @@
       <x:c r="B144" s="33"/>
       <x:c r="C144" s="59"/>
       <x:c r="D144" s="52" t="str">
-        <x:f>IF($B144="","",IF(OR(RIGHT(TRIM($B144),2)="P140",RIGHT(TRIM($B144),2)="P141",RIGHT(TRIM($B144),2)="P142",RIGHT(TRIM($B144),2)="P143"),"PS","GS"))</x:f>
+        <x:f>IF($B144="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B144),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E144" s="62" t="str">
         <x:f>IF($D144="","",IF($D144="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8416,7 +8758,7 @@
       <x:c r="B145" s="33"/>
       <x:c r="C145" s="59"/>
       <x:c r="D145" s="52" t="str">
-        <x:f>IF($B145="","",IF(OR(RIGHT(TRIM($B145),2)="P141",RIGHT(TRIM($B145),2)="P142",RIGHT(TRIM($B145),2)="P143",RIGHT(TRIM($B145),2)="P144"),"PS","GS"))</x:f>
+        <x:f>IF($B145="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B145),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E145" s="62" t="str">
         <x:f>IF($D145="","",IF($D145="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8469,7 +8811,7 @@
       <x:c r="B146" s="33"/>
       <x:c r="C146" s="59"/>
       <x:c r="D146" s="52" t="str">
-        <x:f>IF($B146="","",IF(OR(RIGHT(TRIM($B146),2)="P142",RIGHT(TRIM($B146),2)="P143",RIGHT(TRIM($B146),2)="P144",RIGHT(TRIM($B146),2)="P145"),"PS","GS"))</x:f>
+        <x:f>IF($B146="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B146),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E146" s="62" t="str">
         <x:f>IF($D146="","",IF($D146="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8522,7 +8864,7 @@
       <x:c r="B147" s="33"/>
       <x:c r="C147" s="59"/>
       <x:c r="D147" s="52" t="str">
-        <x:f>IF($B147="","",IF(OR(RIGHT(TRIM($B147),2)="P143",RIGHT(TRIM($B147),2)="P144",RIGHT(TRIM($B147),2)="P145",RIGHT(TRIM($B147),2)="P146"),"PS","GS"))</x:f>
+        <x:f>IF($B147="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B147),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E147" s="62" t="str">
         <x:f>IF($D147="","",IF($D147="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8575,7 +8917,7 @@
       <x:c r="B148" s="33"/>
       <x:c r="C148" s="59"/>
       <x:c r="D148" s="52" t="str">
-        <x:f>IF($B148="","",IF(OR(RIGHT(TRIM($B148),2)="P144",RIGHT(TRIM($B148),2)="P145",RIGHT(TRIM($B148),2)="P146",RIGHT(TRIM($B148),2)="P147"),"PS","GS"))</x:f>
+        <x:f>IF($B148="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B148),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E148" s="62" t="str">
         <x:f>IF($D148="","",IF($D148="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8628,7 +8970,7 @@
       <x:c r="B149" s="33"/>
       <x:c r="C149" s="59"/>
       <x:c r="D149" s="52" t="str">
-        <x:f>IF($B149="","",IF(OR(RIGHT(TRIM($B149),2)="P145",RIGHT(TRIM($B149),2)="P146",RIGHT(TRIM($B149),2)="P147",RIGHT(TRIM($B149),2)="P148"),"PS","GS"))</x:f>
+        <x:f>IF($B149="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B149),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E149" s="62" t="str">
         <x:f>IF($D149="","",IF($D149="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8681,7 +9023,7 @@
       <x:c r="B150" s="33"/>
       <x:c r="C150" s="59"/>
       <x:c r="D150" s="52" t="str">
-        <x:f>IF($B150="","",IF(OR(RIGHT(TRIM($B150),2)="P146",RIGHT(TRIM($B150),2)="P147",RIGHT(TRIM($B150),2)="P148",RIGHT(TRIM($B150),2)="P149"),"PS","GS"))</x:f>
+        <x:f>IF($B150="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B150),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E150" s="62" t="str">
         <x:f>IF($D150="","",IF($D150="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8734,7 +9076,7 @@
       <x:c r="B151" s="33"/>
       <x:c r="C151" s="59"/>
       <x:c r="D151" s="52" t="str">
-        <x:f>IF($B151="","",IF(OR(RIGHT(TRIM($B151),2)="P147",RIGHT(TRIM($B151),2)="P148",RIGHT(TRIM($B151),2)="P149",RIGHT(TRIM($B151),2)="P150"),"PS","GS"))</x:f>
+        <x:f>IF($B151="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B151),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E151" s="62" t="str">
         <x:f>IF($D151="","",IF($D151="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8787,7 +9129,7 @@
       <x:c r="B152" s="33"/>
       <x:c r="C152" s="59"/>
       <x:c r="D152" s="52" t="str">
-        <x:f>IF($B152="","",IF(OR(RIGHT(TRIM($B152),2)="P148",RIGHT(TRIM($B152),2)="P149",RIGHT(TRIM($B152),2)="P150",RIGHT(TRIM($B152),2)="P151"),"PS","GS"))</x:f>
+        <x:f>IF($B152="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B152),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E152" s="62" t="str">
         <x:f>IF($D152="","",IF($D152="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8840,7 +9182,7 @@
       <x:c r="B153" s="33"/>
       <x:c r="C153" s="59"/>
       <x:c r="D153" s="52" t="str">
-        <x:f>IF($B153="","",IF(OR(RIGHT(TRIM($B153),2)="P149",RIGHT(TRIM($B153),2)="P150",RIGHT(TRIM($B153),2)="P151",RIGHT(TRIM($B153),2)="P152"),"PS","GS"))</x:f>
+        <x:f>IF($B153="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B153),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E153" s="62" t="str">
         <x:f>IF($D153="","",IF($D153="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8893,7 +9235,7 @@
       <x:c r="B154" s="33"/>
       <x:c r="C154" s="59"/>
       <x:c r="D154" s="52" t="str">
-        <x:f>IF($B154="","",IF(OR(RIGHT(TRIM($B154),2)="P150",RIGHT(TRIM($B154),2)="P151",RIGHT(TRIM($B154),2)="P152",RIGHT(TRIM($B154),2)="P153"),"PS","GS"))</x:f>
+        <x:f>IF($B154="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B154),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E154" s="62" t="str">
         <x:f>IF($D154="","",IF($D154="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8946,7 +9288,7 @@
       <x:c r="B155" s="33"/>
       <x:c r="C155" s="59"/>
       <x:c r="D155" s="52" t="str">
-        <x:f>IF($B155="","",IF(OR(RIGHT(TRIM($B155),2)="P151",RIGHT(TRIM($B155),2)="P152",RIGHT(TRIM($B155),2)="P153",RIGHT(TRIM($B155),2)="P154"),"PS","GS"))</x:f>
+        <x:f>IF($B155="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B155),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E155" s="62" t="str">
         <x:f>IF($D155="","",IF($D155="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -8999,7 +9341,7 @@
       <x:c r="B156" s="33"/>
       <x:c r="C156" s="59"/>
       <x:c r="D156" s="52" t="str">
-        <x:f>IF($B156="","",IF(OR(RIGHT(TRIM($B156),2)="P152",RIGHT(TRIM($B156),2)="P153",RIGHT(TRIM($B156),2)="P154",RIGHT(TRIM($B156),2)="P155"),"PS","GS"))</x:f>
+        <x:f>IF($B156="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B156),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E156" s="62" t="str">
         <x:f>IF($D156="","",IF($D156="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9052,7 +9394,7 @@
       <x:c r="B157" s="33"/>
       <x:c r="C157" s="59"/>
       <x:c r="D157" s="52" t="str">
-        <x:f>IF($B157="","",IF(OR(RIGHT(TRIM($B157),2)="P153",RIGHT(TRIM($B157),2)="P154",RIGHT(TRIM($B157),2)="P155",RIGHT(TRIM($B157),2)="P156"),"PS","GS"))</x:f>
+        <x:f>IF($B157="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B157),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E157" s="62" t="str">
         <x:f>IF($D157="","",IF($D157="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9105,7 +9447,7 @@
       <x:c r="B158" s="33"/>
       <x:c r="C158" s="59"/>
       <x:c r="D158" s="52" t="str">
-        <x:f>IF($B158="","",IF(OR(RIGHT(TRIM($B158),2)="P154",RIGHT(TRIM($B158),2)="P155",RIGHT(TRIM($B158),2)="P156",RIGHT(TRIM($B158),2)="P157"),"PS","GS"))</x:f>
+        <x:f>IF($B158="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B158),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E158" s="62" t="str">
         <x:f>IF($D158="","",IF($D158="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9158,7 +9500,7 @@
       <x:c r="B159" s="33"/>
       <x:c r="C159" s="59"/>
       <x:c r="D159" s="52" t="str">
-        <x:f>IF($B159="","",IF(OR(RIGHT(TRIM($B159),2)="P155",RIGHT(TRIM($B159),2)="P156",RIGHT(TRIM($B159),2)="P157",RIGHT(TRIM($B159),2)="P158"),"PS","GS"))</x:f>
+        <x:f>IF($B159="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B159),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E159" s="62" t="str">
         <x:f>IF($D159="","",IF($D159="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9211,7 +9553,7 @@
       <x:c r="B160" s="33"/>
       <x:c r="C160" s="59"/>
       <x:c r="D160" s="52" t="str">
-        <x:f>IF($B160="","",IF(OR(RIGHT(TRIM($B160),2)="P156",RIGHT(TRIM($B160),2)="P157",RIGHT(TRIM($B160),2)="P158",RIGHT(TRIM($B160),2)="P159"),"PS","GS"))</x:f>
+        <x:f>IF($B160="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B160),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E160" s="62" t="str">
         <x:f>IF($D160="","",IF($D160="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9264,7 +9606,7 @@
       <x:c r="B161" s="33"/>
       <x:c r="C161" s="59"/>
       <x:c r="D161" s="52" t="str">
-        <x:f>IF($B161="","",IF(OR(RIGHT(TRIM($B161),2)="P157",RIGHT(TRIM($B161),2)="P158",RIGHT(TRIM($B161),2)="P159",RIGHT(TRIM($B161),2)="P160"),"PS","GS"))</x:f>
+        <x:f>IF($B161="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B161),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E161" s="62" t="str">
         <x:f>IF($D161="","",IF($D161="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9317,7 +9659,7 @@
       <x:c r="B162" s="33"/>
       <x:c r="C162" s="59"/>
       <x:c r="D162" s="52" t="str">
-        <x:f>IF($B162="","",IF(OR(RIGHT(TRIM($B162),2)="P158",RIGHT(TRIM($B162),2)="P159",RIGHT(TRIM($B162),2)="P160",RIGHT(TRIM($B162),2)="P161"),"PS","GS"))</x:f>
+        <x:f>IF($B162="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B162),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E162" s="62" t="str">
         <x:f>IF($D162="","",IF($D162="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9370,7 +9712,7 @@
       <x:c r="B163" s="33"/>
       <x:c r="C163" s="59"/>
       <x:c r="D163" s="52" t="str">
-        <x:f>IF($B163="","",IF(OR(RIGHT(TRIM($B163),2)="P159",RIGHT(TRIM($B163),2)="P160",RIGHT(TRIM($B163),2)="P161",RIGHT(TRIM($B163),2)="P162"),"PS","GS"))</x:f>
+        <x:f>IF($B163="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B163),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E163" s="62" t="str">
         <x:f>IF($D163="","",IF($D163="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9423,7 +9765,7 @@
       <x:c r="B164" s="33"/>
       <x:c r="C164" s="59"/>
       <x:c r="D164" s="52" t="str">
-        <x:f>IF($B164="","",IF(OR(RIGHT(TRIM($B164),2)="P160",RIGHT(TRIM($B164),2)="P161",RIGHT(TRIM($B164),2)="P162",RIGHT(TRIM($B164),2)="P163"),"PS","GS"))</x:f>
+        <x:f>IF($B164="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B164),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E164" s="62" t="str">
         <x:f>IF($D164="","",IF($D164="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9476,7 +9818,7 @@
       <x:c r="B165" s="33"/>
       <x:c r="C165" s="59"/>
       <x:c r="D165" s="52" t="str">
-        <x:f>IF($B165="","",IF(OR(RIGHT(TRIM($B165),2)="P161",RIGHT(TRIM($B165),2)="P162",RIGHT(TRIM($B165),2)="P163",RIGHT(TRIM($B165),2)="P164"),"PS","GS"))</x:f>
+        <x:f>IF($B165="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B165),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E165" s="62" t="str">
         <x:f>IF($D165="","",IF($D165="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9529,7 +9871,7 @@
       <x:c r="B166" s="33"/>
       <x:c r="C166" s="59"/>
       <x:c r="D166" s="52" t="str">
-        <x:f>IF($B166="","",IF(OR(RIGHT(TRIM($B166),2)="P162",RIGHT(TRIM($B166),2)="P163",RIGHT(TRIM($B166),2)="P164",RIGHT(TRIM($B166),2)="P165"),"PS","GS"))</x:f>
+        <x:f>IF($B166="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B166),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E166" s="62" t="str">
         <x:f>IF($D166="","",IF($D166="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9582,7 +9924,7 @@
       <x:c r="B167" s="33"/>
       <x:c r="C167" s="59"/>
       <x:c r="D167" s="52" t="str">
-        <x:f>IF($B167="","",IF(OR(RIGHT(TRIM($B167),2)="P163",RIGHT(TRIM($B167),2)="P164",RIGHT(TRIM($B167),2)="P165",RIGHT(TRIM($B167),2)="P166"),"PS","GS"))</x:f>
+        <x:f>IF($B167="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B167),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E167" s="62" t="str">
         <x:f>IF($D167="","",IF($D167="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9635,7 +9977,7 @@
       <x:c r="B168" s="33"/>
       <x:c r="C168" s="59"/>
       <x:c r="D168" s="52" t="str">
-        <x:f>IF($B168="","",IF(OR(RIGHT(TRIM($B168),2)="P164",RIGHT(TRIM($B168),2)="P165",RIGHT(TRIM($B168),2)="P166",RIGHT(TRIM($B168),2)="P167"),"PS","GS"))</x:f>
+        <x:f>IF($B168="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B168),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E168" s="62" t="str">
         <x:f>IF($D168="","",IF($D168="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9688,7 +10030,7 @@
       <x:c r="B169" s="33"/>
       <x:c r="C169" s="59"/>
       <x:c r="D169" s="52" t="str">
-        <x:f>IF($B169="","",IF(OR(RIGHT(TRIM($B169),2)="P165",RIGHT(TRIM($B169),2)="P166",RIGHT(TRIM($B169),2)="P167",RIGHT(TRIM($B169),2)="P168"),"PS","GS"))</x:f>
+        <x:f>IF($B169="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B169),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E169" s="62" t="str">
         <x:f>IF($D169="","",IF($D169="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9741,7 +10083,7 @@
       <x:c r="B170" s="33"/>
       <x:c r="C170" s="59"/>
       <x:c r="D170" s="52" t="str">
-        <x:f>IF($B170="","",IF(OR(RIGHT(TRIM($B170),2)="P166",RIGHT(TRIM($B170),2)="P167",RIGHT(TRIM($B170),2)="P168",RIGHT(TRIM($B170),2)="P169"),"PS","GS"))</x:f>
+        <x:f>IF($B170="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B170),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E170" s="62" t="str">
         <x:f>IF($D170="","",IF($D170="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9794,7 +10136,7 @@
       <x:c r="B171" s="33"/>
       <x:c r="C171" s="59"/>
       <x:c r="D171" s="52" t="str">
-        <x:f>IF($B171="","",IF(OR(RIGHT(TRIM($B171),2)="P167",RIGHT(TRIM($B171),2)="P168",RIGHT(TRIM($B171),2)="P169",RIGHT(TRIM($B171),2)="P170"),"PS","GS"))</x:f>
+        <x:f>IF($B171="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B171),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E171" s="62" t="str">
         <x:f>IF($D171="","",IF($D171="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9847,7 +10189,7 @@
       <x:c r="B172" s="33"/>
       <x:c r="C172" s="59"/>
       <x:c r="D172" s="52" t="str">
-        <x:f>IF($B172="","",IF(OR(RIGHT(TRIM($B172),2)="P168",RIGHT(TRIM($B172),2)="P169",RIGHT(TRIM($B172),2)="P170",RIGHT(TRIM($B172),2)="P171"),"PS","GS"))</x:f>
+        <x:f>IF($B172="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B172),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E172" s="62" t="str">
         <x:f>IF($D172="","",IF($D172="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9900,7 +10242,7 @@
       <x:c r="B173" s="33"/>
       <x:c r="C173" s="59"/>
       <x:c r="D173" s="52" t="str">
-        <x:f>IF($B173="","",IF(OR(RIGHT(TRIM($B173),2)="P169",RIGHT(TRIM($B173),2)="P170",RIGHT(TRIM($B173),2)="P171",RIGHT(TRIM($B173),2)="P172"),"PS","GS"))</x:f>
+        <x:f>IF($B173="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B173),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E173" s="62" t="str">
         <x:f>IF($D173="","",IF($D173="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -9953,7 +10295,7 @@
       <x:c r="B174" s="33"/>
       <x:c r="C174" s="59"/>
       <x:c r="D174" s="52" t="str">
-        <x:f>IF($B174="","",IF(OR(RIGHT(TRIM($B174),2)="P170",RIGHT(TRIM($B174),2)="P171",RIGHT(TRIM($B174),2)="P172",RIGHT(TRIM($B174),2)="P173"),"PS","GS"))</x:f>
+        <x:f>IF($B174="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B174),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E174" s="62" t="str">
         <x:f>IF($D174="","",IF($D174="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10006,7 +10348,7 @@
       <x:c r="B175" s="33"/>
       <x:c r="C175" s="59"/>
       <x:c r="D175" s="52" t="str">
-        <x:f>IF($B175="","",IF(OR(RIGHT(TRIM($B175),2)="P171",RIGHT(TRIM($B175),2)="P172",RIGHT(TRIM($B175),2)="P173",RIGHT(TRIM($B175),2)="P174"),"PS","GS"))</x:f>
+        <x:f>IF($B175="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B175),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E175" s="62" t="str">
         <x:f>IF($D175="","",IF($D175="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10059,7 +10401,7 @@
       <x:c r="B176" s="33"/>
       <x:c r="C176" s="59"/>
       <x:c r="D176" s="52" t="str">
-        <x:f>IF($B176="","",IF(OR(RIGHT(TRIM($B176),2)="P172",RIGHT(TRIM($B176),2)="P173",RIGHT(TRIM($B176),2)="P174",RIGHT(TRIM($B176),2)="P175"),"PS","GS"))</x:f>
+        <x:f>IF($B176="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B176),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E176" s="62" t="str">
         <x:f>IF($D176="","",IF($D176="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10112,7 +10454,7 @@
       <x:c r="B177" s="33"/>
       <x:c r="C177" s="59"/>
       <x:c r="D177" s="52" t="str">
-        <x:f>IF($B177="","",IF(OR(RIGHT(TRIM($B177),2)="P173",RIGHT(TRIM($B177),2)="P174",RIGHT(TRIM($B177),2)="P175",RIGHT(TRIM($B177),2)="P176"),"PS","GS"))</x:f>
+        <x:f>IF($B177="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B177),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E177" s="62" t="str">
         <x:f>IF($D177="","",IF($D177="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10165,7 +10507,7 @@
       <x:c r="B178" s="33"/>
       <x:c r="C178" s="59"/>
       <x:c r="D178" s="52" t="str">
-        <x:f>IF($B178="","",IF(OR(RIGHT(TRIM($B178),2)="P174",RIGHT(TRIM($B178),2)="P175",RIGHT(TRIM($B178),2)="P176",RIGHT(TRIM($B178),2)="P177"),"PS","GS"))</x:f>
+        <x:f>IF($B178="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B178),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E178" s="62" t="str">
         <x:f>IF($D178="","",IF($D178="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10218,7 +10560,7 @@
       <x:c r="B179" s="33"/>
       <x:c r="C179" s="59"/>
       <x:c r="D179" s="52" t="str">
-        <x:f>IF($B179="","",IF(OR(RIGHT(TRIM($B179),2)="P175",RIGHT(TRIM($B179),2)="P176",RIGHT(TRIM($B179),2)="P177",RIGHT(TRIM($B179),2)="P178"),"PS","GS"))</x:f>
+        <x:f>IF($B179="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B179),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E179" s="62" t="str">
         <x:f>IF($D179="","",IF($D179="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10271,7 +10613,7 @@
       <x:c r="B180" s="33"/>
       <x:c r="C180" s="59"/>
       <x:c r="D180" s="52" t="str">
-        <x:f>IF($B180="","",IF(OR(RIGHT(TRIM($B180),2)="P176",RIGHT(TRIM($B180),2)="P177",RIGHT(TRIM($B180),2)="P178",RIGHT(TRIM($B180),2)="P179"),"PS","GS"))</x:f>
+        <x:f>IF($B180="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B180),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E180" s="62" t="str">
         <x:f>IF($D180="","",IF($D180="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10324,7 +10666,7 @@
       <x:c r="B181" s="33"/>
       <x:c r="C181" s="59"/>
       <x:c r="D181" s="52" t="str">
-        <x:f>IF($B181="","",IF(OR(RIGHT(TRIM($B181),2)="P177",RIGHT(TRIM($B181),2)="P178",RIGHT(TRIM($B181),2)="P179",RIGHT(TRIM($B181),2)="P180"),"PS","GS"))</x:f>
+        <x:f>IF($B181="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B181),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E181" s="62" t="str">
         <x:f>IF($D181="","",IF($D181="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10377,7 +10719,7 @@
       <x:c r="B182" s="33"/>
       <x:c r="C182" s="59"/>
       <x:c r="D182" s="52" t="str">
-        <x:f>IF($B182="","",IF(OR(RIGHT(TRIM($B182),2)="P178",RIGHT(TRIM($B182),2)="P179",RIGHT(TRIM($B182),2)="P180",RIGHT(TRIM($B182),2)="P181"),"PS","GS"))</x:f>
+        <x:f>IF($B182="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B182),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E182" s="62" t="str">
         <x:f>IF($D182="","",IF($D182="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10430,7 +10772,7 @@
       <x:c r="B183" s="33"/>
       <x:c r="C183" s="59"/>
       <x:c r="D183" s="52" t="str">
-        <x:f>IF($B183="","",IF(OR(RIGHT(TRIM($B183),2)="P179",RIGHT(TRIM($B183),2)="P180",RIGHT(TRIM($B183),2)="P181",RIGHT(TRIM($B183),2)="P182"),"PS","GS"))</x:f>
+        <x:f>IF($B183="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B183),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E183" s="62" t="str">
         <x:f>IF($D183="","",IF($D183="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10483,7 +10825,7 @@
       <x:c r="B184" s="33"/>
       <x:c r="C184" s="59"/>
       <x:c r="D184" s="52" t="str">
-        <x:f>IF($B184="","",IF(OR(RIGHT(TRIM($B184),2)="P180",RIGHT(TRIM($B184),2)="P181",RIGHT(TRIM($B184),2)="P182",RIGHT(TRIM($B184),2)="P183"),"PS","GS"))</x:f>
+        <x:f>IF($B184="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B184),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E184" s="62" t="str">
         <x:f>IF($D184="","",IF($D184="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10536,7 +10878,7 @@
       <x:c r="B185" s="33"/>
       <x:c r="C185" s="59"/>
       <x:c r="D185" s="52" t="str">
-        <x:f>IF($B185="","",IF(OR(RIGHT(TRIM($B185),2)="P181",RIGHT(TRIM($B185),2)="P182",RIGHT(TRIM($B185),2)="P183",RIGHT(TRIM($B185),2)="P184"),"PS","GS"))</x:f>
+        <x:f>IF($B185="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B185),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E185" s="62" t="str">
         <x:f>IF($D185="","",IF($D185="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10589,7 +10931,7 @@
       <x:c r="B186" s="33"/>
       <x:c r="C186" s="59"/>
       <x:c r="D186" s="52" t="str">
-        <x:f>IF($B186="","",IF(OR(RIGHT(TRIM($B186),2)="P182",RIGHT(TRIM($B186),2)="P183",RIGHT(TRIM($B186),2)="P184",RIGHT(TRIM($B186),2)="P185"),"PS","GS"))</x:f>
+        <x:f>IF($B186="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B186),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E186" s="62" t="str">
         <x:f>IF($D186="","",IF($D186="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10642,7 +10984,7 @@
       <x:c r="B187" s="33"/>
       <x:c r="C187" s="59"/>
       <x:c r="D187" s="52" t="str">
-        <x:f>IF($B187="","",IF(OR(RIGHT(TRIM($B187),2)="P183",RIGHT(TRIM($B187),2)="P184",RIGHT(TRIM($B187),2)="P185",RIGHT(TRIM($B187),2)="P186"),"PS","GS"))</x:f>
+        <x:f>IF($B187="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B187),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E187" s="62" t="str">
         <x:f>IF($D187="","",IF($D187="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10695,7 +11037,7 @@
       <x:c r="B188" s="33"/>
       <x:c r="C188" s="59"/>
       <x:c r="D188" s="52" t="str">
-        <x:f>IF($B188="","",IF(OR(RIGHT(TRIM($B188),2)="P184",RIGHT(TRIM($B188),2)="P185",RIGHT(TRIM($B188),2)="P186",RIGHT(TRIM($B188),2)="P187"),"PS","GS"))</x:f>
+        <x:f>IF($B188="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B188),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E188" s="62" t="str">
         <x:f>IF($D188="","",IF($D188="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10748,7 +11090,7 @@
       <x:c r="B189" s="33"/>
       <x:c r="C189" s="59"/>
       <x:c r="D189" s="52" t="str">
-        <x:f>IF($B189="","",IF(OR(RIGHT(TRIM($B189),2)="P185",RIGHT(TRIM($B189),2)="P186",RIGHT(TRIM($B189),2)="P187",RIGHT(TRIM($B189),2)="P188"),"PS","GS"))</x:f>
+        <x:f>IF($B189="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B189),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E189" s="62" t="str">
         <x:f>IF($D189="","",IF($D189="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10801,7 +11143,7 @@
       <x:c r="B190" s="33"/>
       <x:c r="C190" s="59"/>
       <x:c r="D190" s="52" t="str">
-        <x:f>IF($B190="","",IF(OR(RIGHT(TRIM($B190),2)="P186",RIGHT(TRIM($B190),2)="P187",RIGHT(TRIM($B190),2)="P188",RIGHT(TRIM($B190),2)="P189"),"PS","GS"))</x:f>
+        <x:f>IF($B190="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B190),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E190" s="62" t="str">
         <x:f>IF($D190="","",IF($D190="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10854,7 +11196,7 @@
       <x:c r="B191" s="33"/>
       <x:c r="C191" s="59"/>
       <x:c r="D191" s="52" t="str">
-        <x:f>IF($B191="","",IF(OR(RIGHT(TRIM($B191),2)="P187",RIGHT(TRIM($B191),2)="P188",RIGHT(TRIM($B191),2)="P189",RIGHT(TRIM($B191),2)="P190"),"PS","GS"))</x:f>
+        <x:f>IF($B191="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B191),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E191" s="62" t="str">
         <x:f>IF($D191="","",IF($D191="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10907,7 +11249,7 @@
       <x:c r="B192" s="33"/>
       <x:c r="C192" s="59"/>
       <x:c r="D192" s="52" t="str">
-        <x:f>IF($B192="","",IF(OR(RIGHT(TRIM($B192),2)="P188",RIGHT(TRIM($B192),2)="P189",RIGHT(TRIM($B192),2)="P190",RIGHT(TRIM($B192),2)="P191"),"PS","GS"))</x:f>
+        <x:f>IF($B192="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B192),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E192" s="62" t="str">
         <x:f>IF($D192="","",IF($D192="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -10960,7 +11302,7 @@
       <x:c r="B193" s="33"/>
       <x:c r="C193" s="59"/>
       <x:c r="D193" s="52" t="str">
-        <x:f>IF($B193="","",IF(OR(RIGHT(TRIM($B193),2)="P189",RIGHT(TRIM($B193),2)="P190",RIGHT(TRIM($B193),2)="P191",RIGHT(TRIM($B193),2)="P192"),"PS","GS"))</x:f>
+        <x:f>IF($B193="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B193),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E193" s="62" t="str">
         <x:f>IF($D193="","",IF($D193="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11013,7 +11355,7 @@
       <x:c r="B194" s="33"/>
       <x:c r="C194" s="59"/>
       <x:c r="D194" s="52" t="str">
-        <x:f>IF($B194="","",IF(OR(RIGHT(TRIM($B194),2)="P190",RIGHT(TRIM($B194),2)="P191",RIGHT(TRIM($B194),2)="P192",RIGHT(TRIM($B194),2)="P193"),"PS","GS"))</x:f>
+        <x:f>IF($B194="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B194),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E194" s="62" t="str">
         <x:f>IF($D194="","",IF($D194="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11066,7 +11408,7 @@
       <x:c r="B195" s="33"/>
       <x:c r="C195" s="59"/>
       <x:c r="D195" s="52" t="str">
-        <x:f>IF($B195="","",IF(OR(RIGHT(TRIM($B195),2)="P191",RIGHT(TRIM($B195),2)="P192",RIGHT(TRIM($B195),2)="P193",RIGHT(TRIM($B195),2)="P194"),"PS","GS"))</x:f>
+        <x:f>IF($B195="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B195),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E195" s="62" t="str">
         <x:f>IF($D195="","",IF($D195="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11119,7 +11461,7 @@
       <x:c r="B196" s="33"/>
       <x:c r="C196" s="59"/>
       <x:c r="D196" s="52" t="str">
-        <x:f>IF($B196="","",IF(OR(RIGHT(TRIM($B196),2)="P192",RIGHT(TRIM($B196),2)="P193",RIGHT(TRIM($B196),2)="P194",RIGHT(TRIM($B196),2)="P195"),"PS","GS"))</x:f>
+        <x:f>IF($B196="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B196),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E196" s="62" t="str">
         <x:f>IF($D196="","",IF($D196="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11172,7 +11514,7 @@
       <x:c r="B197" s="33"/>
       <x:c r="C197" s="59"/>
       <x:c r="D197" s="52" t="str">
-        <x:f>IF($B197="","",IF(OR(RIGHT(TRIM($B197),2)="P193",RIGHT(TRIM($B197),2)="P194",RIGHT(TRIM($B197),2)="P195",RIGHT(TRIM($B197),2)="P196"),"PS","GS"))</x:f>
+        <x:f>IF($B197="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B197),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E197" s="62" t="str">
         <x:f>IF($D197="","",IF($D197="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11225,7 +11567,7 @@
       <x:c r="B198" s="33"/>
       <x:c r="C198" s="59"/>
       <x:c r="D198" s="52" t="str">
-        <x:f>IF($B198="","",IF(OR(RIGHT(TRIM($B198),2)="P194",RIGHT(TRIM($B198),2)="P195",RIGHT(TRIM($B198),2)="P196",RIGHT(TRIM($B198),2)="P197"),"PS","GS"))</x:f>
+        <x:f>IF($B198="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B198),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E198" s="62" t="str">
         <x:f>IF($D198="","",IF($D198="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11278,7 +11620,7 @@
       <x:c r="B199" s="33"/>
       <x:c r="C199" s="59"/>
       <x:c r="D199" s="52" t="str">
-        <x:f>IF($B199="","",IF(OR(RIGHT(TRIM($B199),2)="P195",RIGHT(TRIM($B199),2)="P196",RIGHT(TRIM($B199),2)="P197",RIGHT(TRIM($B199),2)="P198"),"PS","GS"))</x:f>
+        <x:f>IF($B199="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B199),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E199" s="62" t="str">
         <x:f>IF($D199="","",IF($D199="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11331,7 +11673,7 @@
       <x:c r="B200" s="33"/>
       <x:c r="C200" s="59"/>
       <x:c r="D200" s="52" t="str">
-        <x:f>IF($B200="","",IF(OR(RIGHT(TRIM($B200),2)="P196",RIGHT(TRIM($B200),2)="P197",RIGHT(TRIM($B200),2)="P198",RIGHT(TRIM($B200),2)="P199"),"PS","GS"))</x:f>
+        <x:f>IF($B200="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B200),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E200" s="62" t="str">
         <x:f>IF($D200="","",IF($D200="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11384,7 +11726,7 @@
       <x:c r="B201" s="33"/>
       <x:c r="C201" s="59"/>
       <x:c r="D201" s="52" t="str">
-        <x:f>IF($B201="","",IF(OR(RIGHT(TRIM($B201),2)="P197",RIGHT(TRIM($B201),2)="P198",RIGHT(TRIM($B201),2)="P199",RIGHT(TRIM($B201),2)="P200"),"PS","GS"))</x:f>
+        <x:f>IF($B201="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B201),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E201" s="62" t="str">
         <x:f>IF($D201="","",IF($D201="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11437,7 +11779,7 @@
       <x:c r="B202" s="33"/>
       <x:c r="C202" s="59"/>
       <x:c r="D202" s="52" t="str">
-        <x:f>IF($B202="","",IF(OR(RIGHT(TRIM($B202),2)="P198",RIGHT(TRIM($B202),2)="P199",RIGHT(TRIM($B202),2)="P200",RIGHT(TRIM($B202),2)="P201"),"PS","GS"))</x:f>
+        <x:f>IF($B202="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B202),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E202" s="62" t="str">
         <x:f>IF($D202="","",IF($D202="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11490,7 +11832,7 @@
       <x:c r="B203" s="33"/>
       <x:c r="C203" s="59"/>
       <x:c r="D203" s="52" t="str">
-        <x:f>IF($B203="","",IF(OR(RIGHT(TRIM($B203),2)="P199",RIGHT(TRIM($B203),2)="P200",RIGHT(TRIM($B203),2)="P201",RIGHT(TRIM($B203),2)="P202"),"PS","GS"))</x:f>
+        <x:f>IF($B203="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B203),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E203" s="62" t="str">
         <x:f>IF($D203="","",IF($D203="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11543,7 +11885,7 @@
       <x:c r="B204" s="33"/>
       <x:c r="C204" s="59"/>
       <x:c r="D204" s="52" t="str">
-        <x:f>IF($B204="","",IF(OR(RIGHT(TRIM($B204),2)="P200",RIGHT(TRIM($B204),2)="P201",RIGHT(TRIM($B204),2)="P202",RIGHT(TRIM($B204),2)="P203"),"PS","GS"))</x:f>
+        <x:f>IF($B204="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B204),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E204" s="62" t="str">
         <x:f>IF($D204="","",IF($D204="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11596,7 +11938,7 @@
       <x:c r="B205" s="33"/>
       <x:c r="C205" s="59"/>
       <x:c r="D205" s="52" t="str">
-        <x:f>IF($B205="","",IF(OR(RIGHT(TRIM($B205),2)="P201",RIGHT(TRIM($B205),2)="P202",RIGHT(TRIM($B205),2)="P203",RIGHT(TRIM($B205),2)="P204"),"PS","GS"))</x:f>
+        <x:f>IF($B205="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B205),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E205" s="62" t="str">
         <x:f>IF($D205="","",IF($D205="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11649,7 +11991,7 @@
       <x:c r="B206" s="33"/>
       <x:c r="C206" s="59"/>
       <x:c r="D206" s="52" t="str">
-        <x:f>IF($B206="","",IF(OR(RIGHT(TRIM($B206),2)="P202",RIGHT(TRIM($B206),2)="P203",RIGHT(TRIM($B206),2)="P204",RIGHT(TRIM($B206),2)="P205"),"PS","GS"))</x:f>
+        <x:f>IF($B206="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B206),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E206" s="62" t="str">
         <x:f>IF($D206="","",IF($D206="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11702,7 +12044,7 @@
       <x:c r="B207" s="33"/>
       <x:c r="C207" s="59"/>
       <x:c r="D207" s="52" t="str">
-        <x:f>IF($B207="","",IF(OR(RIGHT(TRIM($B207),2)="P203",RIGHT(TRIM($B207),2)="P204",RIGHT(TRIM($B207),2)="P205",RIGHT(TRIM($B207),2)="P206"),"PS","GS"))</x:f>
+        <x:f>IF($B207="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B207),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E207" s="62" t="str">
         <x:f>IF($D207="","",IF($D207="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11755,7 +12097,7 @@
       <x:c r="B208" s="33"/>
       <x:c r="C208" s="59"/>
       <x:c r="D208" s="52" t="str">
-        <x:f>IF($B208="","",IF(OR(RIGHT(TRIM($B208),2)="P204",RIGHT(TRIM($B208),2)="P205",RIGHT(TRIM($B208),2)="P206",RIGHT(TRIM($B208),2)="P207"),"PS","GS"))</x:f>
+        <x:f>IF($B208="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B208),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E208" s="62" t="str">
         <x:f>IF($D208="","",IF($D208="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11808,7 +12150,7 @@
       <x:c r="B209" s="33"/>
       <x:c r="C209" s="59"/>
       <x:c r="D209" s="52" t="str">
-        <x:f>IF($B209="","",IF(OR(RIGHT(TRIM($B209),2)="P205",RIGHT(TRIM($B209),2)="P206",RIGHT(TRIM($B209),2)="P207",RIGHT(TRIM($B209),2)="P208"),"PS","GS"))</x:f>
+        <x:f>IF($B209="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B209),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E209" s="62" t="str">
         <x:f>IF($D209="","",IF($D209="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11861,7 +12203,7 @@
       <x:c r="B210" s="33"/>
       <x:c r="C210" s="59"/>
       <x:c r="D210" s="52" t="str">
-        <x:f>IF($B210="","",IF(OR(RIGHT(TRIM($B210),2)="P206",RIGHT(TRIM($B210),2)="P207",RIGHT(TRIM($B210),2)="P208",RIGHT(TRIM($B210),2)="P209"),"PS","GS"))</x:f>
+        <x:f>IF($B210="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B210),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E210" s="62" t="str">
         <x:f>IF($D210="","",IF($D210="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11914,7 +12256,7 @@
       <x:c r="B211" s="33"/>
       <x:c r="C211" s="59"/>
       <x:c r="D211" s="52" t="str">
-        <x:f>IF($B211="","",IF(OR(RIGHT(TRIM($B211),2)="P207",RIGHT(TRIM($B211),2)="P208",RIGHT(TRIM($B211),2)="P209",RIGHT(TRIM($B211),2)="P210"),"PS","GS"))</x:f>
+        <x:f>IF($B211="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B211),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E211" s="62" t="str">
         <x:f>IF($D211="","",IF($D211="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -11967,7 +12309,7 @@
       <x:c r="B212" s="33"/>
       <x:c r="C212" s="59"/>
       <x:c r="D212" s="52" t="str">
-        <x:f>IF($B212="","",IF(OR(RIGHT(TRIM($B212),2)="P208",RIGHT(TRIM($B212),2)="P209",RIGHT(TRIM($B212),2)="P210",RIGHT(TRIM($B212),2)="P211"),"PS","GS"))</x:f>
+        <x:f>IF($B212="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B212),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E212" s="62" t="str">
         <x:f>IF($D212="","",IF($D212="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12020,7 +12362,7 @@
       <x:c r="B213" s="33"/>
       <x:c r="C213" s="59"/>
       <x:c r="D213" s="52" t="str">
-        <x:f>IF($B213="","",IF(OR(RIGHT(TRIM($B213),2)="P209",RIGHT(TRIM($B213),2)="P210",RIGHT(TRIM($B213),2)="P211",RIGHT(TRIM($B213),2)="P212"),"PS","GS"))</x:f>
+        <x:f>IF($B213="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B213),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E213" s="62" t="str">
         <x:f>IF($D213="","",IF($D213="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12073,7 +12415,7 @@
       <x:c r="B214" s="33"/>
       <x:c r="C214" s="59"/>
       <x:c r="D214" s="52" t="str">
-        <x:f>IF($B214="","",IF(OR(RIGHT(TRIM($B214),2)="P210",RIGHT(TRIM($B214),2)="P211",RIGHT(TRIM($B214),2)="P212",RIGHT(TRIM($B214),2)="P213"),"PS","GS"))</x:f>
+        <x:f>IF($B214="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B214),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E214" s="62" t="str">
         <x:f>IF($D214="","",IF($D214="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12126,7 +12468,7 @@
       <x:c r="B215" s="33"/>
       <x:c r="C215" s="59"/>
       <x:c r="D215" s="52" t="str">
-        <x:f>IF($B215="","",IF(OR(RIGHT(TRIM($B215),2)="P211",RIGHT(TRIM($B215),2)="P212",RIGHT(TRIM($B215),2)="P213",RIGHT(TRIM($B215),2)="P214"),"PS","GS"))</x:f>
+        <x:f>IF($B215="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B215),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E215" s="62" t="str">
         <x:f>IF($D215="","",IF($D215="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12179,7 +12521,7 @@
       <x:c r="B216" s="33"/>
       <x:c r="C216" s="59"/>
       <x:c r="D216" s="52" t="str">
-        <x:f>IF($B216="","",IF(OR(RIGHT(TRIM($B216),2)="P212",RIGHT(TRIM($B216),2)="P213",RIGHT(TRIM($B216),2)="P214",RIGHT(TRIM($B216),2)="P215"),"PS","GS"))</x:f>
+        <x:f>IF($B216="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B216),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E216" s="62" t="str">
         <x:f>IF($D216="","",IF($D216="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12232,7 +12574,7 @@
       <x:c r="B217" s="33"/>
       <x:c r="C217" s="59"/>
       <x:c r="D217" s="52" t="str">
-        <x:f>IF($B217="","",IF(OR(RIGHT(TRIM($B217),2)="P213",RIGHT(TRIM($B217),2)="P214",RIGHT(TRIM($B217),2)="P215",RIGHT(TRIM($B217),2)="P216"),"PS","GS"))</x:f>
+        <x:f>IF($B217="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B217),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E217" s="62" t="str">
         <x:f>IF($D217="","",IF($D217="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12285,7 +12627,7 @@
       <x:c r="B218" s="33"/>
       <x:c r="C218" s="59"/>
       <x:c r="D218" s="52" t="str">
-        <x:f>IF($B218="","",IF(OR(RIGHT(TRIM($B218),2)="P214",RIGHT(TRIM($B218),2)="P215",RIGHT(TRIM($B218),2)="P216",RIGHT(TRIM($B218),2)="P217"),"PS","GS"))</x:f>
+        <x:f>IF($B218="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B218),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E218" s="62" t="str">
         <x:f>IF($D218="","",IF($D218="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12338,7 +12680,7 @@
       <x:c r="B219" s="33"/>
       <x:c r="C219" s="59"/>
       <x:c r="D219" s="52" t="str">
-        <x:f>IF($B219="","",IF(OR(RIGHT(TRIM($B219),2)="P215",RIGHT(TRIM($B219),2)="P216",RIGHT(TRIM($B219),2)="P217",RIGHT(TRIM($B219),2)="P218"),"PS","GS"))</x:f>
+        <x:f>IF($B219="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B219),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E219" s="62" t="str">
         <x:f>IF($D219="","",IF($D219="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12391,7 +12733,7 @@
       <x:c r="B220" s="33"/>
       <x:c r="C220" s="59"/>
       <x:c r="D220" s="52" t="str">
-        <x:f>IF($B220="","",IF(OR(RIGHT(TRIM($B220),2)="P216",RIGHT(TRIM($B220),2)="P217",RIGHT(TRIM($B220),2)="P218",RIGHT(TRIM($B220),2)="P219"),"PS","GS"))</x:f>
+        <x:f>IF($B220="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B220),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E220" s="62" t="str">
         <x:f>IF($D220="","",IF($D220="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12444,7 +12786,7 @@
       <x:c r="B221" s="33"/>
       <x:c r="C221" s="59"/>
       <x:c r="D221" s="52" t="str">
-        <x:f>IF($B221="","",IF(OR(RIGHT(TRIM($B221),2)="P217",RIGHT(TRIM($B221),2)="P218",RIGHT(TRIM($B221),2)="P219",RIGHT(TRIM($B221),2)="P220"),"PS","GS"))</x:f>
+        <x:f>IF($B221="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B221),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E221" s="62" t="str">
         <x:f>IF($D221="","",IF($D221="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12497,7 +12839,7 @@
       <x:c r="B222" s="33"/>
       <x:c r="C222" s="59"/>
       <x:c r="D222" s="52" t="str">
-        <x:f>IF($B222="","",IF(OR(RIGHT(TRIM($B222),2)="P218",RIGHT(TRIM($B222),2)="P219",RIGHT(TRIM($B222),2)="P220",RIGHT(TRIM($B222),2)="P221"),"PS","GS"))</x:f>
+        <x:f>IF($B222="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B222),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E222" s="62" t="str">
         <x:f>IF($D222="","",IF($D222="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12550,7 +12892,7 @@
       <x:c r="B223" s="33"/>
       <x:c r="C223" s="59"/>
       <x:c r="D223" s="52" t="str">
-        <x:f>IF($B223="","",IF(OR(RIGHT(TRIM($B223),2)="P219",RIGHT(TRIM($B223),2)="P220",RIGHT(TRIM($B223),2)="P221",RIGHT(TRIM($B223),2)="P222"),"PS","GS"))</x:f>
+        <x:f>IF($B223="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B223),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E223" s="62" t="str">
         <x:f>IF($D223="","",IF($D223="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12603,7 +12945,7 @@
       <x:c r="B224" s="33"/>
       <x:c r="C224" s="59"/>
       <x:c r="D224" s="52" t="str">
-        <x:f>IF($B224="","",IF(OR(RIGHT(TRIM($B224),2)="P220",RIGHT(TRIM($B224),2)="P221",RIGHT(TRIM($B224),2)="P222",RIGHT(TRIM($B224),2)="P223"),"PS","GS"))</x:f>
+        <x:f>IF($B224="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B224),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E224" s="62" t="str">
         <x:f>IF($D224="","",IF($D224="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12656,7 +12998,7 @@
       <x:c r="B225" s="33"/>
       <x:c r="C225" s="59"/>
       <x:c r="D225" s="52" t="str">
-        <x:f>IF($B225="","",IF(OR(RIGHT(TRIM($B225),2)="P221",RIGHT(TRIM($B225),2)="P222",RIGHT(TRIM($B225),2)="P223",RIGHT(TRIM($B225),2)="P224"),"PS","GS"))</x:f>
+        <x:f>IF($B225="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B225),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E225" s="62" t="str">
         <x:f>IF($D225="","",IF($D225="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12709,7 +13051,7 @@
       <x:c r="B226" s="33"/>
       <x:c r="C226" s="59"/>
       <x:c r="D226" s="52" t="str">
-        <x:f>IF($B226="","",IF(OR(RIGHT(TRIM($B226),2)="P222",RIGHT(TRIM($B226),2)="P223",RIGHT(TRIM($B226),2)="P224",RIGHT(TRIM($B226),2)="P225"),"PS","GS"))</x:f>
+        <x:f>IF($B226="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B226),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E226" s="62" t="str">
         <x:f>IF($D226="","",IF($D226="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12762,7 +13104,7 @@
       <x:c r="B227" s="33"/>
       <x:c r="C227" s="59"/>
       <x:c r="D227" s="52" t="str">
-        <x:f>IF($B227="","",IF(OR(RIGHT(TRIM($B227),2)="P223",RIGHT(TRIM($B227),2)="P224",RIGHT(TRIM($B227),2)="P225",RIGHT(TRIM($B227),2)="P226"),"PS","GS"))</x:f>
+        <x:f>IF($B227="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B227),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E227" s="62" t="str">
         <x:f>IF($D227="","",IF($D227="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12815,7 +13157,7 @@
       <x:c r="B228" s="33"/>
       <x:c r="C228" s="59"/>
       <x:c r="D228" s="52" t="str">
-        <x:f>IF($B228="","",IF(OR(RIGHT(TRIM($B228),2)="P224",RIGHT(TRIM($B228),2)="P225",RIGHT(TRIM($B228),2)="P226",RIGHT(TRIM($B228),2)="P227"),"PS","GS"))</x:f>
+        <x:f>IF($B228="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B228),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E228" s="62" t="str">
         <x:f>IF($D228="","",IF($D228="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12868,7 +13210,7 @@
       <x:c r="B229" s="33"/>
       <x:c r="C229" s="59"/>
       <x:c r="D229" s="52" t="str">
-        <x:f>IF($B229="","",IF(OR(RIGHT(TRIM($B229),2)="P225",RIGHT(TRIM($B229),2)="P226",RIGHT(TRIM($B229),2)="P227",RIGHT(TRIM($B229),2)="P228"),"PS","GS"))</x:f>
+        <x:f>IF($B229="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B229),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E229" s="62" t="str">
         <x:f>IF($D229="","",IF($D229="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12921,7 +13263,7 @@
       <x:c r="B230" s="33"/>
       <x:c r="C230" s="59"/>
       <x:c r="D230" s="52" t="str">
-        <x:f>IF($B230="","",IF(OR(RIGHT(TRIM($B230),2)="P226",RIGHT(TRIM($B230),2)="P227",RIGHT(TRIM($B230),2)="P228",RIGHT(TRIM($B230),2)="P229"),"PS","GS"))</x:f>
+        <x:f>IF($B230="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B230),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E230" s="62" t="str">
         <x:f>IF($D230="","",IF($D230="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -12974,7 +13316,7 @@
       <x:c r="B231" s="33"/>
       <x:c r="C231" s="59"/>
       <x:c r="D231" s="52" t="str">
-        <x:f>IF($B231="","",IF(OR(RIGHT(TRIM($B231),2)="P227",RIGHT(TRIM($B231),2)="P228",RIGHT(TRIM($B231),2)="P229",RIGHT(TRIM($B231),2)="P230"),"PS","GS"))</x:f>
+        <x:f>IF($B231="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B231),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E231" s="62" t="str">
         <x:f>IF($D231="","",IF($D231="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13027,7 +13369,7 @@
       <x:c r="B232" s="33"/>
       <x:c r="C232" s="59"/>
       <x:c r="D232" s="52" t="str">
-        <x:f>IF($B232="","",IF(OR(RIGHT(TRIM($B232),2)="P228",RIGHT(TRIM($B232),2)="P229",RIGHT(TRIM($B232),2)="P230",RIGHT(TRIM($B232),2)="P231"),"PS","GS"))</x:f>
+        <x:f>IF($B232="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B232),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E232" s="62" t="str">
         <x:f>IF($D232="","",IF($D232="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13080,7 +13422,7 @@
       <x:c r="B233" s="33"/>
       <x:c r="C233" s="59"/>
       <x:c r="D233" s="52" t="str">
-        <x:f>IF($B233="","",IF(OR(RIGHT(TRIM($B233),2)="P229",RIGHT(TRIM($B233),2)="P230",RIGHT(TRIM($B233),2)="P231",RIGHT(TRIM($B233),2)="P232"),"PS","GS"))</x:f>
+        <x:f>IF($B233="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B233),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E233" s="62" t="str">
         <x:f>IF($D233="","",IF($D233="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13133,7 +13475,7 @@
       <x:c r="B234" s="33"/>
       <x:c r="C234" s="59"/>
       <x:c r="D234" s="52" t="str">
-        <x:f>IF($B234="","",IF(OR(RIGHT(TRIM($B234),2)="P230",RIGHT(TRIM($B234),2)="P231",RIGHT(TRIM($B234),2)="P232",RIGHT(TRIM($B234),2)="P233"),"PS","GS"))</x:f>
+        <x:f>IF($B234="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B234),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E234" s="62" t="str">
         <x:f>IF($D234="","",IF($D234="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13186,7 +13528,7 @@
       <x:c r="B235" s="33"/>
       <x:c r="C235" s="59"/>
       <x:c r="D235" s="52" t="str">
-        <x:f>IF($B235="","",IF(OR(RIGHT(TRIM($B235),2)="P231",RIGHT(TRIM($B235),2)="P232",RIGHT(TRIM($B235),2)="P233",RIGHT(TRIM($B235),2)="P234"),"PS","GS"))</x:f>
+        <x:f>IF($B235="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B235),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E235" s="62" t="str">
         <x:f>IF($D235="","",IF($D235="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13239,7 +13581,7 @@
       <x:c r="B236" s="33"/>
       <x:c r="C236" s="59"/>
       <x:c r="D236" s="52" t="str">
-        <x:f>IF($B236="","",IF(OR(RIGHT(TRIM($B236),2)="P232",RIGHT(TRIM($B236),2)="P233",RIGHT(TRIM($B236),2)="P234",RIGHT(TRIM($B236),2)="P235"),"PS","GS"))</x:f>
+        <x:f>IF($B236="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B236),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E236" s="62" t="str">
         <x:f>IF($D236="","",IF($D236="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13292,7 +13634,7 @@
       <x:c r="B237" s="33"/>
       <x:c r="C237" s="59"/>
       <x:c r="D237" s="52" t="str">
-        <x:f>IF($B237="","",IF(OR(RIGHT(TRIM($B237),2)="P233",RIGHT(TRIM($B237),2)="P234",RIGHT(TRIM($B237),2)="P235",RIGHT(TRIM($B237),2)="P236"),"PS","GS"))</x:f>
+        <x:f>IF($B237="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B237),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E237" s="62" t="str">
         <x:f>IF($D237="","",IF($D237="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13345,7 +13687,7 @@
       <x:c r="B238" s="33"/>
       <x:c r="C238" s="59"/>
       <x:c r="D238" s="52" t="str">
-        <x:f>IF($B238="","",IF(OR(RIGHT(TRIM($B238),2)="P234",RIGHT(TRIM($B238),2)="P235",RIGHT(TRIM($B238),2)="P236",RIGHT(TRIM($B238),2)="P237"),"PS","GS"))</x:f>
+        <x:f>IF($B238="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B238),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E238" s="62" t="str">
         <x:f>IF($D238="","",IF($D238="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13398,7 +13740,7 @@
       <x:c r="B239" s="33"/>
       <x:c r="C239" s="59"/>
       <x:c r="D239" s="52" t="str">
-        <x:f>IF($B239="","",IF(OR(RIGHT(TRIM($B239),2)="P235",RIGHT(TRIM($B239),2)="P236",RIGHT(TRIM($B239),2)="P237",RIGHT(TRIM($B239),2)="P238"),"PS","GS"))</x:f>
+        <x:f>IF($B239="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B239),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E239" s="62" t="str">
         <x:f>IF($D239="","",IF($D239="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13451,7 +13793,7 @@
       <x:c r="B240" s="33"/>
       <x:c r="C240" s="59"/>
       <x:c r="D240" s="52" t="str">
-        <x:f>IF($B240="","",IF(OR(RIGHT(TRIM($B240),2)="P236",RIGHT(TRIM($B240),2)="P237",RIGHT(TRIM($B240),2)="P238",RIGHT(TRIM($B240),2)="P239"),"PS","GS"))</x:f>
+        <x:f>IF($B240="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B240),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E240" s="62" t="str">
         <x:f>IF($D240="","",IF($D240="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13504,7 +13846,7 @@
       <x:c r="B241" s="33"/>
       <x:c r="C241" s="59"/>
       <x:c r="D241" s="52" t="str">
-        <x:f>IF($B241="","",IF(OR(RIGHT(TRIM($B241),2)="P237",RIGHT(TRIM($B241),2)="P238",RIGHT(TRIM($B241),2)="P239",RIGHT(TRIM($B241),2)="P240"),"PS","GS"))</x:f>
+        <x:f>IF($B241="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B241),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E241" s="62" t="str">
         <x:f>IF($D241="","",IF($D241="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13557,7 +13899,7 @@
       <x:c r="B242" s="33"/>
       <x:c r="C242" s="59"/>
       <x:c r="D242" s="52" t="str">
-        <x:f>IF($B242="","",IF(OR(RIGHT(TRIM($B242),2)="P238",RIGHT(TRIM($B242),2)="P239",RIGHT(TRIM($B242),2)="P240",RIGHT(TRIM($B242),2)="P241"),"PS","GS"))</x:f>
+        <x:f>IF($B242="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B242),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E242" s="62" t="str">
         <x:f>IF($D242="","",IF($D242="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13610,7 +13952,7 @@
       <x:c r="B243" s="33"/>
       <x:c r="C243" s="59"/>
       <x:c r="D243" s="52" t="str">
-        <x:f>IF($B243="","",IF(OR(RIGHT(TRIM($B243),2)="P239",RIGHT(TRIM($B243),2)="P240",RIGHT(TRIM($B243),2)="P241",RIGHT(TRIM($B243),2)="P242"),"PS","GS"))</x:f>
+        <x:f>IF($B243="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B243),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E243" s="62" t="str">
         <x:f>IF($D243="","",IF($D243="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13663,7 +14005,7 @@
       <x:c r="B244" s="33"/>
       <x:c r="C244" s="59"/>
       <x:c r="D244" s="52" t="str">
-        <x:f>IF($B244="","",IF(OR(RIGHT(TRIM($B244),2)="P240",RIGHT(TRIM($B244),2)="P241",RIGHT(TRIM($B244),2)="P242",RIGHT(TRIM($B244),2)="P243"),"PS","GS"))</x:f>
+        <x:f>IF($B244="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B244),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E244" s="62" t="str">
         <x:f>IF($D244="","",IF($D244="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13716,7 +14058,7 @@
       <x:c r="B245" s="33"/>
       <x:c r="C245" s="59"/>
       <x:c r="D245" s="52" t="str">
-        <x:f>IF($B245="","",IF(OR(RIGHT(TRIM($B245),2)="P241",RIGHT(TRIM($B245),2)="P242",RIGHT(TRIM($B245),2)="P243",RIGHT(TRIM($B245),2)="P244"),"PS","GS"))</x:f>
+        <x:f>IF($B245="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B245),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E245" s="62" t="str">
         <x:f>IF($D245="","",IF($D245="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13769,7 +14111,7 @@
       <x:c r="B246" s="33"/>
       <x:c r="C246" s="59"/>
       <x:c r="D246" s="52" t="str">
-        <x:f>IF($B246="","",IF(OR(RIGHT(TRIM($B246),2)="P242",RIGHT(TRIM($B246),2)="P243",RIGHT(TRIM($B246),2)="P244",RIGHT(TRIM($B246),2)="P245"),"PS","GS"))</x:f>
+        <x:f>IF($B246="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B246),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E246" s="62" t="str">
         <x:f>IF($D246="","",IF($D246="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13822,7 +14164,7 @@
       <x:c r="B247" s="33"/>
       <x:c r="C247" s="59"/>
       <x:c r="D247" s="52" t="str">
-        <x:f>IF($B247="","",IF(OR(RIGHT(TRIM($B247),2)="P243",RIGHT(TRIM($B247),2)="P244",RIGHT(TRIM($B247),2)="P245",RIGHT(TRIM($B247),2)="P246"),"PS","GS"))</x:f>
+        <x:f>IF($B247="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B247),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E247" s="62" t="str">
         <x:f>IF($D247="","",IF($D247="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13875,7 +14217,7 @@
       <x:c r="B248" s="33"/>
       <x:c r="C248" s="59"/>
       <x:c r="D248" s="52" t="str">
-        <x:f>IF($B248="","",IF(OR(RIGHT(TRIM($B248),2)="P244",RIGHT(TRIM($B248),2)="P245",RIGHT(TRIM($B248),2)="P246",RIGHT(TRIM($B248),2)="P247"),"PS","GS"))</x:f>
+        <x:f>IF($B248="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B248),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E248" s="62" t="str">
         <x:f>IF($D248="","",IF($D248="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13928,7 +14270,7 @@
       <x:c r="B249" s="33"/>
       <x:c r="C249" s="59"/>
       <x:c r="D249" s="52" t="str">
-        <x:f>IF($B249="","",IF(OR(RIGHT(TRIM($B249),2)="P245",RIGHT(TRIM($B249),2)="P246",RIGHT(TRIM($B249),2)="P247",RIGHT(TRIM($B249),2)="P248"),"PS","GS"))</x:f>
+        <x:f>IF($B249="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B249),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E249" s="62" t="str">
         <x:f>IF($D249="","",IF($D249="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -13981,7 +14323,7 @@
       <x:c r="B250" s="33"/>
       <x:c r="C250" s="59"/>
       <x:c r="D250" s="52" t="str">
-        <x:f>IF($B250="","",IF(OR(RIGHT(TRIM($B250),2)="P246",RIGHT(TRIM($B250),2)="P247",RIGHT(TRIM($B250),2)="P248",RIGHT(TRIM($B250),2)="P249"),"PS","GS"))</x:f>
+        <x:f>IF($B250="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B250),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E250" s="62" t="str">
         <x:f>IF($D250="","",IF($D250="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14034,7 +14376,7 @@
       <x:c r="B251" s="33"/>
       <x:c r="C251" s="59"/>
       <x:c r="D251" s="52" t="str">
-        <x:f>IF($B251="","",IF(OR(RIGHT(TRIM($B251),2)="P247",RIGHT(TRIM($B251),2)="P248",RIGHT(TRIM($B251),2)="P249",RIGHT(TRIM($B251),2)="P250"),"PS","GS"))</x:f>
+        <x:f>IF($B251="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B251),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E251" s="62" t="str">
         <x:f>IF($D251="","",IF($D251="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14087,7 +14429,7 @@
       <x:c r="B252" s="33"/>
       <x:c r="C252" s="59"/>
       <x:c r="D252" s="52" t="str">
-        <x:f>IF($B252="","",IF(OR(RIGHT(TRIM($B252),2)="P248",RIGHT(TRIM($B252),2)="P249",RIGHT(TRIM($B252),2)="P250",RIGHT(TRIM($B252),2)="P251"),"PS","GS"))</x:f>
+        <x:f>IF($B252="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B252),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E252" s="62" t="str">
         <x:f>IF($D252="","",IF($D252="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14140,7 +14482,7 @@
       <x:c r="B253" s="33"/>
       <x:c r="C253" s="59"/>
       <x:c r="D253" s="52" t="str">
-        <x:f>IF($B253="","",IF(OR(RIGHT(TRIM($B253),2)="P249",RIGHT(TRIM($B253),2)="P250",RIGHT(TRIM($B253),2)="P251",RIGHT(TRIM($B253),2)="P252"),"PS","GS"))</x:f>
+        <x:f>IF($B253="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B253),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E253" s="62" t="str">
         <x:f>IF($D253="","",IF($D253="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14193,7 +14535,7 @@
       <x:c r="B254" s="33"/>
       <x:c r="C254" s="59"/>
       <x:c r="D254" s="52" t="str">
-        <x:f>IF($B254="","",IF(OR(RIGHT(TRIM($B254),2)="P250",RIGHT(TRIM($B254),2)="P251",RIGHT(TRIM($B254),2)="P252",RIGHT(TRIM($B254),2)="P253"),"PS","GS"))</x:f>
+        <x:f>IF($B254="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B254),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E254" s="62" t="str">
         <x:f>IF($D254="","",IF($D254="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14246,7 +14588,7 @@
       <x:c r="B255" s="33"/>
       <x:c r="C255" s="59"/>
       <x:c r="D255" s="52" t="str">
-        <x:f>IF($B255="","",IF(OR(RIGHT(TRIM($B255),2)="P251",RIGHT(TRIM($B255),2)="P252",RIGHT(TRIM($B255),2)="P253",RIGHT(TRIM($B255),2)="P254"),"PS","GS"))</x:f>
+        <x:f>IF($B255="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B255),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E255" s="62" t="str">
         <x:f>IF($D255="","",IF($D255="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14299,7 +14641,7 @@
       <x:c r="B256" s="33"/>
       <x:c r="C256" s="59"/>
       <x:c r="D256" s="52" t="str">
-        <x:f>IF($B256="","",IF(OR(RIGHT(TRIM($B256),2)="P252",RIGHT(TRIM($B256),2)="P253",RIGHT(TRIM($B256),2)="P254",RIGHT(TRIM($B256),2)="P255"),"PS","GS"))</x:f>
+        <x:f>IF($B256="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B256),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E256" s="62" t="str">
         <x:f>IF($D256="","",IF($D256="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14352,7 +14694,7 @@
       <x:c r="B257" s="33"/>
       <x:c r="C257" s="59"/>
       <x:c r="D257" s="52" t="str">
-        <x:f>IF($B257="","",IF(OR(RIGHT(TRIM($B257),2)="P253",RIGHT(TRIM($B257),2)="P254",RIGHT(TRIM($B257),2)="P255",RIGHT(TRIM($B257),2)="P256"),"PS","GS"))</x:f>
+        <x:f>IF($B257="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B257),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E257" s="62" t="str">
         <x:f>IF($D257="","",IF($D257="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14405,7 +14747,7 @@
       <x:c r="B258" s="33"/>
       <x:c r="C258" s="59"/>
       <x:c r="D258" s="52" t="str">
-        <x:f>IF($B258="","",IF(OR(RIGHT(TRIM($B258),2)="P254",RIGHT(TRIM($B258),2)="P255",RIGHT(TRIM($B258),2)="P256",RIGHT(TRIM($B258),2)="P257"),"PS","GS"))</x:f>
+        <x:f>IF($B258="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B258),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E258" s="62" t="str">
         <x:f>IF($D258="","",IF($D258="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14458,7 +14800,7 @@
       <x:c r="B259" s="33"/>
       <x:c r="C259" s="59"/>
       <x:c r="D259" s="52" t="str">
-        <x:f>IF($B259="","",IF(OR(RIGHT(TRIM($B259),2)="P255",RIGHT(TRIM($B259),2)="P256",RIGHT(TRIM($B259),2)="P257",RIGHT(TRIM($B259),2)="P258"),"PS","GS"))</x:f>
+        <x:f>IF($B259="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B259),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E259" s="62" t="str">
         <x:f>IF($D259="","",IF($D259="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14511,7 +14853,7 @@
       <x:c r="B260" s="33"/>
       <x:c r="C260" s="59"/>
       <x:c r="D260" s="52" t="str">
-        <x:f>IF($B260="","",IF(OR(RIGHT(TRIM($B260),2)="P256",RIGHT(TRIM($B260),2)="P257",RIGHT(TRIM($B260),2)="P258",RIGHT(TRIM($B260),2)="P259"),"PS","GS"))</x:f>
+        <x:f>IF($B260="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B260),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E260" s="62" t="str">
         <x:f>IF($D260="","",IF($D260="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14564,7 +14906,7 @@
       <x:c r="B261" s="33"/>
       <x:c r="C261" s="59"/>
       <x:c r="D261" s="52" t="str">
-        <x:f>IF($B261="","",IF(OR(RIGHT(TRIM($B261),2)="P257",RIGHT(TRIM($B261),2)="P258",RIGHT(TRIM($B261),2)="P259",RIGHT(TRIM($B261),2)="P260"),"PS","GS"))</x:f>
+        <x:f>IF($B261="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B261),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E261" s="62" t="str">
         <x:f>IF($D261="","",IF($D261="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14617,7 +14959,7 @@
       <x:c r="B262" s="33"/>
       <x:c r="C262" s="59"/>
       <x:c r="D262" s="52" t="str">
-        <x:f>IF($B262="","",IF(OR(RIGHT(TRIM($B262),2)="P258",RIGHT(TRIM($B262),2)="P259",RIGHT(TRIM($B262),2)="P260",RIGHT(TRIM($B262),2)="P261"),"PS","GS"))</x:f>
+        <x:f>IF($B262="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B262),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E262" s="62" t="str">
         <x:f>IF($D262="","",IF($D262="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14670,7 +15012,7 @@
       <x:c r="B263" s="33"/>
       <x:c r="C263" s="59"/>
       <x:c r="D263" s="52" t="str">
-        <x:f>IF($B263="","",IF(OR(RIGHT(TRIM($B263),2)="P259",RIGHT(TRIM($B263),2)="P260",RIGHT(TRIM($B263),2)="P261",RIGHT(TRIM($B263),2)="P262"),"PS","GS"))</x:f>
+        <x:f>IF($B263="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B263),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E263" s="62" t="str">
         <x:f>IF($D263="","",IF($D263="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14723,7 +15065,7 @@
       <x:c r="B264" s="33"/>
       <x:c r="C264" s="59"/>
       <x:c r="D264" s="52" t="str">
-        <x:f>IF($B264="","",IF(OR(RIGHT(TRIM($B264),2)="P260",RIGHT(TRIM($B264),2)="P261",RIGHT(TRIM($B264),2)="P262",RIGHT(TRIM($B264),2)="P263"),"PS","GS"))</x:f>
+        <x:f>IF($B264="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B264),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E264" s="62" t="str">
         <x:f>IF($D264="","",IF($D264="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14776,7 +15118,7 @@
       <x:c r="B265" s="33"/>
       <x:c r="C265" s="59"/>
       <x:c r="D265" s="52" t="str">
-        <x:f>IF($B265="","",IF(OR(RIGHT(TRIM($B265),2)="P261",RIGHT(TRIM($B265),2)="P262",RIGHT(TRIM($B265),2)="P263",RIGHT(TRIM($B265),2)="P264"),"PS","GS"))</x:f>
+        <x:f>IF($B265="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B265),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E265" s="62" t="str">
         <x:f>IF($D265="","",IF($D265="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14829,7 +15171,7 @@
       <x:c r="B266" s="33"/>
       <x:c r="C266" s="59"/>
       <x:c r="D266" s="52" t="str">
-        <x:f>IF($B266="","",IF(OR(RIGHT(TRIM($B266),2)="P262",RIGHT(TRIM($B266),2)="P263",RIGHT(TRIM($B266),2)="P264",RIGHT(TRIM($B266),2)="P265"),"PS","GS"))</x:f>
+        <x:f>IF($B266="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B266),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E266" s="62" t="str">
         <x:f>IF($D266="","",IF($D266="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14882,7 +15224,7 @@
       <x:c r="B267" s="33"/>
       <x:c r="C267" s="59"/>
       <x:c r="D267" s="52" t="str">
-        <x:f>IF($B267="","",IF(OR(RIGHT(TRIM($B267),2)="P263",RIGHT(TRIM($B267),2)="P264",RIGHT(TRIM($B267),2)="P265",RIGHT(TRIM($B267),2)="P266"),"PS","GS"))</x:f>
+        <x:f>IF($B267="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B267),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E267" s="62" t="str">
         <x:f>IF($D267="","",IF($D267="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14935,7 +15277,7 @@
       <x:c r="B268" s="33"/>
       <x:c r="C268" s="59"/>
       <x:c r="D268" s="52" t="str">
-        <x:f>IF($B268="","",IF(OR(RIGHT(TRIM($B268),2)="P264",RIGHT(TRIM($B268),2)="P265",RIGHT(TRIM($B268),2)="P266",RIGHT(TRIM($B268),2)="P267"),"PS","GS"))</x:f>
+        <x:f>IF($B268="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B268),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E268" s="62" t="str">
         <x:f>IF($D268="","",IF($D268="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -14988,7 +15330,7 @@
       <x:c r="B269" s="33"/>
       <x:c r="C269" s="59"/>
       <x:c r="D269" s="52" t="str">
-        <x:f>IF($B269="","",IF(OR(RIGHT(TRIM($B269),2)="P265",RIGHT(TRIM($B269),2)="P266",RIGHT(TRIM($B269),2)="P267",RIGHT(TRIM($B269),2)="P268"),"PS","GS"))</x:f>
+        <x:f>IF($B269="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B269),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E269" s="62" t="str">
         <x:f>IF($D269="","",IF($D269="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15041,7 +15383,7 @@
       <x:c r="B270" s="33"/>
       <x:c r="C270" s="59"/>
       <x:c r="D270" s="52" t="str">
-        <x:f>IF($B270="","",IF(OR(RIGHT(TRIM($B270),2)="P266",RIGHT(TRIM($B270),2)="P267",RIGHT(TRIM($B270),2)="P268",RIGHT(TRIM($B270),2)="P269"),"PS","GS"))</x:f>
+        <x:f>IF($B270="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B270),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E270" s="62" t="str">
         <x:f>IF($D270="","",IF($D270="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15094,7 +15436,7 @@
       <x:c r="B271" s="33"/>
       <x:c r="C271" s="59"/>
       <x:c r="D271" s="52" t="str">
-        <x:f>IF($B271="","",IF(OR(RIGHT(TRIM($B271),2)="P267",RIGHT(TRIM($B271),2)="P268",RIGHT(TRIM($B271),2)="P269",RIGHT(TRIM($B271),2)="P270"),"PS","GS"))</x:f>
+        <x:f>IF($B271="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B271),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E271" s="62" t="str">
         <x:f>IF($D271="","",IF($D271="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15147,7 +15489,7 @@
       <x:c r="B272" s="33"/>
       <x:c r="C272" s="59"/>
       <x:c r="D272" s="52" t="str">
-        <x:f>IF($B272="","",IF(OR(RIGHT(TRIM($B272),2)="P268",RIGHT(TRIM($B272),2)="P269",RIGHT(TRIM($B272),2)="P270",RIGHT(TRIM($B272),2)="P271"),"PS","GS"))</x:f>
+        <x:f>IF($B272="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B272),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E272" s="62" t="str">
         <x:f>IF($D272="","",IF($D272="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15200,7 +15542,7 @@
       <x:c r="B273" s="33"/>
       <x:c r="C273" s="59"/>
       <x:c r="D273" s="52" t="str">
-        <x:f>IF($B273="","",IF(OR(RIGHT(TRIM($B273),2)="P269",RIGHT(TRIM($B273),2)="P270",RIGHT(TRIM($B273),2)="P271",RIGHT(TRIM($B273),2)="P272"),"PS","GS"))</x:f>
+        <x:f>IF($B273="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B273),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E273" s="62" t="str">
         <x:f>IF($D273="","",IF($D273="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15253,7 +15595,7 @@
       <x:c r="B274" s="33"/>
       <x:c r="C274" s="59"/>
       <x:c r="D274" s="52" t="str">
-        <x:f>IF($B274="","",IF(OR(RIGHT(TRIM($B274),2)="P270",RIGHT(TRIM($B274),2)="P271",RIGHT(TRIM($B274),2)="P272",RIGHT(TRIM($B274),2)="P273"),"PS","GS"))</x:f>
+        <x:f>IF($B274="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B274),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E274" s="62" t="str">
         <x:f>IF($D274="","",IF($D274="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15306,7 +15648,7 @@
       <x:c r="B275" s="33"/>
       <x:c r="C275" s="59"/>
       <x:c r="D275" s="52" t="str">
-        <x:f>IF($B275="","",IF(OR(RIGHT(TRIM($B275),2)="P271",RIGHT(TRIM($B275),2)="P272",RIGHT(TRIM($B275),2)="P273",RIGHT(TRIM($B275),2)="P274"),"PS","GS"))</x:f>
+        <x:f>IF($B275="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B275),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E275" s="62" t="str">
         <x:f>IF($D275="","",IF($D275="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15359,7 +15701,7 @@
       <x:c r="B276" s="33"/>
       <x:c r="C276" s="59"/>
       <x:c r="D276" s="52" t="str">
-        <x:f>IF($B276="","",IF(OR(RIGHT(TRIM($B276),2)="P272",RIGHT(TRIM($B276),2)="P273",RIGHT(TRIM($B276),2)="P274",RIGHT(TRIM($B276),2)="P275"),"PS","GS"))</x:f>
+        <x:f>IF($B276="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B276),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E276" s="62" t="str">
         <x:f>IF($D276="","",IF($D276="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15412,7 +15754,7 @@
       <x:c r="B277" s="33"/>
       <x:c r="C277" s="59"/>
       <x:c r="D277" s="52" t="str">
-        <x:f>IF($B277="","",IF(OR(RIGHT(TRIM($B277),2)="P273",RIGHT(TRIM($B277),2)="P274",RIGHT(TRIM($B277),2)="P275",RIGHT(TRIM($B277),2)="P276"),"PS","GS"))</x:f>
+        <x:f>IF($B277="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B277),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E277" s="62" t="str">
         <x:f>IF($D277="","",IF($D277="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15465,7 +15807,7 @@
       <x:c r="B278" s="33"/>
       <x:c r="C278" s="59"/>
       <x:c r="D278" s="52" t="str">
-        <x:f>IF($B278="","",IF(OR(RIGHT(TRIM($B278),2)="P274",RIGHT(TRIM($B278),2)="P275",RIGHT(TRIM($B278),2)="P276",RIGHT(TRIM($B278),2)="P277"),"PS","GS"))</x:f>
+        <x:f>IF($B278="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B278),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E278" s="62" t="str">
         <x:f>IF($D278="","",IF($D278="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15518,7 +15860,7 @@
       <x:c r="B279" s="33"/>
       <x:c r="C279" s="59"/>
       <x:c r="D279" s="52" t="str">
-        <x:f>IF($B279="","",IF(OR(RIGHT(TRIM($B279),2)="P275",RIGHT(TRIM($B279),2)="P276",RIGHT(TRIM($B279),2)="P277",RIGHT(TRIM($B279),2)="P278"),"PS","GS"))</x:f>
+        <x:f>IF($B279="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B279),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E279" s="62" t="str">
         <x:f>IF($D279="","",IF($D279="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15571,7 +15913,7 @@
       <x:c r="B280" s="33"/>
       <x:c r="C280" s="59"/>
       <x:c r="D280" s="52" t="str">
-        <x:f>IF($B280="","",IF(OR(RIGHT(TRIM($B280),2)="P276",RIGHT(TRIM($B280),2)="P277",RIGHT(TRIM($B280),2)="P278",RIGHT(TRIM($B280),2)="P279"),"PS","GS"))</x:f>
+        <x:f>IF($B280="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B280),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E280" s="62" t="str">
         <x:f>IF($D280="","",IF($D280="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15624,7 +15966,7 @@
       <x:c r="B281" s="33"/>
       <x:c r="C281" s="59"/>
       <x:c r="D281" s="52" t="str">
-        <x:f>IF($B281="","",IF(OR(RIGHT(TRIM($B281),2)="P277",RIGHT(TRIM($B281),2)="P278",RIGHT(TRIM($B281),2)="P279",RIGHT(TRIM($B281),2)="P280"),"PS","GS"))</x:f>
+        <x:f>IF($B281="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B281),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E281" s="62" t="str">
         <x:f>IF($D281="","",IF($D281="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15677,7 +16019,7 @@
       <x:c r="B282" s="33"/>
       <x:c r="C282" s="59"/>
       <x:c r="D282" s="52" t="str">
-        <x:f>IF($B282="","",IF(OR(RIGHT(TRIM($B282),2)="P278",RIGHT(TRIM($B282),2)="P279",RIGHT(TRIM($B282),2)="P280",RIGHT(TRIM($B282),2)="P281"),"PS","GS"))</x:f>
+        <x:f>IF($B282="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B282),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E282" s="62" t="str">
         <x:f>IF($D282="","",IF($D282="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15730,7 +16072,7 @@
       <x:c r="B283" s="33"/>
       <x:c r="C283" s="59"/>
       <x:c r="D283" s="52" t="str">
-        <x:f>IF($B283="","",IF(OR(RIGHT(TRIM($B283),2)="P279",RIGHT(TRIM($B283),2)="P280",RIGHT(TRIM($B283),2)="P281",RIGHT(TRIM($B283),2)="P282"),"PS","GS"))</x:f>
+        <x:f>IF($B283="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B283),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E283" s="62" t="str">
         <x:f>IF($D283="","",IF($D283="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15783,7 +16125,7 @@
       <x:c r="B284" s="33"/>
       <x:c r="C284" s="59"/>
       <x:c r="D284" s="52" t="str">
-        <x:f>IF($B284="","",IF(OR(RIGHT(TRIM($B284),2)="P280",RIGHT(TRIM($B284),2)="P281",RIGHT(TRIM($B284),2)="P282",RIGHT(TRIM($B284),2)="P283"),"PS","GS"))</x:f>
+        <x:f>IF($B284="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B284),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E284" s="62" t="str">
         <x:f>IF($D284="","",IF($D284="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15836,7 +16178,7 @@
       <x:c r="B285" s="33"/>
       <x:c r="C285" s="59"/>
       <x:c r="D285" s="52" t="str">
-        <x:f>IF($B285="","",IF(OR(RIGHT(TRIM($B285),2)="P281",RIGHT(TRIM($B285),2)="P282",RIGHT(TRIM($B285),2)="P283",RIGHT(TRIM($B285),2)="P284"),"PS","GS"))</x:f>
+        <x:f>IF($B285="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B285),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E285" s="62" t="str">
         <x:f>IF($D285="","",IF($D285="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15889,7 +16231,7 @@
       <x:c r="B286" s="33"/>
       <x:c r="C286" s="59"/>
       <x:c r="D286" s="52" t="str">
-        <x:f>IF($B286="","",IF(OR(RIGHT(TRIM($B286),2)="P282",RIGHT(TRIM($B286),2)="P283",RIGHT(TRIM($B286),2)="P284",RIGHT(TRIM($B286),2)="P285"),"PS","GS"))</x:f>
+        <x:f>IF($B286="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B286),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E286" s="62" t="str">
         <x:f>IF($D286="","",IF($D286="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15942,7 +16284,7 @@
       <x:c r="B287" s="33"/>
       <x:c r="C287" s="59"/>
       <x:c r="D287" s="52" t="str">
-        <x:f>IF($B287="","",IF(OR(RIGHT(TRIM($B287),2)="P283",RIGHT(TRIM($B287),2)="P284",RIGHT(TRIM($B287),2)="P285",RIGHT(TRIM($B287),2)="P286"),"PS","GS"))</x:f>
+        <x:f>IF($B287="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B287),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E287" s="62" t="str">
         <x:f>IF($D287="","",IF($D287="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -15995,7 +16337,7 @@
       <x:c r="B288" s="33"/>
       <x:c r="C288" s="59"/>
       <x:c r="D288" s="52" t="str">
-        <x:f>IF($B288="","",IF(OR(RIGHT(TRIM($B288),2)="P284",RIGHT(TRIM($B288),2)="P285",RIGHT(TRIM($B288),2)="P286",RIGHT(TRIM($B288),2)="P287"),"PS","GS"))</x:f>
+        <x:f>IF($B288="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B288),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E288" s="62" t="str">
         <x:f>IF($D288="","",IF($D288="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16048,7 +16390,7 @@
       <x:c r="B289" s="33"/>
       <x:c r="C289" s="59"/>
       <x:c r="D289" s="52" t="str">
-        <x:f>IF($B289="","",IF(OR(RIGHT(TRIM($B289),2)="P285",RIGHT(TRIM($B289),2)="P286",RIGHT(TRIM($B289),2)="P287",RIGHT(TRIM($B289),2)="P288"),"PS","GS"))</x:f>
+        <x:f>IF($B289="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B289),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E289" s="62" t="str">
         <x:f>IF($D289="","",IF($D289="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16101,7 +16443,7 @@
       <x:c r="B290" s="33"/>
       <x:c r="C290" s="59"/>
       <x:c r="D290" s="52" t="str">
-        <x:f>IF($B290="","",IF(OR(RIGHT(TRIM($B290),2)="P286",RIGHT(TRIM($B290),2)="P287",RIGHT(TRIM($B290),2)="P288",RIGHT(TRIM($B290),2)="P289"),"PS","GS"))</x:f>
+        <x:f>IF($B290="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B290),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E290" s="62" t="str">
         <x:f>IF($D290="","",IF($D290="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16154,7 +16496,7 @@
       <x:c r="B291" s="33"/>
       <x:c r="C291" s="59"/>
       <x:c r="D291" s="52" t="str">
-        <x:f>IF($B291="","",IF(OR(RIGHT(TRIM($B291),2)="P287",RIGHT(TRIM($B291),2)="P288",RIGHT(TRIM($B291),2)="P289",RIGHT(TRIM($B291),2)="P290"),"PS","GS"))</x:f>
+        <x:f>IF($B291="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B291),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E291" s="62" t="str">
         <x:f>IF($D291="","",IF($D291="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16207,7 +16549,7 @@
       <x:c r="B292" s="33"/>
       <x:c r="C292" s="59"/>
       <x:c r="D292" s="52" t="str">
-        <x:f>IF($B292="","",IF(OR(RIGHT(TRIM($B292),2)="P288",RIGHT(TRIM($B292),2)="P289",RIGHT(TRIM($B292),2)="P290",RIGHT(TRIM($B292),2)="P291"),"PS","GS"))</x:f>
+        <x:f>IF($B292="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B292),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E292" s="62" t="str">
         <x:f>IF($D292="","",IF($D292="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16260,7 +16602,7 @@
       <x:c r="B293" s="33"/>
       <x:c r="C293" s="59"/>
       <x:c r="D293" s="52" t="str">
-        <x:f>IF($B293="","",IF(OR(RIGHT(TRIM($B293),2)="P289",RIGHT(TRIM($B293),2)="P290",RIGHT(TRIM($B293),2)="P291",RIGHT(TRIM($B293),2)="P292"),"PS","GS"))</x:f>
+        <x:f>IF($B293="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B293),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E293" s="62" t="str">
         <x:f>IF($D293="","",IF($D293="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16313,7 +16655,7 @@
       <x:c r="B294" s="33"/>
       <x:c r="C294" s="59"/>
       <x:c r="D294" s="52" t="str">
-        <x:f>IF($B294="","",IF(OR(RIGHT(TRIM($B294),2)="P290",RIGHT(TRIM($B294),2)="P291",RIGHT(TRIM($B294),2)="P292",RIGHT(TRIM($B294),2)="P293"),"PS","GS"))</x:f>
+        <x:f>IF($B294="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B294),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E294" s="62" t="str">
         <x:f>IF($D294="","",IF($D294="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16366,7 +16708,7 @@
       <x:c r="B295" s="33"/>
       <x:c r="C295" s="59"/>
       <x:c r="D295" s="52" t="str">
-        <x:f>IF($B295="","",IF(OR(RIGHT(TRIM($B295),2)="P291",RIGHT(TRIM($B295),2)="P292",RIGHT(TRIM($B295),2)="P293",RIGHT(TRIM($B295),2)="P294"),"PS","GS"))</x:f>
+        <x:f>IF($B295="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B295),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E295" s="62" t="str">
         <x:f>IF($D295="","",IF($D295="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16419,7 +16761,7 @@
       <x:c r="B296" s="33"/>
       <x:c r="C296" s="59"/>
       <x:c r="D296" s="52" t="str">
-        <x:f>IF($B296="","",IF(OR(RIGHT(TRIM($B296),2)="P292",RIGHT(TRIM($B296),2)="P293",RIGHT(TRIM($B296),2)="P294",RIGHT(TRIM($B296),2)="P295"),"PS","GS"))</x:f>
+        <x:f>IF($B296="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B296),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E296" s="62" t="str">
         <x:f>IF($D296="","",IF($D296="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16472,7 +16814,7 @@
       <x:c r="B297" s="33"/>
       <x:c r="C297" s="59"/>
       <x:c r="D297" s="52" t="str">
-        <x:f>IF($B297="","",IF(OR(RIGHT(TRIM($B297),2)="P293",RIGHT(TRIM($B297),2)="P294",RIGHT(TRIM($B297),2)="P295",RIGHT(TRIM($B297),2)="P296"),"PS","GS"))</x:f>
+        <x:f>IF($B297="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B297),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E297" s="62" t="str">
         <x:f>IF($D297="","",IF($D297="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16525,7 +16867,7 @@
       <x:c r="B298" s="33"/>
       <x:c r="C298" s="59"/>
       <x:c r="D298" s="52" t="str">
-        <x:f>IF($B298="","",IF(OR(RIGHT(TRIM($B298),2)="P294",RIGHT(TRIM($B298),2)="P295",RIGHT(TRIM($B298),2)="P296",RIGHT(TRIM($B298),2)="P297"),"PS","GS"))</x:f>
+        <x:f>IF($B298="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B298),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E298" s="62" t="str">
         <x:f>IF($D298="","",IF($D298="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16578,7 +16920,7 @@
       <x:c r="B299" s="33"/>
       <x:c r="C299" s="59"/>
       <x:c r="D299" s="52" t="str">
-        <x:f>IF($B299="","",IF(OR(RIGHT(TRIM($B299),2)="P295",RIGHT(TRIM($B299),2)="P296",RIGHT(TRIM($B299),2)="P297",RIGHT(TRIM($B299),2)="P298"),"PS","GS"))</x:f>
+        <x:f>IF($B299="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B299),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E299" s="62" t="str">
         <x:f>IF($D299="","",IF($D299="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16631,7 +16973,7 @@
       <x:c r="B300" s="33"/>
       <x:c r="C300" s="59"/>
       <x:c r="D300" s="52" t="str">
-        <x:f>IF($B300="","",IF(OR(RIGHT(TRIM($B300),2)="P296",RIGHT(TRIM($B300),2)="P297",RIGHT(TRIM($B300),2)="P298",RIGHT(TRIM($B300),2)="P299"),"PS","GS"))</x:f>
+        <x:f>IF($B300="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B300),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E300" s="62" t="str">
         <x:f>IF($D300="","",IF($D300="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16684,7 +17026,7 @@
       <x:c r="B301" s="33"/>
       <x:c r="C301" s="59"/>
       <x:c r="D301" s="52" t="str">
-        <x:f>IF($B301="","",IF(OR(RIGHT(TRIM($B301),2)="P297",RIGHT(TRIM($B301),2)="P298",RIGHT(TRIM($B301),2)="P299",RIGHT(TRIM($B301),2)="P300"),"PS","GS"))</x:f>
+        <x:f>IF($B301="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B301),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E301" s="62" t="str">
         <x:f>IF($D301="","",IF($D301="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16737,7 +17079,7 @@
       <x:c r="B302" s="33"/>
       <x:c r="C302" s="59"/>
       <x:c r="D302" s="52" t="str">
-        <x:f>IF($B302="","",IF(OR(RIGHT(TRIM($B302),2)="P298",RIGHT(TRIM($B302),2)="P299",RIGHT(TRIM($B302),2)="P300",RIGHT(TRIM($B302),2)="P301"),"PS","GS"))</x:f>
+        <x:f>IF($B302="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B302),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E302" s="62" t="str">
         <x:f>IF($D302="","",IF($D302="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16790,7 +17132,7 @@
       <x:c r="B303" s="33"/>
       <x:c r="C303" s="59"/>
       <x:c r="D303" s="52" t="str">
-        <x:f>IF($B303="","",IF(OR(RIGHT(TRIM($B303),2)="P299",RIGHT(TRIM($B303),2)="P300",RIGHT(TRIM($B303),2)="P301",RIGHT(TRIM($B303),2)="P302"),"PS","GS"))</x:f>
+        <x:f>IF($B303="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B303),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E303" s="62" t="str">
         <x:f>IF($D303="","",IF($D303="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16843,7 +17185,7 @@
       <x:c r="B304" s="33"/>
       <x:c r="C304" s="59"/>
       <x:c r="D304" s="52" t="str">
-        <x:f>IF($B304="","",IF(OR(RIGHT(TRIM($B304),2)="P300",RIGHT(TRIM($B304),2)="P301",RIGHT(TRIM($B304),2)="P302",RIGHT(TRIM($B304),2)="P303"),"PS","GS"))</x:f>
+        <x:f>IF($B304="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B304),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E304" s="62" t="str">
         <x:f>IF($D304="","",IF($D304="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16896,7 +17238,7 @@
       <x:c r="B305" s="33"/>
       <x:c r="C305" s="59"/>
       <x:c r="D305" s="52" t="str">
-        <x:f>IF($B305="","",IF(OR(RIGHT(TRIM($B305),2)="P301",RIGHT(TRIM($B305),2)="P302",RIGHT(TRIM($B305),2)="P303",RIGHT(TRIM($B305),2)="P304"),"PS","GS"))</x:f>
+        <x:f>IF($B305="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B305),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E305" s="62" t="str">
         <x:f>IF($D305="","",IF($D305="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -16949,7 +17291,7 @@
       <x:c r="B306" s="33"/>
       <x:c r="C306" s="59"/>
       <x:c r="D306" s="52" t="str">
-        <x:f>IF($B306="","",IF(OR(RIGHT(TRIM($B306),2)="P302",RIGHT(TRIM($B306),2)="P303",RIGHT(TRIM($B306),2)="P304",RIGHT(TRIM($B306),2)="P305"),"PS","GS"))</x:f>
+        <x:f>IF($B306="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B306),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E306" s="62" t="str">
         <x:f>IF($D306="","",IF($D306="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17002,7 +17344,7 @@
       <x:c r="B307" s="33"/>
       <x:c r="C307" s="59"/>
       <x:c r="D307" s="52" t="str">
-        <x:f>IF($B307="","",IF(OR(RIGHT(TRIM($B307),2)="P303",RIGHT(TRIM($B307),2)="P304",RIGHT(TRIM($B307),2)="P305",RIGHT(TRIM($B307),2)="P306"),"PS","GS"))</x:f>
+        <x:f>IF($B307="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B307),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E307" s="62" t="str">
         <x:f>IF($D307="","",IF($D307="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17055,7 +17397,7 @@
       <x:c r="B308" s="33"/>
       <x:c r="C308" s="59"/>
       <x:c r="D308" s="52" t="str">
-        <x:f>IF($B308="","",IF(OR(RIGHT(TRIM($B308),2)="P304",RIGHT(TRIM($B308),2)="P305",RIGHT(TRIM($B308),2)="P306",RIGHT(TRIM($B308),2)="P307"),"PS","GS"))</x:f>
+        <x:f>IF($B308="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B308),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E308" s="62" t="str">
         <x:f>IF($D308="","",IF($D308="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17108,7 +17450,7 @@
       <x:c r="B309" s="33"/>
       <x:c r="C309" s="59"/>
       <x:c r="D309" s="52" t="str">
-        <x:f>IF($B309="","",IF(OR(RIGHT(TRIM($B309),2)="P305",RIGHT(TRIM($B309),2)="P306",RIGHT(TRIM($B309),2)="P307",RIGHT(TRIM($B309),2)="P308"),"PS","GS"))</x:f>
+        <x:f>IF($B309="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B309),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E309" s="62" t="str">
         <x:f>IF($D309="","",IF($D309="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17161,7 +17503,7 @@
       <x:c r="B310" s="33"/>
       <x:c r="C310" s="59"/>
       <x:c r="D310" s="52" t="str">
-        <x:f>IF($B310="","",IF(OR(RIGHT(TRIM($B310),2)="P306",RIGHT(TRIM($B310),2)="P307",RIGHT(TRIM($B310),2)="P308",RIGHT(TRIM($B310),2)="P309"),"PS","GS"))</x:f>
+        <x:f>IF($B310="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B310),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E310" s="62" t="str">
         <x:f>IF($D310="","",IF($D310="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17214,7 +17556,7 @@
       <x:c r="B311" s="33"/>
       <x:c r="C311" s="59"/>
       <x:c r="D311" s="52" t="str">
-        <x:f>IF($B311="","",IF(OR(RIGHT(TRIM($B311),2)="P307",RIGHT(TRIM($B311),2)="P308",RIGHT(TRIM($B311),2)="P309",RIGHT(TRIM($B311),2)="P310"),"PS","GS"))</x:f>
+        <x:f>IF($B311="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B311),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E311" s="62" t="str">
         <x:f>IF($D311="","",IF($D311="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17267,7 +17609,7 @@
       <x:c r="B312" s="33"/>
       <x:c r="C312" s="59"/>
       <x:c r="D312" s="52" t="str">
-        <x:f>IF($B312="","",IF(OR(RIGHT(TRIM($B312),2)="P308",RIGHT(TRIM($B312),2)="P309",RIGHT(TRIM($B312),2)="P310",RIGHT(TRIM($B312),2)="P311"),"PS","GS"))</x:f>
+        <x:f>IF($B312="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B312),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E312" s="62" t="str">
         <x:f>IF($D312="","",IF($D312="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17320,7 +17662,7 @@
       <x:c r="B313" s="33"/>
       <x:c r="C313" s="59"/>
       <x:c r="D313" s="52" t="str">
-        <x:f>IF($B313="","",IF(OR(RIGHT(TRIM($B313),2)="P309",RIGHT(TRIM($B313),2)="P310",RIGHT(TRIM($B313),2)="P311",RIGHT(TRIM($B313),2)="P312"),"PS","GS"))</x:f>
+        <x:f>IF($B313="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B313),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E313" s="62" t="str">
         <x:f>IF($D313="","",IF($D313="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17373,7 +17715,7 @@
       <x:c r="B314" s="33"/>
       <x:c r="C314" s="59"/>
       <x:c r="D314" s="52" t="str">
-        <x:f>IF($B314="","",IF(OR(RIGHT(TRIM($B314),2)="P310",RIGHT(TRIM($B314),2)="P311",RIGHT(TRIM($B314),2)="P312",RIGHT(TRIM($B314),2)="P313"),"PS","GS"))</x:f>
+        <x:f>IF($B314="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B314),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E314" s="62" t="str">
         <x:f>IF($D314="","",IF($D314="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17426,7 +17768,7 @@
       <x:c r="B315" s="33"/>
       <x:c r="C315" s="59"/>
       <x:c r="D315" s="52" t="str">
-        <x:f>IF($B315="","",IF(OR(RIGHT(TRIM($B315),2)="P311",RIGHT(TRIM($B315),2)="P312",RIGHT(TRIM($B315),2)="P313",RIGHT(TRIM($B315),2)="P314"),"PS","GS"))</x:f>
+        <x:f>IF($B315="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B315),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E315" s="62" t="str">
         <x:f>IF($D315="","",IF($D315="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17479,7 +17821,7 @@
       <x:c r="B316" s="33"/>
       <x:c r="C316" s="59"/>
       <x:c r="D316" s="52" t="str">
-        <x:f>IF($B316="","",IF(OR(RIGHT(TRIM($B316),2)="P312",RIGHT(TRIM($B316),2)="P313",RIGHT(TRIM($B316),2)="P314",RIGHT(TRIM($B316),2)="P315"),"PS","GS"))</x:f>
+        <x:f>IF($B316="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B316),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E316" s="62" t="str">
         <x:f>IF($D316="","",IF($D316="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17532,7 +17874,7 @@
       <x:c r="B317" s="33"/>
       <x:c r="C317" s="59"/>
       <x:c r="D317" s="52" t="str">
-        <x:f>IF($B317="","",IF(OR(RIGHT(TRIM($B317),2)="P313",RIGHT(TRIM($B317),2)="P314",RIGHT(TRIM($B317),2)="P315",RIGHT(TRIM($B317),2)="P316"),"PS","GS"))</x:f>
+        <x:f>IF($B317="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B317),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E317" s="62" t="str">
         <x:f>IF($D317="","",IF($D317="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17585,7 +17927,7 @@
       <x:c r="B318" s="33"/>
       <x:c r="C318" s="59"/>
       <x:c r="D318" s="52" t="str">
-        <x:f>IF($B318="","",IF(OR(RIGHT(TRIM($B318),2)="P314",RIGHT(TRIM($B318),2)="P315",RIGHT(TRIM($B318),2)="P316",RIGHT(TRIM($B318),2)="P317"),"PS","GS"))</x:f>
+        <x:f>IF($B318="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B318),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E318" s="62" t="str">
         <x:f>IF($D318="","",IF($D318="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17638,7 +17980,7 @@
       <x:c r="B319" s="33"/>
       <x:c r="C319" s="59"/>
       <x:c r="D319" s="52" t="str">
-        <x:f>IF($B319="","",IF(OR(RIGHT(TRIM($B319),2)="P315",RIGHT(TRIM($B319),2)="P316",RIGHT(TRIM($B319),2)="P317",RIGHT(TRIM($B319),2)="P318"),"PS","GS"))</x:f>
+        <x:f>IF($B319="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B319),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E319" s="62" t="str">
         <x:f>IF($D319="","",IF($D319="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17691,7 +18033,7 @@
       <x:c r="B320" s="33"/>
       <x:c r="C320" s="59"/>
       <x:c r="D320" s="52" t="str">
-        <x:f>IF($B320="","",IF(OR(RIGHT(TRIM($B320),2)="P316",RIGHT(TRIM($B320),2)="P317",RIGHT(TRIM($B320),2)="P318",RIGHT(TRIM($B320),2)="P319"),"PS","GS"))</x:f>
+        <x:f>IF($B320="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B320),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E320" s="62" t="str">
         <x:f>IF($D320="","",IF($D320="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17744,7 +18086,7 @@
       <x:c r="B321" s="33"/>
       <x:c r="C321" s="59"/>
       <x:c r="D321" s="52" t="str">
-        <x:f>IF($B321="","",IF(OR(RIGHT(TRIM($B321),2)="P317",RIGHT(TRIM($B321),2)="P318",RIGHT(TRIM($B321),2)="P319",RIGHT(TRIM($B321),2)="P320"),"PS","GS"))</x:f>
+        <x:f>IF($B321="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B321),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E321" s="62" t="str">
         <x:f>IF($D321="","",IF($D321="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17797,7 +18139,7 @@
       <x:c r="B322" s="33"/>
       <x:c r="C322" s="59"/>
       <x:c r="D322" s="52" t="str">
-        <x:f>IF($B322="","",IF(OR(RIGHT(TRIM($B322),2)="P318",RIGHT(TRIM($B322),2)="P319",RIGHT(TRIM($B322),2)="P320",RIGHT(TRIM($B322),2)="P321"),"PS","GS"))</x:f>
+        <x:f>IF($B322="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B322),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E322" s="62" t="str">
         <x:f>IF($D322="","",IF($D322="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17850,7 +18192,7 @@
       <x:c r="B323" s="33"/>
       <x:c r="C323" s="59"/>
       <x:c r="D323" s="52" t="str">
-        <x:f>IF($B323="","",IF(OR(RIGHT(TRIM($B323),2)="P319",RIGHT(TRIM($B323),2)="P320",RIGHT(TRIM($B323),2)="P321",RIGHT(TRIM($B323),2)="P322"),"PS","GS"))</x:f>
+        <x:f>IF($B323="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B323),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E323" s="62" t="str">
         <x:f>IF($D323="","",IF($D323="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17903,7 +18245,7 @@
       <x:c r="B324" s="33"/>
       <x:c r="C324" s="59"/>
       <x:c r="D324" s="52" t="str">
-        <x:f>IF($B324="","",IF(OR(RIGHT(TRIM($B324),2)="P320",RIGHT(TRIM($B324),2)="P321",RIGHT(TRIM($B324),2)="P322",RIGHT(TRIM($B324),2)="P323"),"PS","GS"))</x:f>
+        <x:f>IF($B324="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B324),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E324" s="62" t="str">
         <x:f>IF($D324="","",IF($D324="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -17956,7 +18298,7 @@
       <x:c r="B325" s="33"/>
       <x:c r="C325" s="59"/>
       <x:c r="D325" s="52" t="str">
-        <x:f>IF($B325="","",IF(OR(RIGHT(TRIM($B325),2)="P321",RIGHT(TRIM($B325),2)="P322",RIGHT(TRIM($B325),2)="P323",RIGHT(TRIM($B325),2)="P324"),"PS","GS"))</x:f>
+        <x:f>IF($B325="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B325),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E325" s="62" t="str">
         <x:f>IF($D325="","",IF($D325="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18009,7 +18351,7 @@
       <x:c r="B326" s="33"/>
       <x:c r="C326" s="59"/>
       <x:c r="D326" s="52" t="str">
-        <x:f>IF($B326="","",IF(OR(RIGHT(TRIM($B326),2)="P322",RIGHT(TRIM($B326),2)="P323",RIGHT(TRIM($B326),2)="P324",RIGHT(TRIM($B326),2)="P325"),"PS","GS"))</x:f>
+        <x:f>IF($B326="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B326),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E326" s="62" t="str">
         <x:f>IF($D326="","",IF($D326="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18062,7 +18404,7 @@
       <x:c r="B327" s="33"/>
       <x:c r="C327" s="59"/>
       <x:c r="D327" s="52" t="str">
-        <x:f>IF($B327="","",IF(OR(RIGHT(TRIM($B327),2)="P323",RIGHT(TRIM($B327),2)="P324",RIGHT(TRIM($B327),2)="P325",RIGHT(TRIM($B327),2)="P326"),"PS","GS"))</x:f>
+        <x:f>IF($B327="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B327),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E327" s="62" t="str">
         <x:f>IF($D327="","",IF($D327="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18115,7 +18457,7 @@
       <x:c r="B328" s="33"/>
       <x:c r="C328" s="59"/>
       <x:c r="D328" s="52" t="str">
-        <x:f>IF($B328="","",IF(OR(RIGHT(TRIM($B328),2)="P324",RIGHT(TRIM($B328),2)="P325",RIGHT(TRIM($B328),2)="P326",RIGHT(TRIM($B328),2)="P327"),"PS","GS"))</x:f>
+        <x:f>IF($B328="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B328),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E328" s="62" t="str">
         <x:f>IF($D328="","",IF($D328="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18168,7 +18510,7 @@
       <x:c r="B329" s="33"/>
       <x:c r="C329" s="59"/>
       <x:c r="D329" s="52" t="str">
-        <x:f>IF($B329="","",IF(OR(RIGHT(TRIM($B329),2)="P325",RIGHT(TRIM($B329),2)="P326",RIGHT(TRIM($B329),2)="P327",RIGHT(TRIM($B329),2)="P328"),"PS","GS"))</x:f>
+        <x:f>IF($B329="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B329),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E329" s="62" t="str">
         <x:f>IF($D329="","",IF($D329="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18221,7 +18563,7 @@
       <x:c r="B330" s="33"/>
       <x:c r="C330" s="59"/>
       <x:c r="D330" s="52" t="str">
-        <x:f>IF($B330="","",IF(OR(RIGHT(TRIM($B330),2)="P326",RIGHT(TRIM($B330),2)="P327",RIGHT(TRIM($B330),2)="P328",RIGHT(TRIM($B330),2)="P329"),"PS","GS"))</x:f>
+        <x:f>IF($B330="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B330),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E330" s="62" t="str">
         <x:f>IF($D330="","",IF($D330="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18274,7 +18616,7 @@
       <x:c r="B331" s="33"/>
       <x:c r="C331" s="59"/>
       <x:c r="D331" s="52" t="str">
-        <x:f>IF($B331="","",IF(OR(RIGHT(TRIM($B331),2)="P327",RIGHT(TRIM($B331),2)="P328",RIGHT(TRIM($B331),2)="P329",RIGHT(TRIM($B331),2)="P330"),"PS","GS"))</x:f>
+        <x:f>IF($B331="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B331),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E331" s="62" t="str">
         <x:f>IF($D331="","",IF($D331="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18327,7 +18669,7 @@
       <x:c r="B332" s="33"/>
       <x:c r="C332" s="59"/>
       <x:c r="D332" s="52" t="str">
-        <x:f>IF($B332="","",IF(OR(RIGHT(TRIM($B332),2)="P328",RIGHT(TRIM($B332),2)="P329",RIGHT(TRIM($B332),2)="P330",RIGHT(TRIM($B332),2)="P331"),"PS","GS"))</x:f>
+        <x:f>IF($B332="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B332),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E332" s="62" t="str">
         <x:f>IF($D332="","",IF($D332="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18380,7 +18722,7 @@
       <x:c r="B333" s="33"/>
       <x:c r="C333" s="59"/>
       <x:c r="D333" s="52" t="str">
-        <x:f>IF($B333="","",IF(OR(RIGHT(TRIM($B333),2)="P329",RIGHT(TRIM($B333),2)="P330",RIGHT(TRIM($B333),2)="P331",RIGHT(TRIM($B333),2)="P332"),"PS","GS"))</x:f>
+        <x:f>IF($B333="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B333),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E333" s="62" t="str">
         <x:f>IF($D333="","",IF($D333="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18433,7 +18775,7 @@
       <x:c r="B334" s="33"/>
       <x:c r="C334" s="59"/>
       <x:c r="D334" s="52" t="str">
-        <x:f>IF($B334="","",IF(OR(RIGHT(TRIM($B334),2)="P330",RIGHT(TRIM($B334),2)="P331",RIGHT(TRIM($B334),2)="P332",RIGHT(TRIM($B334),2)="P333"),"PS","GS"))</x:f>
+        <x:f>IF($B334="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B334),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E334" s="62" t="str">
         <x:f>IF($D334="","",IF($D334="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18486,7 +18828,7 @@
       <x:c r="B335" s="33"/>
       <x:c r="C335" s="59"/>
       <x:c r="D335" s="52" t="str">
-        <x:f>IF($B335="","",IF(OR(RIGHT(TRIM($B335),2)="P331",RIGHT(TRIM($B335),2)="P332",RIGHT(TRIM($B335),2)="P333",RIGHT(TRIM($B335),2)="P334"),"PS","GS"))</x:f>
+        <x:f>IF($B335="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B335),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E335" s="62" t="str">
         <x:f>IF($D335="","",IF($D335="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18539,7 +18881,7 @@
       <x:c r="B336" s="33"/>
       <x:c r="C336" s="59"/>
       <x:c r="D336" s="52" t="str">
-        <x:f>IF($B336="","",IF(OR(RIGHT(TRIM($B336),2)="P332",RIGHT(TRIM($B336),2)="P333",RIGHT(TRIM($B336),2)="P334",RIGHT(TRIM($B336),2)="P335"),"PS","GS"))</x:f>
+        <x:f>IF($B336="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B336),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E336" s="62" t="str">
         <x:f>IF($D336="","",IF($D336="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18592,7 +18934,7 @@
       <x:c r="B337" s="33"/>
       <x:c r="C337" s="59"/>
       <x:c r="D337" s="52" t="str">
-        <x:f>IF($B337="","",IF(OR(RIGHT(TRIM($B337),2)="P333",RIGHT(TRIM($B337),2)="P334",RIGHT(TRIM($B337),2)="P335",RIGHT(TRIM($B337),2)="P336"),"PS","GS"))</x:f>
+        <x:f>IF($B337="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B337),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E337" s="62" t="str">
         <x:f>IF($D337="","",IF($D337="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18645,7 +18987,7 @@
       <x:c r="B338" s="33"/>
       <x:c r="C338" s="59"/>
       <x:c r="D338" s="52" t="str">
-        <x:f>IF($B338="","",IF(OR(RIGHT(TRIM($B338),2)="P334",RIGHT(TRIM($B338),2)="P335",RIGHT(TRIM($B338),2)="P336",RIGHT(TRIM($B338),2)="P337"),"PS","GS"))</x:f>
+        <x:f>IF($B338="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B338),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E338" s="62" t="str">
         <x:f>IF($D338="","",IF($D338="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18698,7 +19040,7 @@
       <x:c r="B339" s="33"/>
       <x:c r="C339" s="59"/>
       <x:c r="D339" s="52" t="str">
-        <x:f>IF($B339="","",IF(OR(RIGHT(TRIM($B339),2)="P335",RIGHT(TRIM($B339),2)="P336",RIGHT(TRIM($B339),2)="P337",RIGHT(TRIM($B339),2)="P338"),"PS","GS"))</x:f>
+        <x:f>IF($B339="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B339),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E339" s="62" t="str">
         <x:f>IF($D339="","",IF($D339="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18751,7 +19093,7 @@
       <x:c r="B340" s="33"/>
       <x:c r="C340" s="59"/>
       <x:c r="D340" s="52" t="str">
-        <x:f>IF($B340="","",IF(OR(RIGHT(TRIM($B340),2)="P336",RIGHT(TRIM($B340),2)="P337",RIGHT(TRIM($B340),2)="P338",RIGHT(TRIM($B340),2)="P339"),"PS","GS"))</x:f>
+        <x:f>IF($B340="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B340),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E340" s="62" t="str">
         <x:f>IF($D340="","",IF($D340="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18804,7 +19146,7 @@
       <x:c r="B341" s="33"/>
       <x:c r="C341" s="59"/>
       <x:c r="D341" s="52" t="str">
-        <x:f>IF($B341="","",IF(OR(RIGHT(TRIM($B341),2)="P337",RIGHT(TRIM($B341),2)="P338",RIGHT(TRIM($B341),2)="P339",RIGHT(TRIM($B341),2)="P340"),"PS","GS"))</x:f>
+        <x:f>IF($B341="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B341),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E341" s="62" t="str">
         <x:f>IF($D341="","",IF($D341="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18857,7 +19199,7 @@
       <x:c r="B342" s="33"/>
       <x:c r="C342" s="59"/>
       <x:c r="D342" s="52" t="str">
-        <x:f>IF($B342="","",IF(OR(RIGHT(TRIM($B342),2)="P338",RIGHT(TRIM($B342),2)="P339",RIGHT(TRIM($B342),2)="P340",RIGHT(TRIM($B342),2)="P341"),"PS","GS"))</x:f>
+        <x:f>IF($B342="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B342),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E342" s="62" t="str">
         <x:f>IF($D342="","",IF($D342="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18910,7 +19252,7 @@
       <x:c r="B343" s="33"/>
       <x:c r="C343" s="59"/>
       <x:c r="D343" s="52" t="str">
-        <x:f>IF($B343="","",IF(OR(RIGHT(TRIM($B343),2)="P339",RIGHT(TRIM($B343),2)="P340",RIGHT(TRIM($B343),2)="P341",RIGHT(TRIM($B343),2)="P342"),"PS","GS"))</x:f>
+        <x:f>IF($B343="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B343),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E343" s="62" t="str">
         <x:f>IF($D343="","",IF($D343="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -18963,7 +19305,7 @@
       <x:c r="B344" s="33"/>
       <x:c r="C344" s="59"/>
       <x:c r="D344" s="52" t="str">
-        <x:f>IF($B344="","",IF(OR(RIGHT(TRIM($B344),2)="P340",RIGHT(TRIM($B344),2)="P341",RIGHT(TRIM($B344),2)="P342",RIGHT(TRIM($B344),2)="P343"),"PS","GS"))</x:f>
+        <x:f>IF($B344="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B344),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E344" s="62" t="str">
         <x:f>IF($D344="","",IF($D344="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19016,7 +19358,7 @@
       <x:c r="B345" s="33"/>
       <x:c r="C345" s="59"/>
       <x:c r="D345" s="52" t="str">
-        <x:f>IF($B345="","",IF(OR(RIGHT(TRIM($B345),2)="P341",RIGHT(TRIM($B345),2)="P342",RIGHT(TRIM($B345),2)="P343",RIGHT(TRIM($B345),2)="P344"),"PS","GS"))</x:f>
+        <x:f>IF($B345="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B345),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E345" s="62" t="str">
         <x:f>IF($D345="","",IF($D345="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19069,7 +19411,7 @@
       <x:c r="B346" s="33"/>
       <x:c r="C346" s="59"/>
       <x:c r="D346" s="52" t="str">
-        <x:f>IF($B346="","",IF(OR(RIGHT(TRIM($B346),2)="P342",RIGHT(TRIM($B346),2)="P343",RIGHT(TRIM($B346),2)="P344",RIGHT(TRIM($B346),2)="P345"),"PS","GS"))</x:f>
+        <x:f>IF($B346="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B346),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E346" s="62" t="str">
         <x:f>IF($D346="","",IF($D346="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19122,7 +19464,7 @@
       <x:c r="B347" s="33"/>
       <x:c r="C347" s="59"/>
       <x:c r="D347" s="52" t="str">
-        <x:f>IF($B347="","",IF(OR(RIGHT(TRIM($B347),2)="P343",RIGHT(TRIM($B347),2)="P344",RIGHT(TRIM($B347),2)="P345",RIGHT(TRIM($B347),2)="P346"),"PS","GS"))</x:f>
+        <x:f>IF($B347="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B347),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E347" s="62" t="str">
         <x:f>IF($D347="","",IF($D347="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19175,7 +19517,7 @@
       <x:c r="B348" s="33"/>
       <x:c r="C348" s="59"/>
       <x:c r="D348" s="52" t="str">
-        <x:f>IF($B348="","",IF(OR(RIGHT(TRIM($B348),2)="P344",RIGHT(TRIM($B348),2)="P345",RIGHT(TRIM($B348),2)="P346",RIGHT(TRIM($B348),2)="P347"),"PS","GS"))</x:f>
+        <x:f>IF($B348="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B348),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E348" s="62" t="str">
         <x:f>IF($D348="","",IF($D348="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19228,7 +19570,7 @@
       <x:c r="B349" s="33"/>
       <x:c r="C349" s="59"/>
       <x:c r="D349" s="52" t="str">
-        <x:f>IF($B349="","",IF(OR(RIGHT(TRIM($B349),2)="P345",RIGHT(TRIM($B349),2)="P346",RIGHT(TRIM($B349),2)="P347",RIGHT(TRIM($B349),2)="P348"),"PS","GS"))</x:f>
+        <x:f>IF($B349="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B349),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E349" s="62" t="str">
         <x:f>IF($D349="","",IF($D349="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19281,7 +19623,7 @@
       <x:c r="B350" s="33"/>
       <x:c r="C350" s="59"/>
       <x:c r="D350" s="52" t="str">
-        <x:f>IF($B350="","",IF(OR(RIGHT(TRIM($B350),2)="P346",RIGHT(TRIM($B350),2)="P347",RIGHT(TRIM($B350),2)="P348",RIGHT(TRIM($B350),2)="P349"),"PS","GS"))</x:f>
+        <x:f>IF($B350="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B350),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E350" s="62" t="str">
         <x:f>IF($D350="","",IF($D350="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19334,7 +19676,7 @@
       <x:c r="B351" s="33"/>
       <x:c r="C351" s="59"/>
       <x:c r="D351" s="52" t="str">
-        <x:f>IF($B351="","",IF(OR(RIGHT(TRIM($B351),2)="P347",RIGHT(TRIM($B351),2)="P348",RIGHT(TRIM($B351),2)="P349",RIGHT(TRIM($B351),2)="P350"),"PS","GS"))</x:f>
+        <x:f>IF($B351="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B351),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E351" s="62" t="str">
         <x:f>IF($D351="","",IF($D351="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19387,7 +19729,7 @@
       <x:c r="B352" s="33"/>
       <x:c r="C352" s="59"/>
       <x:c r="D352" s="52" t="str">
-        <x:f>IF($B352="","",IF(OR(RIGHT(TRIM($B352),2)="P348",RIGHT(TRIM($B352),2)="P349",RIGHT(TRIM($B352),2)="P350",RIGHT(TRIM($B352),2)="P351"),"PS","GS"))</x:f>
+        <x:f>IF($B352="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B352),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E352" s="62" t="str">
         <x:f>IF($D352="","",IF($D352="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19440,7 +19782,7 @@
       <x:c r="B353" s="33"/>
       <x:c r="C353" s="59"/>
       <x:c r="D353" s="52" t="str">
-        <x:f>IF($B353="","",IF(OR(RIGHT(TRIM($B353),2)="P349",RIGHT(TRIM($B353),2)="P350",RIGHT(TRIM($B353),2)="P351",RIGHT(TRIM($B353),2)="P352"),"PS","GS"))</x:f>
+        <x:f>IF($B353="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B353),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E353" s="62" t="str">
         <x:f>IF($D353="","",IF($D353="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19493,7 +19835,7 @@
       <x:c r="B354" s="36"/>
       <x:c r="C354" s="60"/>
       <x:c r="D354" s="55" t="str">
-        <x:f>IF($B354="","",IF(OR(RIGHT(TRIM($B354),2)="P350",RIGHT(TRIM($B354),2)="P351",RIGHT(TRIM($B354),2)="P352",RIGHT(TRIM($B354),2)="P353"),"PS","GS"))</x:f>
+        <x:f>IF($B354="","",IF(LEFT(UPPER(TRIM(RIGHT(SUBSTITUTE(SUBSTITUTE(CLEAN($B354),CHAR(160)," "),"-",REPT(" ",100)),100))),1)="P","PS","GS"))</x:f>
       </x:c>
       <x:c r="E354" s="63" t="str">
         <x:f>IF($D354="","",IF($D354="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
@@ -19554,7 +19896,7 @@
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B5:B354">
-      <x:formula1>'Data'!$A$2:$A$113</x:formula1>
+      <x:formula1>$U$2:$U$113</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="decimal" operator="greaterThan" sqref="C5:C354">
       <x:formula1>0</x:formula1>
@@ -19562,7 +19904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8c3a15225444d9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bd3bd83e10947a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add missing Merit Excel job option
</commit_message>
<xml_diff>
--- a/downloads/Merit_2026_Employee_Bulk_Calculator_350_exact.xlsx
+++ b/downloads/Merit_2026_Employee_Bulk_Calculator_350_exact.xlsx
@@ -1017,7 +1017,7 @@
         <x:f>IF($D5="","",IF($D5="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F5" s="50" t="str">
-        <x:f>IF($B5="","",IFERROR(VLOOKUP($B5,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B5="","",IFERROR(VLOOKUP($B5,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G5" s="64" t="str">
         <x:f>IF($F5="","",IFERROR(VLOOKUP($F5,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1073,7 +1073,7 @@
         <x:f>IF($D6="","",IF($D6="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F6" s="53" t="str">
-        <x:f>IF($B6="","",IFERROR(VLOOKUP($B6,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B6="","",IFERROR(VLOOKUP($B6,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G6" s="65" t="str">
         <x:f>IF($F6="","",IFERROR(VLOOKUP($F6,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1129,7 +1129,7 @@
         <x:f>IF($D7="","",IF($D7="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F7" s="53" t="str">
-        <x:f>IF($B7="","",IFERROR(VLOOKUP($B7,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B7="","",IFERROR(VLOOKUP($B7,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G7" s="65" t="str">
         <x:f>IF($F7="","",IFERROR(VLOOKUP($F7,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1185,7 +1185,7 @@
         <x:f>IF($D8="","",IF($D8="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F8" s="53" t="str">
-        <x:f>IF($B8="","",IFERROR(VLOOKUP($B8,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B8="","",IFERROR(VLOOKUP($B8,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G8" s="65" t="str">
         <x:f>IF($F8="","",IFERROR(VLOOKUP($F8,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1241,7 +1241,7 @@
         <x:f>IF($D9="","",IF($D9="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F9" s="53" t="str">
-        <x:f>IF($B9="","",IFERROR(VLOOKUP($B9,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B9="","",IFERROR(VLOOKUP($B9,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G9" s="65" t="str">
         <x:f>IF($F9="","",IFERROR(VLOOKUP($F9,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1297,7 +1297,7 @@
         <x:f>IF($D10="","",IF($D10="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F10" s="53" t="str">
-        <x:f>IF($B10="","",IFERROR(VLOOKUP($B10,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B10="","",IFERROR(VLOOKUP($B10,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G10" s="65" t="str">
         <x:f>IF($F10="","",IFERROR(VLOOKUP($F10,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1353,7 +1353,7 @@
         <x:f>IF($D11="","",IF($D11="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F11" s="53" t="str">
-        <x:f>IF($B11="","",IFERROR(VLOOKUP($B11,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B11="","",IFERROR(VLOOKUP($B11,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G11" s="65" t="str">
         <x:f>IF($F11="","",IFERROR(VLOOKUP($F11,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1409,7 +1409,7 @@
         <x:f>IF($D12="","",IF($D12="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F12" s="53" t="str">
-        <x:f>IF($B12="","",IFERROR(VLOOKUP($B12,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B12="","",IFERROR(VLOOKUP($B12,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G12" s="65" t="str">
         <x:f>IF($F12="","",IFERROR(VLOOKUP($F12,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1465,7 +1465,7 @@
         <x:f>IF($D13="","",IF($D13="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F13" s="53" t="str">
-        <x:f>IF($B13="","",IFERROR(VLOOKUP($B13,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B13="","",IFERROR(VLOOKUP($B13,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G13" s="65" t="str">
         <x:f>IF($F13="","",IFERROR(VLOOKUP($F13,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1521,7 +1521,7 @@
         <x:f>IF($D14="","",IF($D14="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F14" s="53" t="str">
-        <x:f>IF($B14="","",IFERROR(VLOOKUP($B14,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B14="","",IFERROR(VLOOKUP($B14,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G14" s="65" t="str">
         <x:f>IF($F14="","",IFERROR(VLOOKUP($F14,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1577,7 +1577,7 @@
         <x:f>IF($D15="","",IF($D15="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F15" s="53" t="str">
-        <x:f>IF($B15="","",IFERROR(VLOOKUP($B15,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B15="","",IFERROR(VLOOKUP($B15,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G15" s="65" t="str">
         <x:f>IF($F15="","",IFERROR(VLOOKUP($F15,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1633,7 +1633,7 @@
         <x:f>IF($D16="","",IF($D16="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F16" s="53" t="str">
-        <x:f>IF($B16="","",IFERROR(VLOOKUP($B16,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B16="","",IFERROR(VLOOKUP($B16,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G16" s="65" t="str">
         <x:f>IF($F16="","",IFERROR(VLOOKUP($F16,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1689,7 +1689,7 @@
         <x:f>IF($D17="","",IF($D17="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F17" s="53" t="str">
-        <x:f>IF($B17="","",IFERROR(VLOOKUP($B17,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B17="","",IFERROR(VLOOKUP($B17,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G17" s="65" t="str">
         <x:f>IF($F17="","",IFERROR(VLOOKUP($F17,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1745,7 +1745,7 @@
         <x:f>IF($D18="","",IF($D18="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F18" s="53" t="str">
-        <x:f>IF($B18="","",IFERROR(VLOOKUP($B18,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B18="","",IFERROR(VLOOKUP($B18,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G18" s="65" t="str">
         <x:f>IF($F18="","",IFERROR(VLOOKUP($F18,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1801,7 +1801,7 @@
         <x:f>IF($D19="","",IF($D19="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F19" s="53" t="str">
-        <x:f>IF($B19="","",IFERROR(VLOOKUP($B19,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B19="","",IFERROR(VLOOKUP($B19,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G19" s="65" t="str">
         <x:f>IF($F19="","",IFERROR(VLOOKUP($F19,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1857,7 +1857,7 @@
         <x:f>IF($D20="","",IF($D20="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F20" s="53" t="str">
-        <x:f>IF($B20="","",IFERROR(VLOOKUP($B20,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B20="","",IFERROR(VLOOKUP($B20,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G20" s="65" t="str">
         <x:f>IF($F20="","",IFERROR(VLOOKUP($F20,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1913,7 +1913,7 @@
         <x:f>IF($D21="","",IF($D21="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F21" s="53" t="str">
-        <x:f>IF($B21="","",IFERROR(VLOOKUP($B21,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B21="","",IFERROR(VLOOKUP($B21,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G21" s="65" t="str">
         <x:f>IF($F21="","",IFERROR(VLOOKUP($F21,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -1969,7 +1969,7 @@
         <x:f>IF($D22="","",IF($D22="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F22" s="53" t="str">
-        <x:f>IF($B22="","",IFERROR(VLOOKUP($B22,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B22="","",IFERROR(VLOOKUP($B22,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G22" s="65" t="str">
         <x:f>IF($F22="","",IFERROR(VLOOKUP($F22,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2025,7 +2025,7 @@
         <x:f>IF($D23="","",IF($D23="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F23" s="53" t="str">
-        <x:f>IF($B23="","",IFERROR(VLOOKUP($B23,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B23="","",IFERROR(VLOOKUP($B23,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G23" s="65" t="str">
         <x:f>IF($F23="","",IFERROR(VLOOKUP($F23,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2081,7 +2081,7 @@
         <x:f>IF($D24="","",IF($D24="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F24" s="53" t="str">
-        <x:f>IF($B24="","",IFERROR(VLOOKUP($B24,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B24="","",IFERROR(VLOOKUP($B24,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G24" s="65" t="str">
         <x:f>IF($F24="","",IFERROR(VLOOKUP($F24,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2137,7 +2137,7 @@
         <x:f>IF($D25="","",IF($D25="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F25" s="53" t="str">
-        <x:f>IF($B25="","",IFERROR(VLOOKUP($B25,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B25="","",IFERROR(VLOOKUP($B25,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G25" s="65" t="str">
         <x:f>IF($F25="","",IFERROR(VLOOKUP($F25,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2193,7 +2193,7 @@
         <x:f>IF($D26="","",IF($D26="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F26" s="53" t="str">
-        <x:f>IF($B26="","",IFERROR(VLOOKUP($B26,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B26="","",IFERROR(VLOOKUP($B26,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G26" s="65" t="str">
         <x:f>IF($F26="","",IFERROR(VLOOKUP($F26,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2249,7 +2249,7 @@
         <x:f>IF($D27="","",IF($D27="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F27" s="53" t="str">
-        <x:f>IF($B27="","",IFERROR(VLOOKUP($B27,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B27="","",IFERROR(VLOOKUP($B27,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G27" s="65" t="str">
         <x:f>IF($F27="","",IFERROR(VLOOKUP($F27,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2305,7 +2305,7 @@
         <x:f>IF($D28="","",IF($D28="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F28" s="53" t="str">
-        <x:f>IF($B28="","",IFERROR(VLOOKUP($B28,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B28="","",IFERROR(VLOOKUP($B28,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G28" s="65" t="str">
         <x:f>IF($F28="","",IFERROR(VLOOKUP($F28,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2361,7 +2361,7 @@
         <x:f>IF($D29="","",IF($D29="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F29" s="53" t="str">
-        <x:f>IF($B29="","",IFERROR(VLOOKUP($B29,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B29="","",IFERROR(VLOOKUP($B29,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G29" s="65" t="str">
         <x:f>IF($F29="","",IFERROR(VLOOKUP($F29,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2417,7 +2417,7 @@
         <x:f>IF($D30="","",IF($D30="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F30" s="53" t="str">
-        <x:f>IF($B30="","",IFERROR(VLOOKUP($B30,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B30="","",IFERROR(VLOOKUP($B30,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G30" s="65" t="str">
         <x:f>IF($F30="","",IFERROR(VLOOKUP($F30,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2473,7 +2473,7 @@
         <x:f>IF($D31="","",IF($D31="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F31" s="53" t="str">
-        <x:f>IF($B31="","",IFERROR(VLOOKUP($B31,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B31="","",IFERROR(VLOOKUP($B31,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G31" s="65" t="str">
         <x:f>IF($F31="","",IFERROR(VLOOKUP($F31,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2529,7 +2529,7 @@
         <x:f>IF($D32="","",IF($D32="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F32" s="53" t="str">
-        <x:f>IF($B32="","",IFERROR(VLOOKUP($B32,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B32="","",IFERROR(VLOOKUP($B32,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G32" s="65" t="str">
         <x:f>IF($F32="","",IFERROR(VLOOKUP($F32,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2585,7 +2585,7 @@
         <x:f>IF($D33="","",IF($D33="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F33" s="53" t="str">
-        <x:f>IF($B33="","",IFERROR(VLOOKUP($B33,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B33="","",IFERROR(VLOOKUP($B33,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G33" s="65" t="str">
         <x:f>IF($F33="","",IFERROR(VLOOKUP($F33,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2641,7 +2641,7 @@
         <x:f>IF($D34="","",IF($D34="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F34" s="53" t="str">
-        <x:f>IF($B34="","",IFERROR(VLOOKUP($B34,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B34="","",IFERROR(VLOOKUP($B34,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G34" s="65" t="str">
         <x:f>IF($F34="","",IFERROR(VLOOKUP($F34,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2697,7 +2697,7 @@
         <x:f>IF($D35="","",IF($D35="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F35" s="53" t="str">
-        <x:f>IF($B35="","",IFERROR(VLOOKUP($B35,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B35="","",IFERROR(VLOOKUP($B35,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G35" s="65" t="str">
         <x:f>IF($F35="","",IFERROR(VLOOKUP($F35,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2753,7 +2753,7 @@
         <x:f>IF($D36="","",IF($D36="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F36" s="53" t="str">
-        <x:f>IF($B36="","",IFERROR(VLOOKUP($B36,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B36="","",IFERROR(VLOOKUP($B36,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G36" s="65" t="str">
         <x:f>IF($F36="","",IFERROR(VLOOKUP($F36,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2809,7 +2809,7 @@
         <x:f>IF($D37="","",IF($D37="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F37" s="53" t="str">
-        <x:f>IF($B37="","",IFERROR(VLOOKUP($B37,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B37="","",IFERROR(VLOOKUP($B37,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G37" s="65" t="str">
         <x:f>IF($F37="","",IFERROR(VLOOKUP($F37,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2865,7 +2865,7 @@
         <x:f>IF($D38="","",IF($D38="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F38" s="53" t="str">
-        <x:f>IF($B38="","",IFERROR(VLOOKUP($B38,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B38="","",IFERROR(VLOOKUP($B38,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G38" s="65" t="str">
         <x:f>IF($F38="","",IFERROR(VLOOKUP($F38,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2921,7 +2921,7 @@
         <x:f>IF($D39="","",IF($D39="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F39" s="53" t="str">
-        <x:f>IF($B39="","",IFERROR(VLOOKUP($B39,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B39="","",IFERROR(VLOOKUP($B39,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G39" s="65" t="str">
         <x:f>IF($F39="","",IFERROR(VLOOKUP($F39,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -2977,7 +2977,7 @@
         <x:f>IF($D40="","",IF($D40="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F40" s="53" t="str">
-        <x:f>IF($B40="","",IFERROR(VLOOKUP($B40,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B40="","",IFERROR(VLOOKUP($B40,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G40" s="65" t="str">
         <x:f>IF($F40="","",IFERROR(VLOOKUP($F40,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3033,7 +3033,7 @@
         <x:f>IF($D41="","",IF($D41="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F41" s="53" t="str">
-        <x:f>IF($B41="","",IFERROR(VLOOKUP($B41,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B41="","",IFERROR(VLOOKUP($B41,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G41" s="65" t="str">
         <x:f>IF($F41="","",IFERROR(VLOOKUP($F41,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3089,7 +3089,7 @@
         <x:f>IF($D42="","",IF($D42="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F42" s="53" t="str">
-        <x:f>IF($B42="","",IFERROR(VLOOKUP($B42,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B42="","",IFERROR(VLOOKUP($B42,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G42" s="65" t="str">
         <x:f>IF($F42="","",IFERROR(VLOOKUP($F42,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3145,7 +3145,7 @@
         <x:f>IF($D43="","",IF($D43="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F43" s="53" t="str">
-        <x:f>IF($B43="","",IFERROR(VLOOKUP($B43,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B43="","",IFERROR(VLOOKUP($B43,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G43" s="65" t="str">
         <x:f>IF($F43="","",IFERROR(VLOOKUP($F43,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3201,7 +3201,7 @@
         <x:f>IF($D44="","",IF($D44="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F44" s="53" t="str">
-        <x:f>IF($B44="","",IFERROR(VLOOKUP($B44,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B44="","",IFERROR(VLOOKUP($B44,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G44" s="65" t="str">
         <x:f>IF($F44="","",IFERROR(VLOOKUP($F44,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3257,7 +3257,7 @@
         <x:f>IF($D45="","",IF($D45="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F45" s="53" t="str">
-        <x:f>IF($B45="","",IFERROR(VLOOKUP($B45,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B45="","",IFERROR(VLOOKUP($B45,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G45" s="65" t="str">
         <x:f>IF($F45="","",IFERROR(VLOOKUP($F45,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3313,7 +3313,7 @@
         <x:f>IF($D46="","",IF($D46="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F46" s="53" t="str">
-        <x:f>IF($B46="","",IFERROR(VLOOKUP($B46,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B46="","",IFERROR(VLOOKUP($B46,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G46" s="65" t="str">
         <x:f>IF($F46="","",IFERROR(VLOOKUP($F46,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3369,7 +3369,7 @@
         <x:f>IF($D47="","",IF($D47="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F47" s="53" t="str">
-        <x:f>IF($B47="","",IFERROR(VLOOKUP($B47,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B47="","",IFERROR(VLOOKUP($B47,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G47" s="65" t="str">
         <x:f>IF($F47="","",IFERROR(VLOOKUP($F47,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3425,7 +3425,7 @@
         <x:f>IF($D48="","",IF($D48="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F48" s="53" t="str">
-        <x:f>IF($B48="","",IFERROR(VLOOKUP($B48,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B48="","",IFERROR(VLOOKUP($B48,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G48" s="65" t="str">
         <x:f>IF($F48="","",IFERROR(VLOOKUP($F48,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3481,7 +3481,7 @@
         <x:f>IF($D49="","",IF($D49="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F49" s="53" t="str">
-        <x:f>IF($B49="","",IFERROR(VLOOKUP($B49,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B49="","",IFERROR(VLOOKUP($B49,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G49" s="65" t="str">
         <x:f>IF($F49="","",IFERROR(VLOOKUP($F49,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3537,7 +3537,7 @@
         <x:f>IF($D50="","",IF($D50="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F50" s="53" t="str">
-        <x:f>IF($B50="","",IFERROR(VLOOKUP($B50,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B50="","",IFERROR(VLOOKUP($B50,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G50" s="65" t="str">
         <x:f>IF($F50="","",IFERROR(VLOOKUP($F50,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3593,7 +3593,7 @@
         <x:f>IF($D51="","",IF($D51="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F51" s="53" t="str">
-        <x:f>IF($B51="","",IFERROR(VLOOKUP($B51,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B51="","",IFERROR(VLOOKUP($B51,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G51" s="65" t="str">
         <x:f>IF($F51="","",IFERROR(VLOOKUP($F51,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3649,7 +3649,7 @@
         <x:f>IF($D52="","",IF($D52="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F52" s="53" t="str">
-        <x:f>IF($B52="","",IFERROR(VLOOKUP($B52,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B52="","",IFERROR(VLOOKUP($B52,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G52" s="65" t="str">
         <x:f>IF($F52="","",IFERROR(VLOOKUP($F52,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3705,7 +3705,7 @@
         <x:f>IF($D53="","",IF($D53="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F53" s="53" t="str">
-        <x:f>IF($B53="","",IFERROR(VLOOKUP($B53,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B53="","",IFERROR(VLOOKUP($B53,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G53" s="65" t="str">
         <x:f>IF($F53="","",IFERROR(VLOOKUP($F53,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3761,7 +3761,7 @@
         <x:f>IF($D54="","",IF($D54="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F54" s="53" t="str">
-        <x:f>IF($B54="","",IFERROR(VLOOKUP($B54,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B54="","",IFERROR(VLOOKUP($B54,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G54" s="65" t="str">
         <x:f>IF($F54="","",IFERROR(VLOOKUP($F54,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3817,7 +3817,7 @@
         <x:f>IF($D55="","",IF($D55="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F55" s="53" t="str">
-        <x:f>IF($B55="","",IFERROR(VLOOKUP($B55,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B55="","",IFERROR(VLOOKUP($B55,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G55" s="65" t="str">
         <x:f>IF($F55="","",IFERROR(VLOOKUP($F55,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3873,7 +3873,7 @@
         <x:f>IF($D56="","",IF($D56="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F56" s="53" t="str">
-        <x:f>IF($B56="","",IFERROR(VLOOKUP($B56,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B56="","",IFERROR(VLOOKUP($B56,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G56" s="65" t="str">
         <x:f>IF($F56="","",IFERROR(VLOOKUP($F56,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3929,7 +3929,7 @@
         <x:f>IF($D57="","",IF($D57="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F57" s="53" t="str">
-        <x:f>IF($B57="","",IFERROR(VLOOKUP($B57,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B57="","",IFERROR(VLOOKUP($B57,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G57" s="65" t="str">
         <x:f>IF($F57="","",IFERROR(VLOOKUP($F57,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -3985,7 +3985,7 @@
         <x:f>IF($D58="","",IF($D58="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F58" s="53" t="str">
-        <x:f>IF($B58="","",IFERROR(VLOOKUP($B58,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B58="","",IFERROR(VLOOKUP($B58,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G58" s="65" t="str">
         <x:f>IF($F58="","",IFERROR(VLOOKUP($F58,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4041,7 +4041,7 @@
         <x:f>IF($D59="","",IF($D59="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F59" s="53" t="str">
-        <x:f>IF($B59="","",IFERROR(VLOOKUP($B59,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B59="","",IFERROR(VLOOKUP($B59,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G59" s="65" t="str">
         <x:f>IF($F59="","",IFERROR(VLOOKUP($F59,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4097,7 +4097,7 @@
         <x:f>IF($D60="","",IF($D60="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F60" s="53" t="str">
-        <x:f>IF($B60="","",IFERROR(VLOOKUP($B60,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B60="","",IFERROR(VLOOKUP($B60,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G60" s="65" t="str">
         <x:f>IF($F60="","",IFERROR(VLOOKUP($F60,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4153,7 +4153,7 @@
         <x:f>IF($D61="","",IF($D61="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F61" s="53" t="str">
-        <x:f>IF($B61="","",IFERROR(VLOOKUP($B61,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B61="","",IFERROR(VLOOKUP($B61,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G61" s="65" t="str">
         <x:f>IF($F61="","",IFERROR(VLOOKUP($F61,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4209,7 +4209,7 @@
         <x:f>IF($D62="","",IF($D62="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F62" s="53" t="str">
-        <x:f>IF($B62="","",IFERROR(VLOOKUP($B62,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B62="","",IFERROR(VLOOKUP($B62,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G62" s="65" t="str">
         <x:f>IF($F62="","",IFERROR(VLOOKUP($F62,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4265,7 +4265,7 @@
         <x:f>IF($D63="","",IF($D63="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F63" s="53" t="str">
-        <x:f>IF($B63="","",IFERROR(VLOOKUP($B63,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B63="","",IFERROR(VLOOKUP($B63,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G63" s="65" t="str">
         <x:f>IF($F63="","",IFERROR(VLOOKUP($F63,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4321,7 +4321,7 @@
         <x:f>IF($D64="","",IF($D64="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F64" s="53" t="str">
-        <x:f>IF($B64="","",IFERROR(VLOOKUP($B64,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B64="","",IFERROR(VLOOKUP($B64,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G64" s="65" t="str">
         <x:f>IF($F64="","",IFERROR(VLOOKUP($F64,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4377,7 +4377,7 @@
         <x:f>IF($D65="","",IF($D65="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F65" s="53" t="str">
-        <x:f>IF($B65="","",IFERROR(VLOOKUP($B65,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B65="","",IFERROR(VLOOKUP($B65,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G65" s="65" t="str">
         <x:f>IF($F65="","",IFERROR(VLOOKUP($F65,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4433,7 +4433,7 @@
         <x:f>IF($D66="","",IF($D66="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F66" s="53" t="str">
-        <x:f>IF($B66="","",IFERROR(VLOOKUP($B66,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B66="","",IFERROR(VLOOKUP($B66,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G66" s="65" t="str">
         <x:f>IF($F66="","",IFERROR(VLOOKUP($F66,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4489,7 +4489,7 @@
         <x:f>IF($D67="","",IF($D67="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F67" s="53" t="str">
-        <x:f>IF($B67="","",IFERROR(VLOOKUP($B67,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B67="","",IFERROR(VLOOKUP($B67,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G67" s="65" t="str">
         <x:f>IF($F67="","",IFERROR(VLOOKUP($F67,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4545,7 +4545,7 @@
         <x:f>IF($D68="","",IF($D68="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F68" s="53" t="str">
-        <x:f>IF($B68="","",IFERROR(VLOOKUP($B68,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B68="","",IFERROR(VLOOKUP($B68,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G68" s="65" t="str">
         <x:f>IF($F68="","",IFERROR(VLOOKUP($F68,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4601,7 +4601,7 @@
         <x:f>IF($D69="","",IF($D69="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F69" s="53" t="str">
-        <x:f>IF($B69="","",IFERROR(VLOOKUP($B69,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B69="","",IFERROR(VLOOKUP($B69,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G69" s="65" t="str">
         <x:f>IF($F69="","",IFERROR(VLOOKUP($F69,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4657,7 +4657,7 @@
         <x:f>IF($D70="","",IF($D70="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F70" s="53" t="str">
-        <x:f>IF($B70="","",IFERROR(VLOOKUP($B70,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B70="","",IFERROR(VLOOKUP($B70,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G70" s="65" t="str">
         <x:f>IF($F70="","",IFERROR(VLOOKUP($F70,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4713,7 +4713,7 @@
         <x:f>IF($D71="","",IF($D71="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F71" s="53" t="str">
-        <x:f>IF($B71="","",IFERROR(VLOOKUP($B71,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B71="","",IFERROR(VLOOKUP($B71,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G71" s="65" t="str">
         <x:f>IF($F71="","",IFERROR(VLOOKUP($F71,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4769,7 +4769,7 @@
         <x:f>IF($D72="","",IF($D72="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F72" s="53" t="str">
-        <x:f>IF($B72="","",IFERROR(VLOOKUP($B72,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B72="","",IFERROR(VLOOKUP($B72,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G72" s="65" t="str">
         <x:f>IF($F72="","",IFERROR(VLOOKUP($F72,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4825,7 +4825,7 @@
         <x:f>IF($D73="","",IF($D73="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F73" s="53" t="str">
-        <x:f>IF($B73="","",IFERROR(VLOOKUP($B73,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B73="","",IFERROR(VLOOKUP($B73,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G73" s="65" t="str">
         <x:f>IF($F73="","",IFERROR(VLOOKUP($F73,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4881,7 +4881,7 @@
         <x:f>IF($D74="","",IF($D74="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F74" s="53" t="str">
-        <x:f>IF($B74="","",IFERROR(VLOOKUP($B74,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B74="","",IFERROR(VLOOKUP($B74,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G74" s="65" t="str">
         <x:f>IF($F74="","",IFERROR(VLOOKUP($F74,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4937,7 +4937,7 @@
         <x:f>IF($D75="","",IF($D75="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F75" s="53" t="str">
-        <x:f>IF($B75="","",IFERROR(VLOOKUP($B75,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B75="","",IFERROR(VLOOKUP($B75,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G75" s="65" t="str">
         <x:f>IF($F75="","",IFERROR(VLOOKUP($F75,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -4993,7 +4993,7 @@
         <x:f>IF($D76="","",IF($D76="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F76" s="53" t="str">
-        <x:f>IF($B76="","",IFERROR(VLOOKUP($B76,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B76="","",IFERROR(VLOOKUP($B76,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G76" s="65" t="str">
         <x:f>IF($F76="","",IFERROR(VLOOKUP($F76,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5049,7 +5049,7 @@
         <x:f>IF($D77="","",IF($D77="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F77" s="53" t="str">
-        <x:f>IF($B77="","",IFERROR(VLOOKUP($B77,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B77="","",IFERROR(VLOOKUP($B77,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G77" s="65" t="str">
         <x:f>IF($F77="","",IFERROR(VLOOKUP($F77,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5105,7 +5105,7 @@
         <x:f>IF($D78="","",IF($D78="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F78" s="53" t="str">
-        <x:f>IF($B78="","",IFERROR(VLOOKUP($B78,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B78="","",IFERROR(VLOOKUP($B78,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G78" s="65" t="str">
         <x:f>IF($F78="","",IFERROR(VLOOKUP($F78,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5161,7 +5161,7 @@
         <x:f>IF($D79="","",IF($D79="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F79" s="53" t="str">
-        <x:f>IF($B79="","",IFERROR(VLOOKUP($B79,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B79="","",IFERROR(VLOOKUP($B79,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G79" s="65" t="str">
         <x:f>IF($F79="","",IFERROR(VLOOKUP($F79,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5217,7 +5217,7 @@
         <x:f>IF($D80="","",IF($D80="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F80" s="53" t="str">
-        <x:f>IF($B80="","",IFERROR(VLOOKUP($B80,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B80="","",IFERROR(VLOOKUP($B80,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G80" s="65" t="str">
         <x:f>IF($F80="","",IFERROR(VLOOKUP($F80,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5273,7 +5273,7 @@
         <x:f>IF($D81="","",IF($D81="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F81" s="53" t="str">
-        <x:f>IF($B81="","",IFERROR(VLOOKUP($B81,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B81="","",IFERROR(VLOOKUP($B81,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G81" s="65" t="str">
         <x:f>IF($F81="","",IFERROR(VLOOKUP($F81,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5329,7 +5329,7 @@
         <x:f>IF($D82="","",IF($D82="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F82" s="53" t="str">
-        <x:f>IF($B82="","",IFERROR(VLOOKUP($B82,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B82="","",IFERROR(VLOOKUP($B82,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G82" s="65" t="str">
         <x:f>IF($F82="","",IFERROR(VLOOKUP($F82,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5385,7 +5385,7 @@
         <x:f>IF($D83="","",IF($D83="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F83" s="53" t="str">
-        <x:f>IF($B83="","",IFERROR(VLOOKUP($B83,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B83="","",IFERROR(VLOOKUP($B83,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G83" s="65" t="str">
         <x:f>IF($F83="","",IFERROR(VLOOKUP($F83,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5441,7 +5441,7 @@
         <x:f>IF($D84="","",IF($D84="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F84" s="53" t="str">
-        <x:f>IF($B84="","",IFERROR(VLOOKUP($B84,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B84="","",IFERROR(VLOOKUP($B84,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G84" s="65" t="str">
         <x:f>IF($F84="","",IFERROR(VLOOKUP($F84,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5497,7 +5497,7 @@
         <x:f>IF($D85="","",IF($D85="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F85" s="53" t="str">
-        <x:f>IF($B85="","",IFERROR(VLOOKUP($B85,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B85="","",IFERROR(VLOOKUP($B85,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G85" s="65" t="str">
         <x:f>IF($F85="","",IFERROR(VLOOKUP($F85,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5553,7 +5553,7 @@
         <x:f>IF($D86="","",IF($D86="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F86" s="53" t="str">
-        <x:f>IF($B86="","",IFERROR(VLOOKUP($B86,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B86="","",IFERROR(VLOOKUP($B86,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G86" s="65" t="str">
         <x:f>IF($F86="","",IFERROR(VLOOKUP($F86,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5609,7 +5609,7 @@
         <x:f>IF($D87="","",IF($D87="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F87" s="53" t="str">
-        <x:f>IF($B87="","",IFERROR(VLOOKUP($B87,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B87="","",IFERROR(VLOOKUP($B87,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G87" s="65" t="str">
         <x:f>IF($F87="","",IFERROR(VLOOKUP($F87,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5665,7 +5665,7 @@
         <x:f>IF($D88="","",IF($D88="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F88" s="53" t="str">
-        <x:f>IF($B88="","",IFERROR(VLOOKUP($B88,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B88="","",IFERROR(VLOOKUP($B88,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G88" s="65" t="str">
         <x:f>IF($F88="","",IFERROR(VLOOKUP($F88,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5721,7 +5721,7 @@
         <x:f>IF($D89="","",IF($D89="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F89" s="53" t="str">
-        <x:f>IF($B89="","",IFERROR(VLOOKUP($B89,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B89="","",IFERROR(VLOOKUP($B89,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G89" s="65" t="str">
         <x:f>IF($F89="","",IFERROR(VLOOKUP($F89,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5777,7 +5777,7 @@
         <x:f>IF($D90="","",IF($D90="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F90" s="53" t="str">
-        <x:f>IF($B90="","",IFERROR(VLOOKUP($B90,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B90="","",IFERROR(VLOOKUP($B90,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G90" s="65" t="str">
         <x:f>IF($F90="","",IFERROR(VLOOKUP($F90,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5833,7 +5833,7 @@
         <x:f>IF($D91="","",IF($D91="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F91" s="53" t="str">
-        <x:f>IF($B91="","",IFERROR(VLOOKUP($B91,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B91="","",IFERROR(VLOOKUP($B91,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G91" s="65" t="str">
         <x:f>IF($F91="","",IFERROR(VLOOKUP($F91,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5889,7 +5889,7 @@
         <x:f>IF($D92="","",IF($D92="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F92" s="53" t="str">
-        <x:f>IF($B92="","",IFERROR(VLOOKUP($B92,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B92="","",IFERROR(VLOOKUP($B92,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G92" s="65" t="str">
         <x:f>IF($F92="","",IFERROR(VLOOKUP($F92,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -5945,7 +5945,7 @@
         <x:f>IF($D93="","",IF($D93="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F93" s="53" t="str">
-        <x:f>IF($B93="","",IFERROR(VLOOKUP($B93,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B93="","",IFERROR(VLOOKUP($B93,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G93" s="65" t="str">
         <x:f>IF($F93="","",IFERROR(VLOOKUP($F93,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6001,7 +6001,7 @@
         <x:f>IF($D94="","",IF($D94="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F94" s="53" t="str">
-        <x:f>IF($B94="","",IFERROR(VLOOKUP($B94,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B94="","",IFERROR(VLOOKUP($B94,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G94" s="65" t="str">
         <x:f>IF($F94="","",IFERROR(VLOOKUP($F94,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6057,7 +6057,7 @@
         <x:f>IF($D95="","",IF($D95="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F95" s="53" t="str">
-        <x:f>IF($B95="","",IFERROR(VLOOKUP($B95,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B95="","",IFERROR(VLOOKUP($B95,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G95" s="65" t="str">
         <x:f>IF($F95="","",IFERROR(VLOOKUP($F95,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6113,7 +6113,7 @@
         <x:f>IF($D96="","",IF($D96="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F96" s="53" t="str">
-        <x:f>IF($B96="","",IFERROR(VLOOKUP($B96,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B96="","",IFERROR(VLOOKUP($B96,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G96" s="65" t="str">
         <x:f>IF($F96="","",IFERROR(VLOOKUP($F96,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6169,7 +6169,7 @@
         <x:f>IF($D97="","",IF($D97="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F97" s="53" t="str">
-        <x:f>IF($B97="","",IFERROR(VLOOKUP($B97,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B97="","",IFERROR(VLOOKUP($B97,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G97" s="65" t="str">
         <x:f>IF($F97="","",IFERROR(VLOOKUP($F97,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6225,7 +6225,7 @@
         <x:f>IF($D98="","",IF($D98="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F98" s="53" t="str">
-        <x:f>IF($B98="","",IFERROR(VLOOKUP($B98,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B98="","",IFERROR(VLOOKUP($B98,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G98" s="65" t="str">
         <x:f>IF($F98="","",IFERROR(VLOOKUP($F98,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6281,7 +6281,7 @@
         <x:f>IF($D99="","",IF($D99="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F99" s="53" t="str">
-        <x:f>IF($B99="","",IFERROR(VLOOKUP($B99,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B99="","",IFERROR(VLOOKUP($B99,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G99" s="65" t="str">
         <x:f>IF($F99="","",IFERROR(VLOOKUP($F99,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6337,7 +6337,7 @@
         <x:f>IF($D100="","",IF($D100="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F100" s="53" t="str">
-        <x:f>IF($B100="","",IFERROR(VLOOKUP($B100,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B100="","",IFERROR(VLOOKUP($B100,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G100" s="65" t="str">
         <x:f>IF($F100="","",IFERROR(VLOOKUP($F100,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6393,7 +6393,7 @@
         <x:f>IF($D101="","",IF($D101="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F101" s="53" t="str">
-        <x:f>IF($B101="","",IFERROR(VLOOKUP($B101,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B101="","",IFERROR(VLOOKUP($B101,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G101" s="65" t="str">
         <x:f>IF($F101="","",IFERROR(VLOOKUP($F101,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6449,7 +6449,7 @@
         <x:f>IF($D102="","",IF($D102="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F102" s="53" t="str">
-        <x:f>IF($B102="","",IFERROR(VLOOKUP($B102,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B102="","",IFERROR(VLOOKUP($B102,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G102" s="65" t="str">
         <x:f>IF($F102="","",IFERROR(VLOOKUP($F102,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6505,7 +6505,7 @@
         <x:f>IF($D103="","",IF($D103="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F103" s="53" t="str">
-        <x:f>IF($B103="","",IFERROR(VLOOKUP($B103,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B103="","",IFERROR(VLOOKUP($B103,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G103" s="65" t="str">
         <x:f>IF($F103="","",IFERROR(VLOOKUP($F103,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6561,7 +6561,7 @@
         <x:f>IF($D104="","",IF($D104="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F104" s="53" t="str">
-        <x:f>IF($B104="","",IFERROR(VLOOKUP($B104,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B104="","",IFERROR(VLOOKUP($B104,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G104" s="65" t="str">
         <x:f>IF($F104="","",IFERROR(VLOOKUP($F104,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6617,7 +6617,7 @@
         <x:f>IF($D105="","",IF($D105="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F105" s="53" t="str">
-        <x:f>IF($B105="","",IFERROR(VLOOKUP($B105,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B105="","",IFERROR(VLOOKUP($B105,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G105" s="65" t="str">
         <x:f>IF($F105="","",IFERROR(VLOOKUP($F105,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6673,7 +6673,7 @@
         <x:f>IF($D106="","",IF($D106="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F106" s="53" t="str">
-        <x:f>IF($B106="","",IFERROR(VLOOKUP($B106,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B106="","",IFERROR(VLOOKUP($B106,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G106" s="65" t="str">
         <x:f>IF($F106="","",IFERROR(VLOOKUP($F106,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6729,7 +6729,7 @@
         <x:f>IF($D107="","",IF($D107="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F107" s="53" t="str">
-        <x:f>IF($B107="","",IFERROR(VLOOKUP($B107,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B107="","",IFERROR(VLOOKUP($B107,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G107" s="65" t="str">
         <x:f>IF($F107="","",IFERROR(VLOOKUP($F107,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6785,7 +6785,7 @@
         <x:f>IF($D108="","",IF($D108="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F108" s="53" t="str">
-        <x:f>IF($B108="","",IFERROR(VLOOKUP($B108,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B108="","",IFERROR(VLOOKUP($B108,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G108" s="65" t="str">
         <x:f>IF($F108="","",IFERROR(VLOOKUP($F108,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6841,7 +6841,7 @@
         <x:f>IF($D109="","",IF($D109="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F109" s="53" t="str">
-        <x:f>IF($B109="","",IFERROR(VLOOKUP($B109,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B109="","",IFERROR(VLOOKUP($B109,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G109" s="65" t="str">
         <x:f>IF($F109="","",IFERROR(VLOOKUP($F109,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6897,7 +6897,7 @@
         <x:f>IF($D110="","",IF($D110="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F110" s="53" t="str">
-        <x:f>IF($B110="","",IFERROR(VLOOKUP($B110,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B110="","",IFERROR(VLOOKUP($B110,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G110" s="65" t="str">
         <x:f>IF($F110="","",IFERROR(VLOOKUP($F110,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -6953,7 +6953,7 @@
         <x:f>IF($D111="","",IF($D111="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F111" s="53" t="str">
-        <x:f>IF($B111="","",IFERROR(VLOOKUP($B111,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B111="","",IFERROR(VLOOKUP($B111,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G111" s="65" t="str">
         <x:f>IF($F111="","",IFERROR(VLOOKUP($F111,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7009,7 +7009,7 @@
         <x:f>IF($D112="","",IF($D112="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F112" s="53" t="str">
-        <x:f>IF($B112="","",IFERROR(VLOOKUP($B112,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B112="","",IFERROR(VLOOKUP($B112,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G112" s="65" t="str">
         <x:f>IF($F112="","",IFERROR(VLOOKUP($F112,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7065,7 +7065,7 @@
         <x:f>IF($D113="","",IF($D113="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F113" s="53" t="str">
-        <x:f>IF($B113="","",IFERROR(VLOOKUP($B113,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B113="","",IFERROR(VLOOKUP($B113,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G113" s="65" t="str">
         <x:f>IF($F113="","",IFERROR(VLOOKUP($F113,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7121,7 +7121,7 @@
         <x:f>IF($D114="","",IF($D114="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F114" s="53" t="str">
-        <x:f>IF($B114="","",IFERROR(VLOOKUP($B114,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B114="","",IFERROR(VLOOKUP($B114,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G114" s="65" t="str">
         <x:f>IF($F114="","",IFERROR(VLOOKUP($F114,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7161,6 +7161,9 @@
       </x:c>
       <x:c r="S114" s="54" t="str">
         <x:f>IF(AND($A114="",$B114="",$C114=""),"",IF($A114="","Missing Assignment Number",IF($B114="","Select Job Title",IF($C114="","Enter Pay Rate",IF($F114="","Job Title not found","Ready")))))</x:f>
+      </x:c>
+      <x:c r="U114" t="str">
+        <x:v>Production Operator - II - Production &amp; Operations Support (T): Industrial - O2 (Low)</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="22" customHeight="1">
@@ -7174,7 +7177,7 @@
         <x:f>IF($D115="","",IF($D115="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F115" s="53" t="str">
-        <x:f>IF($B115="","",IFERROR(VLOOKUP($B115,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B115="","",IFERROR(VLOOKUP($B115,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G115" s="65" t="str">
         <x:f>IF($F115="","",IFERROR(VLOOKUP($F115,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7227,7 +7230,7 @@
         <x:f>IF($D116="","",IF($D116="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F116" s="53" t="str">
-        <x:f>IF($B116="","",IFERROR(VLOOKUP($B116,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B116="","",IFERROR(VLOOKUP($B116,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G116" s="65" t="str">
         <x:f>IF($F116="","",IFERROR(VLOOKUP($F116,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7280,7 +7283,7 @@
         <x:f>IF($D117="","",IF($D117="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F117" s="53" t="str">
-        <x:f>IF($B117="","",IFERROR(VLOOKUP($B117,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B117="","",IFERROR(VLOOKUP($B117,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G117" s="65" t="str">
         <x:f>IF($F117="","",IFERROR(VLOOKUP($F117,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7333,7 +7336,7 @@
         <x:f>IF($D118="","",IF($D118="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F118" s="53" t="str">
-        <x:f>IF($B118="","",IFERROR(VLOOKUP($B118,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B118="","",IFERROR(VLOOKUP($B118,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G118" s="65" t="str">
         <x:f>IF($F118="","",IFERROR(VLOOKUP($F118,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7386,7 +7389,7 @@
         <x:f>IF($D119="","",IF($D119="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F119" s="53" t="str">
-        <x:f>IF($B119="","",IFERROR(VLOOKUP($B119,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B119="","",IFERROR(VLOOKUP($B119,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G119" s="65" t="str">
         <x:f>IF($F119="","",IFERROR(VLOOKUP($F119,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7439,7 +7442,7 @@
         <x:f>IF($D120="","",IF($D120="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F120" s="53" t="str">
-        <x:f>IF($B120="","",IFERROR(VLOOKUP($B120,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B120="","",IFERROR(VLOOKUP($B120,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G120" s="65" t="str">
         <x:f>IF($F120="","",IFERROR(VLOOKUP($F120,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7492,7 +7495,7 @@
         <x:f>IF($D121="","",IF($D121="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F121" s="53" t="str">
-        <x:f>IF($B121="","",IFERROR(VLOOKUP($B121,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B121="","",IFERROR(VLOOKUP($B121,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G121" s="65" t="str">
         <x:f>IF($F121="","",IFERROR(VLOOKUP($F121,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7545,7 +7548,7 @@
         <x:f>IF($D122="","",IF($D122="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F122" s="53" t="str">
-        <x:f>IF($B122="","",IFERROR(VLOOKUP($B122,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B122="","",IFERROR(VLOOKUP($B122,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G122" s="65" t="str">
         <x:f>IF($F122="","",IFERROR(VLOOKUP($F122,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7598,7 +7601,7 @@
         <x:f>IF($D123="","",IF($D123="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F123" s="53" t="str">
-        <x:f>IF($B123="","",IFERROR(VLOOKUP($B123,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B123="","",IFERROR(VLOOKUP($B123,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G123" s="65" t="str">
         <x:f>IF($F123="","",IFERROR(VLOOKUP($F123,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7651,7 +7654,7 @@
         <x:f>IF($D124="","",IF($D124="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F124" s="53" t="str">
-        <x:f>IF($B124="","",IFERROR(VLOOKUP($B124,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B124="","",IFERROR(VLOOKUP($B124,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G124" s="65" t="str">
         <x:f>IF($F124="","",IFERROR(VLOOKUP($F124,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7704,7 +7707,7 @@
         <x:f>IF($D125="","",IF($D125="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F125" s="53" t="str">
-        <x:f>IF($B125="","",IFERROR(VLOOKUP($B125,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B125="","",IFERROR(VLOOKUP($B125,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G125" s="65" t="str">
         <x:f>IF($F125="","",IFERROR(VLOOKUP($F125,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7757,7 +7760,7 @@
         <x:f>IF($D126="","",IF($D126="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F126" s="53" t="str">
-        <x:f>IF($B126="","",IFERROR(VLOOKUP($B126,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B126="","",IFERROR(VLOOKUP($B126,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G126" s="65" t="str">
         <x:f>IF($F126="","",IFERROR(VLOOKUP($F126,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7810,7 +7813,7 @@
         <x:f>IF($D127="","",IF($D127="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F127" s="53" t="str">
-        <x:f>IF($B127="","",IFERROR(VLOOKUP($B127,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B127="","",IFERROR(VLOOKUP($B127,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G127" s="65" t="str">
         <x:f>IF($F127="","",IFERROR(VLOOKUP($F127,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7863,7 +7866,7 @@
         <x:f>IF($D128="","",IF($D128="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F128" s="53" t="str">
-        <x:f>IF($B128="","",IFERROR(VLOOKUP($B128,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B128="","",IFERROR(VLOOKUP($B128,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G128" s="65" t="str">
         <x:f>IF($F128="","",IFERROR(VLOOKUP($F128,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7916,7 +7919,7 @@
         <x:f>IF($D129="","",IF($D129="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F129" s="53" t="str">
-        <x:f>IF($B129="","",IFERROR(VLOOKUP($B129,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B129="","",IFERROR(VLOOKUP($B129,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G129" s="65" t="str">
         <x:f>IF($F129="","",IFERROR(VLOOKUP($F129,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -7969,7 +7972,7 @@
         <x:f>IF($D130="","",IF($D130="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F130" s="53" t="str">
-        <x:f>IF($B130="","",IFERROR(VLOOKUP($B130,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B130="","",IFERROR(VLOOKUP($B130,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G130" s="65" t="str">
         <x:f>IF($F130="","",IFERROR(VLOOKUP($F130,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8022,7 +8025,7 @@
         <x:f>IF($D131="","",IF($D131="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F131" s="53" t="str">
-        <x:f>IF($B131="","",IFERROR(VLOOKUP($B131,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B131="","",IFERROR(VLOOKUP($B131,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G131" s="65" t="str">
         <x:f>IF($F131="","",IFERROR(VLOOKUP($F131,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8075,7 +8078,7 @@
         <x:f>IF($D132="","",IF($D132="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F132" s="53" t="str">
-        <x:f>IF($B132="","",IFERROR(VLOOKUP($B132,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B132="","",IFERROR(VLOOKUP($B132,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G132" s="65" t="str">
         <x:f>IF($F132="","",IFERROR(VLOOKUP($F132,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8128,7 +8131,7 @@
         <x:f>IF($D133="","",IF($D133="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F133" s="53" t="str">
-        <x:f>IF($B133="","",IFERROR(VLOOKUP($B133,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B133="","",IFERROR(VLOOKUP($B133,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G133" s="65" t="str">
         <x:f>IF($F133="","",IFERROR(VLOOKUP($F133,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8181,7 +8184,7 @@
         <x:f>IF($D134="","",IF($D134="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F134" s="53" t="str">
-        <x:f>IF($B134="","",IFERROR(VLOOKUP($B134,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B134="","",IFERROR(VLOOKUP($B134,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G134" s="65" t="str">
         <x:f>IF($F134="","",IFERROR(VLOOKUP($F134,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8234,7 +8237,7 @@
         <x:f>IF($D135="","",IF($D135="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F135" s="53" t="str">
-        <x:f>IF($B135="","",IFERROR(VLOOKUP($B135,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B135="","",IFERROR(VLOOKUP($B135,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G135" s="65" t="str">
         <x:f>IF($F135="","",IFERROR(VLOOKUP($F135,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8287,7 +8290,7 @@
         <x:f>IF($D136="","",IF($D136="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F136" s="53" t="str">
-        <x:f>IF($B136="","",IFERROR(VLOOKUP($B136,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B136="","",IFERROR(VLOOKUP($B136,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G136" s="65" t="str">
         <x:f>IF($F136="","",IFERROR(VLOOKUP($F136,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8340,7 +8343,7 @@
         <x:f>IF($D137="","",IF($D137="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F137" s="53" t="str">
-        <x:f>IF($B137="","",IFERROR(VLOOKUP($B137,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B137="","",IFERROR(VLOOKUP($B137,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G137" s="65" t="str">
         <x:f>IF($F137="","",IFERROR(VLOOKUP($F137,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8393,7 +8396,7 @@
         <x:f>IF($D138="","",IF($D138="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F138" s="53" t="str">
-        <x:f>IF($B138="","",IFERROR(VLOOKUP($B138,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B138="","",IFERROR(VLOOKUP($B138,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G138" s="65" t="str">
         <x:f>IF($F138="","",IFERROR(VLOOKUP($F138,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8446,7 +8449,7 @@
         <x:f>IF($D139="","",IF($D139="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F139" s="53" t="str">
-        <x:f>IF($B139="","",IFERROR(VLOOKUP($B139,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B139="","",IFERROR(VLOOKUP($B139,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G139" s="65" t="str">
         <x:f>IF($F139="","",IFERROR(VLOOKUP($F139,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8499,7 +8502,7 @@
         <x:f>IF($D140="","",IF($D140="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F140" s="53" t="str">
-        <x:f>IF($B140="","",IFERROR(VLOOKUP($B140,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B140="","",IFERROR(VLOOKUP($B140,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G140" s="65" t="str">
         <x:f>IF($F140="","",IFERROR(VLOOKUP($F140,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8552,7 +8555,7 @@
         <x:f>IF($D141="","",IF($D141="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F141" s="53" t="str">
-        <x:f>IF($B141="","",IFERROR(VLOOKUP($B141,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B141="","",IFERROR(VLOOKUP($B141,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G141" s="65" t="str">
         <x:f>IF($F141="","",IFERROR(VLOOKUP($F141,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8605,7 +8608,7 @@
         <x:f>IF($D142="","",IF($D142="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F142" s="53" t="str">
-        <x:f>IF($B142="","",IFERROR(VLOOKUP($B142,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B142="","",IFERROR(VLOOKUP($B142,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G142" s="65" t="str">
         <x:f>IF($F142="","",IFERROR(VLOOKUP($F142,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8658,7 +8661,7 @@
         <x:f>IF($D143="","",IF($D143="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F143" s="53" t="str">
-        <x:f>IF($B143="","",IFERROR(VLOOKUP($B143,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B143="","",IFERROR(VLOOKUP($B143,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G143" s="65" t="str">
         <x:f>IF($F143="","",IFERROR(VLOOKUP($F143,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8711,7 +8714,7 @@
         <x:f>IF($D144="","",IF($D144="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F144" s="53" t="str">
-        <x:f>IF($B144="","",IFERROR(VLOOKUP($B144,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B144="","",IFERROR(VLOOKUP($B144,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G144" s="65" t="str">
         <x:f>IF($F144="","",IFERROR(VLOOKUP($F144,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8764,7 +8767,7 @@
         <x:f>IF($D145="","",IF($D145="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F145" s="53" t="str">
-        <x:f>IF($B145="","",IFERROR(VLOOKUP($B145,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B145="","",IFERROR(VLOOKUP($B145,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G145" s="65" t="str">
         <x:f>IF($F145="","",IFERROR(VLOOKUP($F145,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8817,7 +8820,7 @@
         <x:f>IF($D146="","",IF($D146="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F146" s="53" t="str">
-        <x:f>IF($B146="","",IFERROR(VLOOKUP($B146,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B146="","",IFERROR(VLOOKUP($B146,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G146" s="65" t="str">
         <x:f>IF($F146="","",IFERROR(VLOOKUP($F146,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8870,7 +8873,7 @@
         <x:f>IF($D147="","",IF($D147="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F147" s="53" t="str">
-        <x:f>IF($B147="","",IFERROR(VLOOKUP($B147,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B147="","",IFERROR(VLOOKUP($B147,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G147" s="65" t="str">
         <x:f>IF($F147="","",IFERROR(VLOOKUP($F147,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8923,7 +8926,7 @@
         <x:f>IF($D148="","",IF($D148="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F148" s="53" t="str">
-        <x:f>IF($B148="","",IFERROR(VLOOKUP($B148,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B148="","",IFERROR(VLOOKUP($B148,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G148" s="65" t="str">
         <x:f>IF($F148="","",IFERROR(VLOOKUP($F148,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -8976,7 +8979,7 @@
         <x:f>IF($D149="","",IF($D149="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F149" s="53" t="str">
-        <x:f>IF($B149="","",IFERROR(VLOOKUP($B149,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B149="","",IFERROR(VLOOKUP($B149,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G149" s="65" t="str">
         <x:f>IF($F149="","",IFERROR(VLOOKUP($F149,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9029,7 +9032,7 @@
         <x:f>IF($D150="","",IF($D150="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F150" s="53" t="str">
-        <x:f>IF($B150="","",IFERROR(VLOOKUP($B150,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B150="","",IFERROR(VLOOKUP($B150,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G150" s="65" t="str">
         <x:f>IF($F150="","",IFERROR(VLOOKUP($F150,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9082,7 +9085,7 @@
         <x:f>IF($D151="","",IF($D151="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F151" s="53" t="str">
-        <x:f>IF($B151="","",IFERROR(VLOOKUP($B151,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B151="","",IFERROR(VLOOKUP($B151,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G151" s="65" t="str">
         <x:f>IF($F151="","",IFERROR(VLOOKUP($F151,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9135,7 +9138,7 @@
         <x:f>IF($D152="","",IF($D152="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F152" s="53" t="str">
-        <x:f>IF($B152="","",IFERROR(VLOOKUP($B152,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B152="","",IFERROR(VLOOKUP($B152,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G152" s="65" t="str">
         <x:f>IF($F152="","",IFERROR(VLOOKUP($F152,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9188,7 +9191,7 @@
         <x:f>IF($D153="","",IF($D153="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F153" s="53" t="str">
-        <x:f>IF($B153="","",IFERROR(VLOOKUP($B153,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B153="","",IFERROR(VLOOKUP($B153,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G153" s="65" t="str">
         <x:f>IF($F153="","",IFERROR(VLOOKUP($F153,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9241,7 +9244,7 @@
         <x:f>IF($D154="","",IF($D154="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F154" s="53" t="str">
-        <x:f>IF($B154="","",IFERROR(VLOOKUP($B154,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B154="","",IFERROR(VLOOKUP($B154,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G154" s="65" t="str">
         <x:f>IF($F154="","",IFERROR(VLOOKUP($F154,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9294,7 +9297,7 @@
         <x:f>IF($D155="","",IF($D155="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F155" s="53" t="str">
-        <x:f>IF($B155="","",IFERROR(VLOOKUP($B155,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B155="","",IFERROR(VLOOKUP($B155,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G155" s="65" t="str">
         <x:f>IF($F155="","",IFERROR(VLOOKUP($F155,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9347,7 +9350,7 @@
         <x:f>IF($D156="","",IF($D156="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F156" s="53" t="str">
-        <x:f>IF($B156="","",IFERROR(VLOOKUP($B156,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B156="","",IFERROR(VLOOKUP($B156,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G156" s="65" t="str">
         <x:f>IF($F156="","",IFERROR(VLOOKUP($F156,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9400,7 +9403,7 @@
         <x:f>IF($D157="","",IF($D157="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F157" s="53" t="str">
-        <x:f>IF($B157="","",IFERROR(VLOOKUP($B157,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B157="","",IFERROR(VLOOKUP($B157,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G157" s="65" t="str">
         <x:f>IF($F157="","",IFERROR(VLOOKUP($F157,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9453,7 +9456,7 @@
         <x:f>IF($D158="","",IF($D158="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F158" s="53" t="str">
-        <x:f>IF($B158="","",IFERROR(VLOOKUP($B158,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B158="","",IFERROR(VLOOKUP($B158,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G158" s="65" t="str">
         <x:f>IF($F158="","",IFERROR(VLOOKUP($F158,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9506,7 +9509,7 @@
         <x:f>IF($D159="","",IF($D159="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F159" s="53" t="str">
-        <x:f>IF($B159="","",IFERROR(VLOOKUP($B159,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B159="","",IFERROR(VLOOKUP($B159,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G159" s="65" t="str">
         <x:f>IF($F159="","",IFERROR(VLOOKUP($F159,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9559,7 +9562,7 @@
         <x:f>IF($D160="","",IF($D160="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F160" s="53" t="str">
-        <x:f>IF($B160="","",IFERROR(VLOOKUP($B160,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B160="","",IFERROR(VLOOKUP($B160,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G160" s="65" t="str">
         <x:f>IF($F160="","",IFERROR(VLOOKUP($F160,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9612,7 +9615,7 @@
         <x:f>IF($D161="","",IF($D161="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F161" s="53" t="str">
-        <x:f>IF($B161="","",IFERROR(VLOOKUP($B161,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B161="","",IFERROR(VLOOKUP($B161,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G161" s="65" t="str">
         <x:f>IF($F161="","",IFERROR(VLOOKUP($F161,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9665,7 +9668,7 @@
         <x:f>IF($D162="","",IF($D162="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F162" s="53" t="str">
-        <x:f>IF($B162="","",IFERROR(VLOOKUP($B162,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B162="","",IFERROR(VLOOKUP($B162,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G162" s="65" t="str">
         <x:f>IF($F162="","",IFERROR(VLOOKUP($F162,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9718,7 +9721,7 @@
         <x:f>IF($D163="","",IF($D163="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F163" s="53" t="str">
-        <x:f>IF($B163="","",IFERROR(VLOOKUP($B163,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B163="","",IFERROR(VLOOKUP($B163,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G163" s="65" t="str">
         <x:f>IF($F163="","",IFERROR(VLOOKUP($F163,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9771,7 +9774,7 @@
         <x:f>IF($D164="","",IF($D164="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F164" s="53" t="str">
-        <x:f>IF($B164="","",IFERROR(VLOOKUP($B164,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B164="","",IFERROR(VLOOKUP($B164,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G164" s="65" t="str">
         <x:f>IF($F164="","",IFERROR(VLOOKUP($F164,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9824,7 +9827,7 @@
         <x:f>IF($D165="","",IF($D165="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F165" s="53" t="str">
-        <x:f>IF($B165="","",IFERROR(VLOOKUP($B165,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B165="","",IFERROR(VLOOKUP($B165,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G165" s="65" t="str">
         <x:f>IF($F165="","",IFERROR(VLOOKUP($F165,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9877,7 +9880,7 @@
         <x:f>IF($D166="","",IF($D166="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F166" s="53" t="str">
-        <x:f>IF($B166="","",IFERROR(VLOOKUP($B166,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B166="","",IFERROR(VLOOKUP($B166,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G166" s="65" t="str">
         <x:f>IF($F166="","",IFERROR(VLOOKUP($F166,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9930,7 +9933,7 @@
         <x:f>IF($D167="","",IF($D167="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F167" s="53" t="str">
-        <x:f>IF($B167="","",IFERROR(VLOOKUP($B167,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B167="","",IFERROR(VLOOKUP($B167,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G167" s="65" t="str">
         <x:f>IF($F167="","",IFERROR(VLOOKUP($F167,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -9983,7 +9986,7 @@
         <x:f>IF($D168="","",IF($D168="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F168" s="53" t="str">
-        <x:f>IF($B168="","",IFERROR(VLOOKUP($B168,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B168="","",IFERROR(VLOOKUP($B168,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G168" s="65" t="str">
         <x:f>IF($F168="","",IFERROR(VLOOKUP($F168,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10036,7 +10039,7 @@
         <x:f>IF($D169="","",IF($D169="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F169" s="53" t="str">
-        <x:f>IF($B169="","",IFERROR(VLOOKUP($B169,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B169="","",IFERROR(VLOOKUP($B169,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G169" s="65" t="str">
         <x:f>IF($F169="","",IFERROR(VLOOKUP($F169,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10089,7 +10092,7 @@
         <x:f>IF($D170="","",IF($D170="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F170" s="53" t="str">
-        <x:f>IF($B170="","",IFERROR(VLOOKUP($B170,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B170="","",IFERROR(VLOOKUP($B170,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G170" s="65" t="str">
         <x:f>IF($F170="","",IFERROR(VLOOKUP($F170,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10142,7 +10145,7 @@
         <x:f>IF($D171="","",IF($D171="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F171" s="53" t="str">
-        <x:f>IF($B171="","",IFERROR(VLOOKUP($B171,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B171="","",IFERROR(VLOOKUP($B171,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G171" s="65" t="str">
         <x:f>IF($F171="","",IFERROR(VLOOKUP($F171,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10195,7 +10198,7 @@
         <x:f>IF($D172="","",IF($D172="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F172" s="53" t="str">
-        <x:f>IF($B172="","",IFERROR(VLOOKUP($B172,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B172="","",IFERROR(VLOOKUP($B172,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G172" s="65" t="str">
         <x:f>IF($F172="","",IFERROR(VLOOKUP($F172,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10248,7 +10251,7 @@
         <x:f>IF($D173="","",IF($D173="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F173" s="53" t="str">
-        <x:f>IF($B173="","",IFERROR(VLOOKUP($B173,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B173="","",IFERROR(VLOOKUP($B173,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G173" s="65" t="str">
         <x:f>IF($F173="","",IFERROR(VLOOKUP($F173,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10301,7 +10304,7 @@
         <x:f>IF($D174="","",IF($D174="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F174" s="53" t="str">
-        <x:f>IF($B174="","",IFERROR(VLOOKUP($B174,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B174="","",IFERROR(VLOOKUP($B174,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G174" s="65" t="str">
         <x:f>IF($F174="","",IFERROR(VLOOKUP($F174,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10354,7 +10357,7 @@
         <x:f>IF($D175="","",IF($D175="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F175" s="53" t="str">
-        <x:f>IF($B175="","",IFERROR(VLOOKUP($B175,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B175="","",IFERROR(VLOOKUP($B175,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G175" s="65" t="str">
         <x:f>IF($F175="","",IFERROR(VLOOKUP($F175,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10407,7 +10410,7 @@
         <x:f>IF($D176="","",IF($D176="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F176" s="53" t="str">
-        <x:f>IF($B176="","",IFERROR(VLOOKUP($B176,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B176="","",IFERROR(VLOOKUP($B176,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G176" s="65" t="str">
         <x:f>IF($F176="","",IFERROR(VLOOKUP($F176,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10460,7 +10463,7 @@
         <x:f>IF($D177="","",IF($D177="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F177" s="53" t="str">
-        <x:f>IF($B177="","",IFERROR(VLOOKUP($B177,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B177="","",IFERROR(VLOOKUP($B177,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G177" s="65" t="str">
         <x:f>IF($F177="","",IFERROR(VLOOKUP($F177,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10513,7 +10516,7 @@
         <x:f>IF($D178="","",IF($D178="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F178" s="53" t="str">
-        <x:f>IF($B178="","",IFERROR(VLOOKUP($B178,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B178="","",IFERROR(VLOOKUP($B178,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G178" s="65" t="str">
         <x:f>IF($F178="","",IFERROR(VLOOKUP($F178,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10566,7 +10569,7 @@
         <x:f>IF($D179="","",IF($D179="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F179" s="53" t="str">
-        <x:f>IF($B179="","",IFERROR(VLOOKUP($B179,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B179="","",IFERROR(VLOOKUP($B179,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G179" s="65" t="str">
         <x:f>IF($F179="","",IFERROR(VLOOKUP($F179,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10619,7 +10622,7 @@
         <x:f>IF($D180="","",IF($D180="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F180" s="53" t="str">
-        <x:f>IF($B180="","",IFERROR(VLOOKUP($B180,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B180="","",IFERROR(VLOOKUP($B180,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G180" s="65" t="str">
         <x:f>IF($F180="","",IFERROR(VLOOKUP($F180,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10672,7 +10675,7 @@
         <x:f>IF($D181="","",IF($D181="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F181" s="53" t="str">
-        <x:f>IF($B181="","",IFERROR(VLOOKUP($B181,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B181="","",IFERROR(VLOOKUP($B181,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G181" s="65" t="str">
         <x:f>IF($F181="","",IFERROR(VLOOKUP($F181,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10725,7 +10728,7 @@
         <x:f>IF($D182="","",IF($D182="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F182" s="53" t="str">
-        <x:f>IF($B182="","",IFERROR(VLOOKUP($B182,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B182="","",IFERROR(VLOOKUP($B182,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G182" s="65" t="str">
         <x:f>IF($F182="","",IFERROR(VLOOKUP($F182,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10778,7 +10781,7 @@
         <x:f>IF($D183="","",IF($D183="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F183" s="53" t="str">
-        <x:f>IF($B183="","",IFERROR(VLOOKUP($B183,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B183="","",IFERROR(VLOOKUP($B183,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G183" s="65" t="str">
         <x:f>IF($F183="","",IFERROR(VLOOKUP($F183,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10831,7 +10834,7 @@
         <x:f>IF($D184="","",IF($D184="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F184" s="53" t="str">
-        <x:f>IF($B184="","",IFERROR(VLOOKUP($B184,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B184="","",IFERROR(VLOOKUP($B184,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G184" s="65" t="str">
         <x:f>IF($F184="","",IFERROR(VLOOKUP($F184,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10884,7 +10887,7 @@
         <x:f>IF($D185="","",IF($D185="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F185" s="53" t="str">
-        <x:f>IF($B185="","",IFERROR(VLOOKUP($B185,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B185="","",IFERROR(VLOOKUP($B185,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G185" s="65" t="str">
         <x:f>IF($F185="","",IFERROR(VLOOKUP($F185,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10937,7 +10940,7 @@
         <x:f>IF($D186="","",IF($D186="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F186" s="53" t="str">
-        <x:f>IF($B186="","",IFERROR(VLOOKUP($B186,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B186="","",IFERROR(VLOOKUP($B186,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G186" s="65" t="str">
         <x:f>IF($F186="","",IFERROR(VLOOKUP($F186,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -10990,7 +10993,7 @@
         <x:f>IF($D187="","",IF($D187="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F187" s="53" t="str">
-        <x:f>IF($B187="","",IFERROR(VLOOKUP($B187,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B187="","",IFERROR(VLOOKUP($B187,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G187" s="65" t="str">
         <x:f>IF($F187="","",IFERROR(VLOOKUP($F187,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11043,7 +11046,7 @@
         <x:f>IF($D188="","",IF($D188="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F188" s="53" t="str">
-        <x:f>IF($B188="","",IFERROR(VLOOKUP($B188,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B188="","",IFERROR(VLOOKUP($B188,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G188" s="65" t="str">
         <x:f>IF($F188="","",IFERROR(VLOOKUP($F188,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11096,7 +11099,7 @@
         <x:f>IF($D189="","",IF($D189="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F189" s="53" t="str">
-        <x:f>IF($B189="","",IFERROR(VLOOKUP($B189,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B189="","",IFERROR(VLOOKUP($B189,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G189" s="65" t="str">
         <x:f>IF($F189="","",IFERROR(VLOOKUP($F189,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11149,7 +11152,7 @@
         <x:f>IF($D190="","",IF($D190="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F190" s="53" t="str">
-        <x:f>IF($B190="","",IFERROR(VLOOKUP($B190,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B190="","",IFERROR(VLOOKUP($B190,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G190" s="65" t="str">
         <x:f>IF($F190="","",IFERROR(VLOOKUP($F190,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11202,7 +11205,7 @@
         <x:f>IF($D191="","",IF($D191="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F191" s="53" t="str">
-        <x:f>IF($B191="","",IFERROR(VLOOKUP($B191,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B191="","",IFERROR(VLOOKUP($B191,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G191" s="65" t="str">
         <x:f>IF($F191="","",IFERROR(VLOOKUP($F191,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11255,7 +11258,7 @@
         <x:f>IF($D192="","",IF($D192="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F192" s="53" t="str">
-        <x:f>IF($B192="","",IFERROR(VLOOKUP($B192,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B192="","",IFERROR(VLOOKUP($B192,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G192" s="65" t="str">
         <x:f>IF($F192="","",IFERROR(VLOOKUP($F192,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11308,7 +11311,7 @@
         <x:f>IF($D193="","",IF($D193="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F193" s="53" t="str">
-        <x:f>IF($B193="","",IFERROR(VLOOKUP($B193,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B193="","",IFERROR(VLOOKUP($B193,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G193" s="65" t="str">
         <x:f>IF($F193="","",IFERROR(VLOOKUP($F193,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11361,7 +11364,7 @@
         <x:f>IF($D194="","",IF($D194="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F194" s="53" t="str">
-        <x:f>IF($B194="","",IFERROR(VLOOKUP($B194,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B194="","",IFERROR(VLOOKUP($B194,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G194" s="65" t="str">
         <x:f>IF($F194="","",IFERROR(VLOOKUP($F194,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11414,7 +11417,7 @@
         <x:f>IF($D195="","",IF($D195="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F195" s="53" t="str">
-        <x:f>IF($B195="","",IFERROR(VLOOKUP($B195,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B195="","",IFERROR(VLOOKUP($B195,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G195" s="65" t="str">
         <x:f>IF($F195="","",IFERROR(VLOOKUP($F195,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11467,7 +11470,7 @@
         <x:f>IF($D196="","",IF($D196="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F196" s="53" t="str">
-        <x:f>IF($B196="","",IFERROR(VLOOKUP($B196,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B196="","",IFERROR(VLOOKUP($B196,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G196" s="65" t="str">
         <x:f>IF($F196="","",IFERROR(VLOOKUP($F196,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11520,7 +11523,7 @@
         <x:f>IF($D197="","",IF($D197="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F197" s="53" t="str">
-        <x:f>IF($B197="","",IFERROR(VLOOKUP($B197,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B197="","",IFERROR(VLOOKUP($B197,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G197" s="65" t="str">
         <x:f>IF($F197="","",IFERROR(VLOOKUP($F197,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11573,7 +11576,7 @@
         <x:f>IF($D198="","",IF($D198="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F198" s="53" t="str">
-        <x:f>IF($B198="","",IFERROR(VLOOKUP($B198,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B198="","",IFERROR(VLOOKUP($B198,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G198" s="65" t="str">
         <x:f>IF($F198="","",IFERROR(VLOOKUP($F198,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11626,7 +11629,7 @@
         <x:f>IF($D199="","",IF($D199="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F199" s="53" t="str">
-        <x:f>IF($B199="","",IFERROR(VLOOKUP($B199,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B199="","",IFERROR(VLOOKUP($B199,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G199" s="65" t="str">
         <x:f>IF($F199="","",IFERROR(VLOOKUP($F199,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11679,7 +11682,7 @@
         <x:f>IF($D200="","",IF($D200="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F200" s="53" t="str">
-        <x:f>IF($B200="","",IFERROR(VLOOKUP($B200,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B200="","",IFERROR(VLOOKUP($B200,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G200" s="65" t="str">
         <x:f>IF($F200="","",IFERROR(VLOOKUP($F200,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11732,7 +11735,7 @@
         <x:f>IF($D201="","",IF($D201="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F201" s="53" t="str">
-        <x:f>IF($B201="","",IFERROR(VLOOKUP($B201,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B201="","",IFERROR(VLOOKUP($B201,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G201" s="65" t="str">
         <x:f>IF($F201="","",IFERROR(VLOOKUP($F201,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11785,7 +11788,7 @@
         <x:f>IF($D202="","",IF($D202="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F202" s="53" t="str">
-        <x:f>IF($B202="","",IFERROR(VLOOKUP($B202,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B202="","",IFERROR(VLOOKUP($B202,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G202" s="65" t="str">
         <x:f>IF($F202="","",IFERROR(VLOOKUP($F202,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11838,7 +11841,7 @@
         <x:f>IF($D203="","",IF($D203="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F203" s="53" t="str">
-        <x:f>IF($B203="","",IFERROR(VLOOKUP($B203,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B203="","",IFERROR(VLOOKUP($B203,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G203" s="65" t="str">
         <x:f>IF($F203="","",IFERROR(VLOOKUP($F203,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11891,7 +11894,7 @@
         <x:f>IF($D204="","",IF($D204="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F204" s="53" t="str">
-        <x:f>IF($B204="","",IFERROR(VLOOKUP($B204,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B204="","",IFERROR(VLOOKUP($B204,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G204" s="65" t="str">
         <x:f>IF($F204="","",IFERROR(VLOOKUP($F204,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11944,7 +11947,7 @@
         <x:f>IF($D205="","",IF($D205="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F205" s="53" t="str">
-        <x:f>IF($B205="","",IFERROR(VLOOKUP($B205,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B205="","",IFERROR(VLOOKUP($B205,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G205" s="65" t="str">
         <x:f>IF($F205="","",IFERROR(VLOOKUP($F205,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -11997,7 +12000,7 @@
         <x:f>IF($D206="","",IF($D206="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F206" s="53" t="str">
-        <x:f>IF($B206="","",IFERROR(VLOOKUP($B206,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B206="","",IFERROR(VLOOKUP($B206,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G206" s="65" t="str">
         <x:f>IF($F206="","",IFERROR(VLOOKUP($F206,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12050,7 +12053,7 @@
         <x:f>IF($D207="","",IF($D207="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F207" s="53" t="str">
-        <x:f>IF($B207="","",IFERROR(VLOOKUP($B207,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B207="","",IFERROR(VLOOKUP($B207,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G207" s="65" t="str">
         <x:f>IF($F207="","",IFERROR(VLOOKUP($F207,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12103,7 +12106,7 @@
         <x:f>IF($D208="","",IF($D208="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F208" s="53" t="str">
-        <x:f>IF($B208="","",IFERROR(VLOOKUP($B208,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B208="","",IFERROR(VLOOKUP($B208,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G208" s="65" t="str">
         <x:f>IF($F208="","",IFERROR(VLOOKUP($F208,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12156,7 +12159,7 @@
         <x:f>IF($D209="","",IF($D209="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F209" s="53" t="str">
-        <x:f>IF($B209="","",IFERROR(VLOOKUP($B209,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B209="","",IFERROR(VLOOKUP($B209,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G209" s="65" t="str">
         <x:f>IF($F209="","",IFERROR(VLOOKUP($F209,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12209,7 +12212,7 @@
         <x:f>IF($D210="","",IF($D210="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F210" s="53" t="str">
-        <x:f>IF($B210="","",IFERROR(VLOOKUP($B210,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B210="","",IFERROR(VLOOKUP($B210,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G210" s="65" t="str">
         <x:f>IF($F210="","",IFERROR(VLOOKUP($F210,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12262,7 +12265,7 @@
         <x:f>IF($D211="","",IF($D211="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F211" s="53" t="str">
-        <x:f>IF($B211="","",IFERROR(VLOOKUP($B211,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B211="","",IFERROR(VLOOKUP($B211,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G211" s="65" t="str">
         <x:f>IF($F211="","",IFERROR(VLOOKUP($F211,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12315,7 +12318,7 @@
         <x:f>IF($D212="","",IF($D212="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F212" s="53" t="str">
-        <x:f>IF($B212="","",IFERROR(VLOOKUP($B212,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B212="","",IFERROR(VLOOKUP($B212,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G212" s="65" t="str">
         <x:f>IF($F212="","",IFERROR(VLOOKUP($F212,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12368,7 +12371,7 @@
         <x:f>IF($D213="","",IF($D213="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F213" s="53" t="str">
-        <x:f>IF($B213="","",IFERROR(VLOOKUP($B213,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B213="","",IFERROR(VLOOKUP($B213,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G213" s="65" t="str">
         <x:f>IF($F213="","",IFERROR(VLOOKUP($F213,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12421,7 +12424,7 @@
         <x:f>IF($D214="","",IF($D214="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F214" s="53" t="str">
-        <x:f>IF($B214="","",IFERROR(VLOOKUP($B214,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B214="","",IFERROR(VLOOKUP($B214,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G214" s="65" t="str">
         <x:f>IF($F214="","",IFERROR(VLOOKUP($F214,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12474,7 +12477,7 @@
         <x:f>IF($D215="","",IF($D215="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F215" s="53" t="str">
-        <x:f>IF($B215="","",IFERROR(VLOOKUP($B215,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B215="","",IFERROR(VLOOKUP($B215,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G215" s="65" t="str">
         <x:f>IF($F215="","",IFERROR(VLOOKUP($F215,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12527,7 +12530,7 @@
         <x:f>IF($D216="","",IF($D216="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F216" s="53" t="str">
-        <x:f>IF($B216="","",IFERROR(VLOOKUP($B216,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B216="","",IFERROR(VLOOKUP($B216,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G216" s="65" t="str">
         <x:f>IF($F216="","",IFERROR(VLOOKUP($F216,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12580,7 +12583,7 @@
         <x:f>IF($D217="","",IF($D217="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F217" s="53" t="str">
-        <x:f>IF($B217="","",IFERROR(VLOOKUP($B217,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B217="","",IFERROR(VLOOKUP($B217,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G217" s="65" t="str">
         <x:f>IF($F217="","",IFERROR(VLOOKUP($F217,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12633,7 +12636,7 @@
         <x:f>IF($D218="","",IF($D218="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F218" s="53" t="str">
-        <x:f>IF($B218="","",IFERROR(VLOOKUP($B218,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B218="","",IFERROR(VLOOKUP($B218,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G218" s="65" t="str">
         <x:f>IF($F218="","",IFERROR(VLOOKUP($F218,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12686,7 +12689,7 @@
         <x:f>IF($D219="","",IF($D219="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F219" s="53" t="str">
-        <x:f>IF($B219="","",IFERROR(VLOOKUP($B219,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B219="","",IFERROR(VLOOKUP($B219,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G219" s="65" t="str">
         <x:f>IF($F219="","",IFERROR(VLOOKUP($F219,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12739,7 +12742,7 @@
         <x:f>IF($D220="","",IF($D220="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F220" s="53" t="str">
-        <x:f>IF($B220="","",IFERROR(VLOOKUP($B220,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B220="","",IFERROR(VLOOKUP($B220,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G220" s="65" t="str">
         <x:f>IF($F220="","",IFERROR(VLOOKUP($F220,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12792,7 +12795,7 @@
         <x:f>IF($D221="","",IF($D221="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F221" s="53" t="str">
-        <x:f>IF($B221="","",IFERROR(VLOOKUP($B221,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B221="","",IFERROR(VLOOKUP($B221,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G221" s="65" t="str">
         <x:f>IF($F221="","",IFERROR(VLOOKUP($F221,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12845,7 +12848,7 @@
         <x:f>IF($D222="","",IF($D222="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F222" s="53" t="str">
-        <x:f>IF($B222="","",IFERROR(VLOOKUP($B222,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B222="","",IFERROR(VLOOKUP($B222,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G222" s="65" t="str">
         <x:f>IF($F222="","",IFERROR(VLOOKUP($F222,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12898,7 +12901,7 @@
         <x:f>IF($D223="","",IF($D223="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F223" s="53" t="str">
-        <x:f>IF($B223="","",IFERROR(VLOOKUP($B223,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B223="","",IFERROR(VLOOKUP($B223,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G223" s="65" t="str">
         <x:f>IF($F223="","",IFERROR(VLOOKUP($F223,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -12951,7 +12954,7 @@
         <x:f>IF($D224="","",IF($D224="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F224" s="53" t="str">
-        <x:f>IF($B224="","",IFERROR(VLOOKUP($B224,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B224="","",IFERROR(VLOOKUP($B224,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G224" s="65" t="str">
         <x:f>IF($F224="","",IFERROR(VLOOKUP($F224,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13004,7 +13007,7 @@
         <x:f>IF($D225="","",IF($D225="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F225" s="53" t="str">
-        <x:f>IF($B225="","",IFERROR(VLOOKUP($B225,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B225="","",IFERROR(VLOOKUP($B225,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G225" s="65" t="str">
         <x:f>IF($F225="","",IFERROR(VLOOKUP($F225,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13057,7 +13060,7 @@
         <x:f>IF($D226="","",IF($D226="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F226" s="53" t="str">
-        <x:f>IF($B226="","",IFERROR(VLOOKUP($B226,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B226="","",IFERROR(VLOOKUP($B226,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G226" s="65" t="str">
         <x:f>IF($F226="","",IFERROR(VLOOKUP($F226,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13110,7 +13113,7 @@
         <x:f>IF($D227="","",IF($D227="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F227" s="53" t="str">
-        <x:f>IF($B227="","",IFERROR(VLOOKUP($B227,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B227="","",IFERROR(VLOOKUP($B227,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G227" s="65" t="str">
         <x:f>IF($F227="","",IFERROR(VLOOKUP($F227,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13163,7 +13166,7 @@
         <x:f>IF($D228="","",IF($D228="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F228" s="53" t="str">
-        <x:f>IF($B228="","",IFERROR(VLOOKUP($B228,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B228="","",IFERROR(VLOOKUP($B228,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G228" s="65" t="str">
         <x:f>IF($F228="","",IFERROR(VLOOKUP($F228,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13216,7 +13219,7 @@
         <x:f>IF($D229="","",IF($D229="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F229" s="53" t="str">
-        <x:f>IF($B229="","",IFERROR(VLOOKUP($B229,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B229="","",IFERROR(VLOOKUP($B229,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G229" s="65" t="str">
         <x:f>IF($F229="","",IFERROR(VLOOKUP($F229,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13269,7 +13272,7 @@
         <x:f>IF($D230="","",IF($D230="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F230" s="53" t="str">
-        <x:f>IF($B230="","",IFERROR(VLOOKUP($B230,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B230="","",IFERROR(VLOOKUP($B230,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G230" s="65" t="str">
         <x:f>IF($F230="","",IFERROR(VLOOKUP($F230,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13322,7 +13325,7 @@
         <x:f>IF($D231="","",IF($D231="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F231" s="53" t="str">
-        <x:f>IF($B231="","",IFERROR(VLOOKUP($B231,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B231="","",IFERROR(VLOOKUP($B231,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G231" s="65" t="str">
         <x:f>IF($F231="","",IFERROR(VLOOKUP($F231,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13375,7 +13378,7 @@
         <x:f>IF($D232="","",IF($D232="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F232" s="53" t="str">
-        <x:f>IF($B232="","",IFERROR(VLOOKUP($B232,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B232="","",IFERROR(VLOOKUP($B232,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G232" s="65" t="str">
         <x:f>IF($F232="","",IFERROR(VLOOKUP($F232,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13428,7 +13431,7 @@
         <x:f>IF($D233="","",IF($D233="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F233" s="53" t="str">
-        <x:f>IF($B233="","",IFERROR(VLOOKUP($B233,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B233="","",IFERROR(VLOOKUP($B233,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G233" s="65" t="str">
         <x:f>IF($F233="","",IFERROR(VLOOKUP($F233,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13481,7 +13484,7 @@
         <x:f>IF($D234="","",IF($D234="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F234" s="53" t="str">
-        <x:f>IF($B234="","",IFERROR(VLOOKUP($B234,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B234="","",IFERROR(VLOOKUP($B234,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G234" s="65" t="str">
         <x:f>IF($F234="","",IFERROR(VLOOKUP($F234,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13534,7 +13537,7 @@
         <x:f>IF($D235="","",IF($D235="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F235" s="53" t="str">
-        <x:f>IF($B235="","",IFERROR(VLOOKUP($B235,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B235="","",IFERROR(VLOOKUP($B235,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G235" s="65" t="str">
         <x:f>IF($F235="","",IFERROR(VLOOKUP($F235,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13587,7 +13590,7 @@
         <x:f>IF($D236="","",IF($D236="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F236" s="53" t="str">
-        <x:f>IF($B236="","",IFERROR(VLOOKUP($B236,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B236="","",IFERROR(VLOOKUP($B236,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G236" s="65" t="str">
         <x:f>IF($F236="","",IFERROR(VLOOKUP($F236,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13640,7 +13643,7 @@
         <x:f>IF($D237="","",IF($D237="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F237" s="53" t="str">
-        <x:f>IF($B237="","",IFERROR(VLOOKUP($B237,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B237="","",IFERROR(VLOOKUP($B237,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G237" s="65" t="str">
         <x:f>IF($F237="","",IFERROR(VLOOKUP($F237,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13693,7 +13696,7 @@
         <x:f>IF($D238="","",IF($D238="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F238" s="53" t="str">
-        <x:f>IF($B238="","",IFERROR(VLOOKUP($B238,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B238="","",IFERROR(VLOOKUP($B238,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G238" s="65" t="str">
         <x:f>IF($F238="","",IFERROR(VLOOKUP($F238,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13746,7 +13749,7 @@
         <x:f>IF($D239="","",IF($D239="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F239" s="53" t="str">
-        <x:f>IF($B239="","",IFERROR(VLOOKUP($B239,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B239="","",IFERROR(VLOOKUP($B239,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G239" s="65" t="str">
         <x:f>IF($F239="","",IFERROR(VLOOKUP($F239,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13799,7 +13802,7 @@
         <x:f>IF($D240="","",IF($D240="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F240" s="53" t="str">
-        <x:f>IF($B240="","",IFERROR(VLOOKUP($B240,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B240="","",IFERROR(VLOOKUP($B240,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G240" s="65" t="str">
         <x:f>IF($F240="","",IFERROR(VLOOKUP($F240,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13852,7 +13855,7 @@
         <x:f>IF($D241="","",IF($D241="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F241" s="53" t="str">
-        <x:f>IF($B241="","",IFERROR(VLOOKUP($B241,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B241="","",IFERROR(VLOOKUP($B241,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G241" s="65" t="str">
         <x:f>IF($F241="","",IFERROR(VLOOKUP($F241,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13905,7 +13908,7 @@
         <x:f>IF($D242="","",IF($D242="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F242" s="53" t="str">
-        <x:f>IF($B242="","",IFERROR(VLOOKUP($B242,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B242="","",IFERROR(VLOOKUP($B242,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G242" s="65" t="str">
         <x:f>IF($F242="","",IFERROR(VLOOKUP($F242,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -13958,7 +13961,7 @@
         <x:f>IF($D243="","",IF($D243="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F243" s="53" t="str">
-        <x:f>IF($B243="","",IFERROR(VLOOKUP($B243,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B243="","",IFERROR(VLOOKUP($B243,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G243" s="65" t="str">
         <x:f>IF($F243="","",IFERROR(VLOOKUP($F243,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14011,7 +14014,7 @@
         <x:f>IF($D244="","",IF($D244="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F244" s="53" t="str">
-        <x:f>IF($B244="","",IFERROR(VLOOKUP($B244,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B244="","",IFERROR(VLOOKUP($B244,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G244" s="65" t="str">
         <x:f>IF($F244="","",IFERROR(VLOOKUP($F244,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14064,7 +14067,7 @@
         <x:f>IF($D245="","",IF($D245="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F245" s="53" t="str">
-        <x:f>IF($B245="","",IFERROR(VLOOKUP($B245,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B245="","",IFERROR(VLOOKUP($B245,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G245" s="65" t="str">
         <x:f>IF($F245="","",IFERROR(VLOOKUP($F245,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14117,7 +14120,7 @@
         <x:f>IF($D246="","",IF($D246="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F246" s="53" t="str">
-        <x:f>IF($B246="","",IFERROR(VLOOKUP($B246,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B246="","",IFERROR(VLOOKUP($B246,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G246" s="65" t="str">
         <x:f>IF($F246="","",IFERROR(VLOOKUP($F246,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14170,7 +14173,7 @@
         <x:f>IF($D247="","",IF($D247="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F247" s="53" t="str">
-        <x:f>IF($B247="","",IFERROR(VLOOKUP($B247,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B247="","",IFERROR(VLOOKUP($B247,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G247" s="65" t="str">
         <x:f>IF($F247="","",IFERROR(VLOOKUP($F247,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14223,7 +14226,7 @@
         <x:f>IF($D248="","",IF($D248="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F248" s="53" t="str">
-        <x:f>IF($B248="","",IFERROR(VLOOKUP($B248,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B248="","",IFERROR(VLOOKUP($B248,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G248" s="65" t="str">
         <x:f>IF($F248="","",IFERROR(VLOOKUP($F248,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14276,7 +14279,7 @@
         <x:f>IF($D249="","",IF($D249="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F249" s="53" t="str">
-        <x:f>IF($B249="","",IFERROR(VLOOKUP($B249,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B249="","",IFERROR(VLOOKUP($B249,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G249" s="65" t="str">
         <x:f>IF($F249="","",IFERROR(VLOOKUP($F249,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14329,7 +14332,7 @@
         <x:f>IF($D250="","",IF($D250="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F250" s="53" t="str">
-        <x:f>IF($B250="","",IFERROR(VLOOKUP($B250,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B250="","",IFERROR(VLOOKUP($B250,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G250" s="65" t="str">
         <x:f>IF($F250="","",IFERROR(VLOOKUP($F250,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14382,7 +14385,7 @@
         <x:f>IF($D251="","",IF($D251="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F251" s="53" t="str">
-        <x:f>IF($B251="","",IFERROR(VLOOKUP($B251,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B251="","",IFERROR(VLOOKUP($B251,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G251" s="65" t="str">
         <x:f>IF($F251="","",IFERROR(VLOOKUP($F251,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14435,7 +14438,7 @@
         <x:f>IF($D252="","",IF($D252="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F252" s="53" t="str">
-        <x:f>IF($B252="","",IFERROR(VLOOKUP($B252,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B252="","",IFERROR(VLOOKUP($B252,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G252" s="65" t="str">
         <x:f>IF($F252="","",IFERROR(VLOOKUP($F252,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14488,7 +14491,7 @@
         <x:f>IF($D253="","",IF($D253="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F253" s="53" t="str">
-        <x:f>IF($B253="","",IFERROR(VLOOKUP($B253,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B253="","",IFERROR(VLOOKUP($B253,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G253" s="65" t="str">
         <x:f>IF($F253="","",IFERROR(VLOOKUP($F253,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14541,7 +14544,7 @@
         <x:f>IF($D254="","",IF($D254="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F254" s="53" t="str">
-        <x:f>IF($B254="","",IFERROR(VLOOKUP($B254,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B254="","",IFERROR(VLOOKUP($B254,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G254" s="65" t="str">
         <x:f>IF($F254="","",IFERROR(VLOOKUP($F254,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14594,7 +14597,7 @@
         <x:f>IF($D255="","",IF($D255="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F255" s="53" t="str">
-        <x:f>IF($B255="","",IFERROR(VLOOKUP($B255,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B255="","",IFERROR(VLOOKUP($B255,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G255" s="65" t="str">
         <x:f>IF($F255="","",IFERROR(VLOOKUP($F255,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14647,7 +14650,7 @@
         <x:f>IF($D256="","",IF($D256="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F256" s="53" t="str">
-        <x:f>IF($B256="","",IFERROR(VLOOKUP($B256,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B256="","",IFERROR(VLOOKUP($B256,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G256" s="65" t="str">
         <x:f>IF($F256="","",IFERROR(VLOOKUP($F256,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14700,7 +14703,7 @@
         <x:f>IF($D257="","",IF($D257="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F257" s="53" t="str">
-        <x:f>IF($B257="","",IFERROR(VLOOKUP($B257,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B257="","",IFERROR(VLOOKUP($B257,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G257" s="65" t="str">
         <x:f>IF($F257="","",IFERROR(VLOOKUP($F257,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14753,7 +14756,7 @@
         <x:f>IF($D258="","",IF($D258="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F258" s="53" t="str">
-        <x:f>IF($B258="","",IFERROR(VLOOKUP($B258,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B258="","",IFERROR(VLOOKUP($B258,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G258" s="65" t="str">
         <x:f>IF($F258="","",IFERROR(VLOOKUP($F258,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14806,7 +14809,7 @@
         <x:f>IF($D259="","",IF($D259="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F259" s="53" t="str">
-        <x:f>IF($B259="","",IFERROR(VLOOKUP($B259,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B259="","",IFERROR(VLOOKUP($B259,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G259" s="65" t="str">
         <x:f>IF($F259="","",IFERROR(VLOOKUP($F259,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14859,7 +14862,7 @@
         <x:f>IF($D260="","",IF($D260="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F260" s="53" t="str">
-        <x:f>IF($B260="","",IFERROR(VLOOKUP($B260,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B260="","",IFERROR(VLOOKUP($B260,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G260" s="65" t="str">
         <x:f>IF($F260="","",IFERROR(VLOOKUP($F260,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14912,7 +14915,7 @@
         <x:f>IF($D261="","",IF($D261="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F261" s="53" t="str">
-        <x:f>IF($B261="","",IFERROR(VLOOKUP($B261,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B261="","",IFERROR(VLOOKUP($B261,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G261" s="65" t="str">
         <x:f>IF($F261="","",IFERROR(VLOOKUP($F261,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -14965,7 +14968,7 @@
         <x:f>IF($D262="","",IF($D262="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F262" s="53" t="str">
-        <x:f>IF($B262="","",IFERROR(VLOOKUP($B262,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B262="","",IFERROR(VLOOKUP($B262,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G262" s="65" t="str">
         <x:f>IF($F262="","",IFERROR(VLOOKUP($F262,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15018,7 +15021,7 @@
         <x:f>IF($D263="","",IF($D263="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F263" s="53" t="str">
-        <x:f>IF($B263="","",IFERROR(VLOOKUP($B263,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B263="","",IFERROR(VLOOKUP($B263,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G263" s="65" t="str">
         <x:f>IF($F263="","",IFERROR(VLOOKUP($F263,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15071,7 +15074,7 @@
         <x:f>IF($D264="","",IF($D264="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F264" s="53" t="str">
-        <x:f>IF($B264="","",IFERROR(VLOOKUP($B264,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B264="","",IFERROR(VLOOKUP($B264,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G264" s="65" t="str">
         <x:f>IF($F264="","",IFERROR(VLOOKUP($F264,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15124,7 +15127,7 @@
         <x:f>IF($D265="","",IF($D265="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F265" s="53" t="str">
-        <x:f>IF($B265="","",IFERROR(VLOOKUP($B265,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B265="","",IFERROR(VLOOKUP($B265,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G265" s="65" t="str">
         <x:f>IF($F265="","",IFERROR(VLOOKUP($F265,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15177,7 +15180,7 @@
         <x:f>IF($D266="","",IF($D266="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F266" s="53" t="str">
-        <x:f>IF($B266="","",IFERROR(VLOOKUP($B266,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B266="","",IFERROR(VLOOKUP($B266,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G266" s="65" t="str">
         <x:f>IF($F266="","",IFERROR(VLOOKUP($F266,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15230,7 +15233,7 @@
         <x:f>IF($D267="","",IF($D267="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F267" s="53" t="str">
-        <x:f>IF($B267="","",IFERROR(VLOOKUP($B267,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B267="","",IFERROR(VLOOKUP($B267,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G267" s="65" t="str">
         <x:f>IF($F267="","",IFERROR(VLOOKUP($F267,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15283,7 +15286,7 @@
         <x:f>IF($D268="","",IF($D268="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F268" s="53" t="str">
-        <x:f>IF($B268="","",IFERROR(VLOOKUP($B268,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B268="","",IFERROR(VLOOKUP($B268,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G268" s="65" t="str">
         <x:f>IF($F268="","",IFERROR(VLOOKUP($F268,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15336,7 +15339,7 @@
         <x:f>IF($D269="","",IF($D269="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F269" s="53" t="str">
-        <x:f>IF($B269="","",IFERROR(VLOOKUP($B269,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B269="","",IFERROR(VLOOKUP($B269,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G269" s="65" t="str">
         <x:f>IF($F269="","",IFERROR(VLOOKUP($F269,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15389,7 +15392,7 @@
         <x:f>IF($D270="","",IF($D270="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F270" s="53" t="str">
-        <x:f>IF($B270="","",IFERROR(VLOOKUP($B270,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B270="","",IFERROR(VLOOKUP($B270,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G270" s="65" t="str">
         <x:f>IF($F270="","",IFERROR(VLOOKUP($F270,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15442,7 +15445,7 @@
         <x:f>IF($D271="","",IF($D271="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F271" s="53" t="str">
-        <x:f>IF($B271="","",IFERROR(VLOOKUP($B271,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B271="","",IFERROR(VLOOKUP($B271,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G271" s="65" t="str">
         <x:f>IF($F271="","",IFERROR(VLOOKUP($F271,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15495,7 +15498,7 @@
         <x:f>IF($D272="","",IF($D272="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F272" s="53" t="str">
-        <x:f>IF($B272="","",IFERROR(VLOOKUP($B272,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B272="","",IFERROR(VLOOKUP($B272,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G272" s="65" t="str">
         <x:f>IF($F272="","",IFERROR(VLOOKUP($F272,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15548,7 +15551,7 @@
         <x:f>IF($D273="","",IF($D273="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F273" s="53" t="str">
-        <x:f>IF($B273="","",IFERROR(VLOOKUP($B273,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B273="","",IFERROR(VLOOKUP($B273,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G273" s="65" t="str">
         <x:f>IF($F273="","",IFERROR(VLOOKUP($F273,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15601,7 +15604,7 @@
         <x:f>IF($D274="","",IF($D274="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F274" s="53" t="str">
-        <x:f>IF($B274="","",IFERROR(VLOOKUP($B274,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B274="","",IFERROR(VLOOKUP($B274,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G274" s="65" t="str">
         <x:f>IF($F274="","",IFERROR(VLOOKUP($F274,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15654,7 +15657,7 @@
         <x:f>IF($D275="","",IF($D275="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F275" s="53" t="str">
-        <x:f>IF($B275="","",IFERROR(VLOOKUP($B275,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B275="","",IFERROR(VLOOKUP($B275,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G275" s="65" t="str">
         <x:f>IF($F275="","",IFERROR(VLOOKUP($F275,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15707,7 +15710,7 @@
         <x:f>IF($D276="","",IF($D276="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F276" s="53" t="str">
-        <x:f>IF($B276="","",IFERROR(VLOOKUP($B276,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B276="","",IFERROR(VLOOKUP($B276,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G276" s="65" t="str">
         <x:f>IF($F276="","",IFERROR(VLOOKUP($F276,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15760,7 +15763,7 @@
         <x:f>IF($D277="","",IF($D277="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F277" s="53" t="str">
-        <x:f>IF($B277="","",IFERROR(VLOOKUP($B277,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B277="","",IFERROR(VLOOKUP($B277,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G277" s="65" t="str">
         <x:f>IF($F277="","",IFERROR(VLOOKUP($F277,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15813,7 +15816,7 @@
         <x:f>IF($D278="","",IF($D278="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F278" s="53" t="str">
-        <x:f>IF($B278="","",IFERROR(VLOOKUP($B278,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B278="","",IFERROR(VLOOKUP($B278,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G278" s="65" t="str">
         <x:f>IF($F278="","",IFERROR(VLOOKUP($F278,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15866,7 +15869,7 @@
         <x:f>IF($D279="","",IF($D279="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F279" s="53" t="str">
-        <x:f>IF($B279="","",IFERROR(VLOOKUP($B279,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B279="","",IFERROR(VLOOKUP($B279,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G279" s="65" t="str">
         <x:f>IF($F279="","",IFERROR(VLOOKUP($F279,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15919,7 +15922,7 @@
         <x:f>IF($D280="","",IF($D280="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F280" s="53" t="str">
-        <x:f>IF($B280="","",IFERROR(VLOOKUP($B280,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B280="","",IFERROR(VLOOKUP($B280,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G280" s="65" t="str">
         <x:f>IF($F280="","",IFERROR(VLOOKUP($F280,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -15972,7 +15975,7 @@
         <x:f>IF($D281="","",IF($D281="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F281" s="53" t="str">
-        <x:f>IF($B281="","",IFERROR(VLOOKUP($B281,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B281="","",IFERROR(VLOOKUP($B281,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G281" s="65" t="str">
         <x:f>IF($F281="","",IFERROR(VLOOKUP($F281,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16025,7 +16028,7 @@
         <x:f>IF($D282="","",IF($D282="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F282" s="53" t="str">
-        <x:f>IF($B282="","",IFERROR(VLOOKUP($B282,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B282="","",IFERROR(VLOOKUP($B282,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G282" s="65" t="str">
         <x:f>IF($F282="","",IFERROR(VLOOKUP($F282,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16078,7 +16081,7 @@
         <x:f>IF($D283="","",IF($D283="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F283" s="53" t="str">
-        <x:f>IF($B283="","",IFERROR(VLOOKUP($B283,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B283="","",IFERROR(VLOOKUP($B283,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G283" s="65" t="str">
         <x:f>IF($F283="","",IFERROR(VLOOKUP($F283,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16131,7 +16134,7 @@
         <x:f>IF($D284="","",IF($D284="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F284" s="53" t="str">
-        <x:f>IF($B284="","",IFERROR(VLOOKUP($B284,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B284="","",IFERROR(VLOOKUP($B284,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G284" s="65" t="str">
         <x:f>IF($F284="","",IFERROR(VLOOKUP($F284,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16184,7 +16187,7 @@
         <x:f>IF($D285="","",IF($D285="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F285" s="53" t="str">
-        <x:f>IF($B285="","",IFERROR(VLOOKUP($B285,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B285="","",IFERROR(VLOOKUP($B285,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G285" s="65" t="str">
         <x:f>IF($F285="","",IFERROR(VLOOKUP($F285,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16237,7 +16240,7 @@
         <x:f>IF($D286="","",IF($D286="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F286" s="53" t="str">
-        <x:f>IF($B286="","",IFERROR(VLOOKUP($B286,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B286="","",IFERROR(VLOOKUP($B286,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G286" s="65" t="str">
         <x:f>IF($F286="","",IFERROR(VLOOKUP($F286,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16290,7 +16293,7 @@
         <x:f>IF($D287="","",IF($D287="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F287" s="53" t="str">
-        <x:f>IF($B287="","",IFERROR(VLOOKUP($B287,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B287="","",IFERROR(VLOOKUP($B287,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G287" s="65" t="str">
         <x:f>IF($F287="","",IFERROR(VLOOKUP($F287,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16343,7 +16346,7 @@
         <x:f>IF($D288="","",IF($D288="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F288" s="53" t="str">
-        <x:f>IF($B288="","",IFERROR(VLOOKUP($B288,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B288="","",IFERROR(VLOOKUP($B288,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G288" s="65" t="str">
         <x:f>IF($F288="","",IFERROR(VLOOKUP($F288,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16396,7 +16399,7 @@
         <x:f>IF($D289="","",IF($D289="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F289" s="53" t="str">
-        <x:f>IF($B289="","",IFERROR(VLOOKUP($B289,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B289="","",IFERROR(VLOOKUP($B289,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G289" s="65" t="str">
         <x:f>IF($F289="","",IFERROR(VLOOKUP($F289,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16449,7 +16452,7 @@
         <x:f>IF($D290="","",IF($D290="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F290" s="53" t="str">
-        <x:f>IF($B290="","",IFERROR(VLOOKUP($B290,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B290="","",IFERROR(VLOOKUP($B290,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G290" s="65" t="str">
         <x:f>IF($F290="","",IFERROR(VLOOKUP($F290,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16502,7 +16505,7 @@
         <x:f>IF($D291="","",IF($D291="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F291" s="53" t="str">
-        <x:f>IF($B291="","",IFERROR(VLOOKUP($B291,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B291="","",IFERROR(VLOOKUP($B291,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G291" s="65" t="str">
         <x:f>IF($F291="","",IFERROR(VLOOKUP($F291,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16555,7 +16558,7 @@
         <x:f>IF($D292="","",IF($D292="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F292" s="53" t="str">
-        <x:f>IF($B292="","",IFERROR(VLOOKUP($B292,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B292="","",IFERROR(VLOOKUP($B292,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G292" s="65" t="str">
         <x:f>IF($F292="","",IFERROR(VLOOKUP($F292,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16608,7 +16611,7 @@
         <x:f>IF($D293="","",IF($D293="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F293" s="53" t="str">
-        <x:f>IF($B293="","",IFERROR(VLOOKUP($B293,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B293="","",IFERROR(VLOOKUP($B293,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G293" s="65" t="str">
         <x:f>IF($F293="","",IFERROR(VLOOKUP($F293,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16661,7 +16664,7 @@
         <x:f>IF($D294="","",IF($D294="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F294" s="53" t="str">
-        <x:f>IF($B294="","",IFERROR(VLOOKUP($B294,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B294="","",IFERROR(VLOOKUP($B294,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G294" s="65" t="str">
         <x:f>IF($F294="","",IFERROR(VLOOKUP($F294,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16714,7 +16717,7 @@
         <x:f>IF($D295="","",IF($D295="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F295" s="53" t="str">
-        <x:f>IF($B295="","",IFERROR(VLOOKUP($B295,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B295="","",IFERROR(VLOOKUP($B295,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G295" s="65" t="str">
         <x:f>IF($F295="","",IFERROR(VLOOKUP($F295,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16767,7 +16770,7 @@
         <x:f>IF($D296="","",IF($D296="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F296" s="53" t="str">
-        <x:f>IF($B296="","",IFERROR(VLOOKUP($B296,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B296="","",IFERROR(VLOOKUP($B296,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G296" s="65" t="str">
         <x:f>IF($F296="","",IFERROR(VLOOKUP($F296,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16820,7 +16823,7 @@
         <x:f>IF($D297="","",IF($D297="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F297" s="53" t="str">
-        <x:f>IF($B297="","",IFERROR(VLOOKUP($B297,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B297="","",IFERROR(VLOOKUP($B297,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G297" s="65" t="str">
         <x:f>IF($F297="","",IFERROR(VLOOKUP($F297,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16873,7 +16876,7 @@
         <x:f>IF($D298="","",IF($D298="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F298" s="53" t="str">
-        <x:f>IF($B298="","",IFERROR(VLOOKUP($B298,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B298="","",IFERROR(VLOOKUP($B298,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G298" s="65" t="str">
         <x:f>IF($F298="","",IFERROR(VLOOKUP($F298,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16926,7 +16929,7 @@
         <x:f>IF($D299="","",IF($D299="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F299" s="53" t="str">
-        <x:f>IF($B299="","",IFERROR(VLOOKUP($B299,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B299="","",IFERROR(VLOOKUP($B299,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G299" s="65" t="str">
         <x:f>IF($F299="","",IFERROR(VLOOKUP($F299,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -16979,7 +16982,7 @@
         <x:f>IF($D300="","",IF($D300="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F300" s="53" t="str">
-        <x:f>IF($B300="","",IFERROR(VLOOKUP($B300,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B300="","",IFERROR(VLOOKUP($B300,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G300" s="65" t="str">
         <x:f>IF($F300="","",IFERROR(VLOOKUP($F300,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17032,7 +17035,7 @@
         <x:f>IF($D301="","",IF($D301="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F301" s="53" t="str">
-        <x:f>IF($B301="","",IFERROR(VLOOKUP($B301,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B301="","",IFERROR(VLOOKUP($B301,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G301" s="65" t="str">
         <x:f>IF($F301="","",IFERROR(VLOOKUP($F301,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17085,7 +17088,7 @@
         <x:f>IF($D302="","",IF($D302="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F302" s="53" t="str">
-        <x:f>IF($B302="","",IFERROR(VLOOKUP($B302,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B302="","",IFERROR(VLOOKUP($B302,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G302" s="65" t="str">
         <x:f>IF($F302="","",IFERROR(VLOOKUP($F302,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17138,7 +17141,7 @@
         <x:f>IF($D303="","",IF($D303="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F303" s="53" t="str">
-        <x:f>IF($B303="","",IFERROR(VLOOKUP($B303,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B303="","",IFERROR(VLOOKUP($B303,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G303" s="65" t="str">
         <x:f>IF($F303="","",IFERROR(VLOOKUP($F303,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17191,7 +17194,7 @@
         <x:f>IF($D304="","",IF($D304="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F304" s="53" t="str">
-        <x:f>IF($B304="","",IFERROR(VLOOKUP($B304,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B304="","",IFERROR(VLOOKUP($B304,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G304" s="65" t="str">
         <x:f>IF($F304="","",IFERROR(VLOOKUP($F304,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17244,7 +17247,7 @@
         <x:f>IF($D305="","",IF($D305="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F305" s="53" t="str">
-        <x:f>IF($B305="","",IFERROR(VLOOKUP($B305,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B305="","",IFERROR(VLOOKUP($B305,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G305" s="65" t="str">
         <x:f>IF($F305="","",IFERROR(VLOOKUP($F305,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17297,7 +17300,7 @@
         <x:f>IF($D306="","",IF($D306="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F306" s="53" t="str">
-        <x:f>IF($B306="","",IFERROR(VLOOKUP($B306,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B306="","",IFERROR(VLOOKUP($B306,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G306" s="65" t="str">
         <x:f>IF($F306="","",IFERROR(VLOOKUP($F306,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17350,7 +17353,7 @@
         <x:f>IF($D307="","",IF($D307="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F307" s="53" t="str">
-        <x:f>IF($B307="","",IFERROR(VLOOKUP($B307,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B307="","",IFERROR(VLOOKUP($B307,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G307" s="65" t="str">
         <x:f>IF($F307="","",IFERROR(VLOOKUP($F307,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17403,7 +17406,7 @@
         <x:f>IF($D308="","",IF($D308="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F308" s="53" t="str">
-        <x:f>IF($B308="","",IFERROR(VLOOKUP($B308,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B308="","",IFERROR(VLOOKUP($B308,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G308" s="65" t="str">
         <x:f>IF($F308="","",IFERROR(VLOOKUP($F308,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17456,7 +17459,7 @@
         <x:f>IF($D309="","",IF($D309="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F309" s="53" t="str">
-        <x:f>IF($B309="","",IFERROR(VLOOKUP($B309,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B309="","",IFERROR(VLOOKUP($B309,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G309" s="65" t="str">
         <x:f>IF($F309="","",IFERROR(VLOOKUP($F309,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17509,7 +17512,7 @@
         <x:f>IF($D310="","",IF($D310="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F310" s="53" t="str">
-        <x:f>IF($B310="","",IFERROR(VLOOKUP($B310,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B310="","",IFERROR(VLOOKUP($B310,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G310" s="65" t="str">
         <x:f>IF($F310="","",IFERROR(VLOOKUP($F310,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17562,7 +17565,7 @@
         <x:f>IF($D311="","",IF($D311="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F311" s="53" t="str">
-        <x:f>IF($B311="","",IFERROR(VLOOKUP($B311,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B311="","",IFERROR(VLOOKUP($B311,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G311" s="65" t="str">
         <x:f>IF($F311="","",IFERROR(VLOOKUP($F311,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17615,7 +17618,7 @@
         <x:f>IF($D312="","",IF($D312="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F312" s="53" t="str">
-        <x:f>IF($B312="","",IFERROR(VLOOKUP($B312,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B312="","",IFERROR(VLOOKUP($B312,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G312" s="65" t="str">
         <x:f>IF($F312="","",IFERROR(VLOOKUP($F312,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17668,7 +17671,7 @@
         <x:f>IF($D313="","",IF($D313="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F313" s="53" t="str">
-        <x:f>IF($B313="","",IFERROR(VLOOKUP($B313,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B313="","",IFERROR(VLOOKUP($B313,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G313" s="65" t="str">
         <x:f>IF($F313="","",IFERROR(VLOOKUP($F313,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17721,7 +17724,7 @@
         <x:f>IF($D314="","",IF($D314="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F314" s="53" t="str">
-        <x:f>IF($B314="","",IFERROR(VLOOKUP($B314,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B314="","",IFERROR(VLOOKUP($B314,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G314" s="65" t="str">
         <x:f>IF($F314="","",IFERROR(VLOOKUP($F314,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17774,7 +17777,7 @@
         <x:f>IF($D315="","",IF($D315="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F315" s="53" t="str">
-        <x:f>IF($B315="","",IFERROR(VLOOKUP($B315,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B315="","",IFERROR(VLOOKUP($B315,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G315" s="65" t="str">
         <x:f>IF($F315="","",IFERROR(VLOOKUP($F315,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17827,7 +17830,7 @@
         <x:f>IF($D316="","",IF($D316="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F316" s="53" t="str">
-        <x:f>IF($B316="","",IFERROR(VLOOKUP($B316,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B316="","",IFERROR(VLOOKUP($B316,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G316" s="65" t="str">
         <x:f>IF($F316="","",IFERROR(VLOOKUP($F316,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17880,7 +17883,7 @@
         <x:f>IF($D317="","",IF($D317="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F317" s="53" t="str">
-        <x:f>IF($B317="","",IFERROR(VLOOKUP($B317,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B317="","",IFERROR(VLOOKUP($B317,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G317" s="65" t="str">
         <x:f>IF($F317="","",IFERROR(VLOOKUP($F317,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17933,7 +17936,7 @@
         <x:f>IF($D318="","",IF($D318="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F318" s="53" t="str">
-        <x:f>IF($B318="","",IFERROR(VLOOKUP($B318,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B318="","",IFERROR(VLOOKUP($B318,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G318" s="65" t="str">
         <x:f>IF($F318="","",IFERROR(VLOOKUP($F318,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -17986,7 +17989,7 @@
         <x:f>IF($D319="","",IF($D319="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F319" s="53" t="str">
-        <x:f>IF($B319="","",IFERROR(VLOOKUP($B319,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B319="","",IFERROR(VLOOKUP($B319,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G319" s="65" t="str">
         <x:f>IF($F319="","",IFERROR(VLOOKUP($F319,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18039,7 +18042,7 @@
         <x:f>IF($D320="","",IF($D320="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F320" s="53" t="str">
-        <x:f>IF($B320="","",IFERROR(VLOOKUP($B320,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B320="","",IFERROR(VLOOKUP($B320,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G320" s="65" t="str">
         <x:f>IF($F320="","",IFERROR(VLOOKUP($F320,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18092,7 +18095,7 @@
         <x:f>IF($D321="","",IF($D321="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F321" s="53" t="str">
-        <x:f>IF($B321="","",IFERROR(VLOOKUP($B321,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B321="","",IFERROR(VLOOKUP($B321,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G321" s="65" t="str">
         <x:f>IF($F321="","",IFERROR(VLOOKUP($F321,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18145,7 +18148,7 @@
         <x:f>IF($D322="","",IF($D322="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F322" s="53" t="str">
-        <x:f>IF($B322="","",IFERROR(VLOOKUP($B322,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B322="","",IFERROR(VLOOKUP($B322,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G322" s="65" t="str">
         <x:f>IF($F322="","",IFERROR(VLOOKUP($F322,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18198,7 +18201,7 @@
         <x:f>IF($D323="","",IF($D323="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F323" s="53" t="str">
-        <x:f>IF($B323="","",IFERROR(VLOOKUP($B323,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B323="","",IFERROR(VLOOKUP($B323,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G323" s="65" t="str">
         <x:f>IF($F323="","",IFERROR(VLOOKUP($F323,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18251,7 +18254,7 @@
         <x:f>IF($D324="","",IF($D324="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F324" s="53" t="str">
-        <x:f>IF($B324="","",IFERROR(VLOOKUP($B324,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B324="","",IFERROR(VLOOKUP($B324,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G324" s="65" t="str">
         <x:f>IF($F324="","",IFERROR(VLOOKUP($F324,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18304,7 +18307,7 @@
         <x:f>IF($D325="","",IF($D325="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F325" s="53" t="str">
-        <x:f>IF($B325="","",IFERROR(VLOOKUP($B325,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B325="","",IFERROR(VLOOKUP($B325,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G325" s="65" t="str">
         <x:f>IF($F325="","",IFERROR(VLOOKUP($F325,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18357,7 +18360,7 @@
         <x:f>IF($D326="","",IF($D326="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F326" s="53" t="str">
-        <x:f>IF($B326="","",IFERROR(VLOOKUP($B326,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B326="","",IFERROR(VLOOKUP($B326,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G326" s="65" t="str">
         <x:f>IF($F326="","",IFERROR(VLOOKUP($F326,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18410,7 +18413,7 @@
         <x:f>IF($D327="","",IF($D327="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F327" s="53" t="str">
-        <x:f>IF($B327="","",IFERROR(VLOOKUP($B327,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B327="","",IFERROR(VLOOKUP($B327,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G327" s="65" t="str">
         <x:f>IF($F327="","",IFERROR(VLOOKUP($F327,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18463,7 +18466,7 @@
         <x:f>IF($D328="","",IF($D328="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F328" s="53" t="str">
-        <x:f>IF($B328="","",IFERROR(VLOOKUP($B328,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B328="","",IFERROR(VLOOKUP($B328,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G328" s="65" t="str">
         <x:f>IF($F328="","",IFERROR(VLOOKUP($F328,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18516,7 +18519,7 @@
         <x:f>IF($D329="","",IF($D329="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F329" s="53" t="str">
-        <x:f>IF($B329="","",IFERROR(VLOOKUP($B329,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B329="","",IFERROR(VLOOKUP($B329,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G329" s="65" t="str">
         <x:f>IF($F329="","",IFERROR(VLOOKUP($F329,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18569,7 +18572,7 @@
         <x:f>IF($D330="","",IF($D330="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F330" s="53" t="str">
-        <x:f>IF($B330="","",IFERROR(VLOOKUP($B330,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B330="","",IFERROR(VLOOKUP($B330,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G330" s="65" t="str">
         <x:f>IF($F330="","",IFERROR(VLOOKUP($F330,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18622,7 +18625,7 @@
         <x:f>IF($D331="","",IF($D331="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F331" s="53" t="str">
-        <x:f>IF($B331="","",IFERROR(VLOOKUP($B331,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B331="","",IFERROR(VLOOKUP($B331,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G331" s="65" t="str">
         <x:f>IF($F331="","",IFERROR(VLOOKUP($F331,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18675,7 +18678,7 @@
         <x:f>IF($D332="","",IF($D332="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F332" s="53" t="str">
-        <x:f>IF($B332="","",IFERROR(VLOOKUP($B332,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B332="","",IFERROR(VLOOKUP($B332,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G332" s="65" t="str">
         <x:f>IF($F332="","",IFERROR(VLOOKUP($F332,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18728,7 +18731,7 @@
         <x:f>IF($D333="","",IF($D333="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F333" s="53" t="str">
-        <x:f>IF($B333="","",IFERROR(VLOOKUP($B333,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B333="","",IFERROR(VLOOKUP($B333,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G333" s="65" t="str">
         <x:f>IF($F333="","",IFERROR(VLOOKUP($F333,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18781,7 +18784,7 @@
         <x:f>IF($D334="","",IF($D334="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F334" s="53" t="str">
-        <x:f>IF($B334="","",IFERROR(VLOOKUP($B334,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B334="","",IFERROR(VLOOKUP($B334,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G334" s="65" t="str">
         <x:f>IF($F334="","",IFERROR(VLOOKUP($F334,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18834,7 +18837,7 @@
         <x:f>IF($D335="","",IF($D335="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F335" s="53" t="str">
-        <x:f>IF($B335="","",IFERROR(VLOOKUP($B335,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B335="","",IFERROR(VLOOKUP($B335,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G335" s="65" t="str">
         <x:f>IF($F335="","",IFERROR(VLOOKUP($F335,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18887,7 +18890,7 @@
         <x:f>IF($D336="","",IF($D336="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F336" s="53" t="str">
-        <x:f>IF($B336="","",IFERROR(VLOOKUP($B336,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B336="","",IFERROR(VLOOKUP($B336,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G336" s="65" t="str">
         <x:f>IF($F336="","",IFERROR(VLOOKUP($F336,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18940,7 +18943,7 @@
         <x:f>IF($D337="","",IF($D337="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F337" s="53" t="str">
-        <x:f>IF($B337="","",IFERROR(VLOOKUP($B337,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B337="","",IFERROR(VLOOKUP($B337,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G337" s="65" t="str">
         <x:f>IF($F337="","",IFERROR(VLOOKUP($F337,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -18993,7 +18996,7 @@
         <x:f>IF($D338="","",IF($D338="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F338" s="53" t="str">
-        <x:f>IF($B338="","",IFERROR(VLOOKUP($B338,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B338="","",IFERROR(VLOOKUP($B338,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G338" s="65" t="str">
         <x:f>IF($F338="","",IFERROR(VLOOKUP($F338,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19046,7 +19049,7 @@
         <x:f>IF($D339="","",IF($D339="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F339" s="53" t="str">
-        <x:f>IF($B339="","",IFERROR(VLOOKUP($B339,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B339="","",IFERROR(VLOOKUP($B339,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G339" s="65" t="str">
         <x:f>IF($F339="","",IFERROR(VLOOKUP($F339,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19099,7 +19102,7 @@
         <x:f>IF($D340="","",IF($D340="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F340" s="53" t="str">
-        <x:f>IF($B340="","",IFERROR(VLOOKUP($B340,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B340="","",IFERROR(VLOOKUP($B340,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G340" s="65" t="str">
         <x:f>IF($F340="","",IFERROR(VLOOKUP($F340,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19152,7 +19155,7 @@
         <x:f>IF($D341="","",IF($D341="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F341" s="53" t="str">
-        <x:f>IF($B341="","",IFERROR(VLOOKUP($B341,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B341="","",IFERROR(VLOOKUP($B341,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G341" s="65" t="str">
         <x:f>IF($F341="","",IFERROR(VLOOKUP($F341,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19205,7 +19208,7 @@
         <x:f>IF($D342="","",IF($D342="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F342" s="53" t="str">
-        <x:f>IF($B342="","",IFERROR(VLOOKUP($B342,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B342="","",IFERROR(VLOOKUP($B342,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G342" s="65" t="str">
         <x:f>IF($F342="","",IFERROR(VLOOKUP($F342,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19258,7 +19261,7 @@
         <x:f>IF($D343="","",IF($D343="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F343" s="53" t="str">
-        <x:f>IF($B343="","",IFERROR(VLOOKUP($B343,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B343="","",IFERROR(VLOOKUP($B343,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G343" s="65" t="str">
         <x:f>IF($F343="","",IFERROR(VLOOKUP($F343,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19311,7 +19314,7 @@
         <x:f>IF($D344="","",IF($D344="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F344" s="53" t="str">
-        <x:f>IF($B344="","",IFERROR(VLOOKUP($B344,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B344="","",IFERROR(VLOOKUP($B344,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G344" s="65" t="str">
         <x:f>IF($F344="","",IFERROR(VLOOKUP($F344,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19364,7 +19367,7 @@
         <x:f>IF($D345="","",IF($D345="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F345" s="53" t="str">
-        <x:f>IF($B345="","",IFERROR(VLOOKUP($B345,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B345="","",IFERROR(VLOOKUP($B345,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G345" s="65" t="str">
         <x:f>IF($F345="","",IFERROR(VLOOKUP($F345,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19417,7 +19420,7 @@
         <x:f>IF($D346="","",IF($D346="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F346" s="53" t="str">
-        <x:f>IF($B346="","",IFERROR(VLOOKUP($B346,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B346="","",IFERROR(VLOOKUP($B346,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G346" s="65" t="str">
         <x:f>IF($F346="","",IFERROR(VLOOKUP($F346,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19470,7 +19473,7 @@
         <x:f>IF($D347="","",IF($D347="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F347" s="53" t="str">
-        <x:f>IF($B347="","",IFERROR(VLOOKUP($B347,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B347="","",IFERROR(VLOOKUP($B347,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G347" s="65" t="str">
         <x:f>IF($F347="","",IFERROR(VLOOKUP($F347,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19523,7 +19526,7 @@
         <x:f>IF($D348="","",IF($D348="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F348" s="53" t="str">
-        <x:f>IF($B348="","",IFERROR(VLOOKUP($B348,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B348="","",IFERROR(VLOOKUP($B348,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G348" s="65" t="str">
         <x:f>IF($F348="","",IFERROR(VLOOKUP($F348,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19576,7 +19579,7 @@
         <x:f>IF($D349="","",IF($D349="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F349" s="53" t="str">
-        <x:f>IF($B349="","",IFERROR(VLOOKUP($B349,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B349="","",IFERROR(VLOOKUP($B349,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G349" s="65" t="str">
         <x:f>IF($F349="","",IFERROR(VLOOKUP($F349,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19629,7 +19632,7 @@
         <x:f>IF($D350="","",IF($D350="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F350" s="53" t="str">
-        <x:f>IF($B350="","",IFERROR(VLOOKUP($B350,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B350="","",IFERROR(VLOOKUP($B350,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G350" s="65" t="str">
         <x:f>IF($F350="","",IFERROR(VLOOKUP($F350,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19682,7 +19685,7 @@
         <x:f>IF($D351="","",IF($D351="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F351" s="53" t="str">
-        <x:f>IF($B351="","",IFERROR(VLOOKUP($B351,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B351="","",IFERROR(VLOOKUP($B351,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G351" s="65" t="str">
         <x:f>IF($F351="","",IFERROR(VLOOKUP($F351,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19735,7 +19738,7 @@
         <x:f>IF($D352="","",IF($D352="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F352" s="53" t="str">
-        <x:f>IF($B352="","",IFERROR(VLOOKUP($B352,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B352="","",IFERROR(VLOOKUP($B352,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G352" s="65" t="str">
         <x:f>IF($F352="","",IFERROR(VLOOKUP($F352,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19788,7 +19791,7 @@
         <x:f>IF($D353="","",IF($D353="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F353" s="53" t="str">
-        <x:f>IF($B353="","",IFERROR(VLOOKUP($B353,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B353="","",IFERROR(VLOOKUP($B353,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G353" s="65" t="str">
         <x:f>IF($F353="","",IFERROR(VLOOKUP($F353,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19841,7 +19844,7 @@
         <x:f>IF($D354="","",IF($D354="PS",'Data'!$O$5,'Data'!$O$4))</x:f>
       </x:c>
       <x:c r="F354" s="56" t="str">
-        <x:f>IF($B354="","",IFERROR(VLOOKUP($B354,'Data'!$A$2:$B$113,2,FALSE),""))</x:f>
+        <x:f>IF($B354="","",IFERROR(VLOOKUP($B354,'Data'!$A$2:$B$114,2,FALSE),""))</x:f>
       </x:c>
       <x:c r="G354" s="66" t="str">
         <x:f>IF($F354="","",IFERROR(VLOOKUP($F354,'Data'!$D$2:$G$14,3,FALSE),""))</x:f>
@@ -19896,7 +19899,7 @@
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B5:B354">
-      <x:formula1>$U$2:$U$113</x:formula1>
+      <x:formula1>$U$2:$U$114</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="decimal" operator="greaterThan" sqref="C5:C354">
       <x:formula1>0</x:formula1>
@@ -21101,6 +21104,14 @@
         <x:v>C</x:v>
       </x:c>
     </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="92" t="str">
+        <x:v>Production Operator - II - Production &amp; Operations Support (T): Industrial - O2 (Low)</x:v>
+      </x:c>
+      <x:c r="B114" s="92" t="str">
+        <x:v>A</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>